<commit_message>
Revision 4: TCGA CPM normalisation, patient-level exclusion in Sanger design, one-model-per-patient and patient-block permutation, Welch, spline, low-n permutation, average-linkage S4 Fig, Fig 1/9/12 update
Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/figures/supporting_information/S2_Table.xlsx
+++ b/figures/supporting_information/S2_Table.xlsx
@@ -425,7 +425,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:K95"/>
+  <dimension ref="A1:L95"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -484,6 +484,11 @@
           <t>confidence_flag</t>
         </is>
       </c>
+      <c r="L1" s="1" t="inlineStr">
+        <is>
+          <t>Retained with one model per patient</t>
+        </is>
+      </c>
     </row>
     <row r="2">
       <c r="A2" t="inlineStr">
@@ -517,7 +522,7 @@
         <v>4.094102258496909e-22</v>
       </c>
       <c r="I2" t="n">
-        <v>3.187197196705966e-18</v>
+        <v>3.187197196705967e-18</v>
       </c>
       <c r="J2" t="b">
         <v>1</v>
@@ -526,6 +531,9 @@
         <is>
           <t>n&gt;=10</t>
         </is>
+      </c>
+      <c r="L2" t="b">
+        <v>1</v>
       </c>
     </row>
     <row r="3">
@@ -570,6 +578,9 @@
           <t>n&gt;=10</t>
         </is>
       </c>
+      <c r="L3" t="b">
+        <v>1</v>
+      </c>
     </row>
     <row r="4">
       <c r="A4" t="inlineStr">
@@ -613,6 +624,9 @@
           <t>n&gt;=10</t>
         </is>
       </c>
+      <c r="L4" t="b">
+        <v>1</v>
+      </c>
     </row>
     <row r="5">
       <c r="A5" t="inlineStr">
@@ -656,6 +670,9 @@
           <t>low sample size (n&lt;10)</t>
         </is>
       </c>
+      <c r="L5" t="b">
+        <v>1</v>
+      </c>
     </row>
     <row r="6">
       <c r="A6" t="inlineStr">
@@ -699,6 +716,9 @@
           <t>n&gt;=10</t>
         </is>
       </c>
+      <c r="L6" t="b">
+        <v>1</v>
+      </c>
     </row>
     <row r="7">
       <c r="A7" t="inlineStr">
@@ -742,6 +762,9 @@
           <t>n&gt;=10</t>
         </is>
       </c>
+      <c r="L7" t="b">
+        <v>1</v>
+      </c>
     </row>
     <row r="8">
       <c r="A8" t="inlineStr">
@@ -785,6 +808,9 @@
           <t>n&gt;=10</t>
         </is>
       </c>
+      <c r="L8" t="b">
+        <v>1</v>
+      </c>
     </row>
     <row r="9">
       <c r="A9" t="inlineStr">
@@ -828,6 +854,9 @@
           <t>n&gt;=10</t>
         </is>
       </c>
+      <c r="L9" t="b">
+        <v>1</v>
+      </c>
     </row>
     <row r="10">
       <c r="A10" t="inlineStr">
@@ -871,6 +900,9 @@
           <t>n&gt;=10</t>
         </is>
       </c>
+      <c r="L10" t="b">
+        <v>1</v>
+      </c>
     </row>
     <row r="11">
       <c r="A11" t="inlineStr">
@@ -914,6 +946,9 @@
           <t>low sample size (n&lt;10)</t>
         </is>
       </c>
+      <c r="L11" t="b">
+        <v>0</v>
+      </c>
     </row>
     <row r="12">
       <c r="A12" t="inlineStr">
@@ -957,6 +992,9 @@
           <t>n&gt;=10</t>
         </is>
       </c>
+      <c r="L12" t="b">
+        <v>1</v>
+      </c>
     </row>
     <row r="13">
       <c r="A13" t="inlineStr">
@@ -1000,6 +1038,9 @@
           <t>n&gt;=10</t>
         </is>
       </c>
+      <c r="L13" t="b">
+        <v>1</v>
+      </c>
     </row>
     <row r="14">
       <c r="A14" t="inlineStr">
@@ -1043,6 +1084,9 @@
           <t>n&gt;=10</t>
         </is>
       </c>
+      <c r="L14" t="b">
+        <v>1</v>
+      </c>
     </row>
     <row r="15">
       <c r="A15" t="inlineStr">
@@ -1086,6 +1130,9 @@
           <t>n&gt;=10</t>
         </is>
       </c>
+      <c r="L15" t="b">
+        <v>1</v>
+      </c>
     </row>
     <row r="16">
       <c r="A16" t="inlineStr">
@@ -1116,7 +1163,7 @@
         <v>-0.9443862012758956</v>
       </c>
       <c r="H16" t="n">
-        <v>5.528624045549505e-29</v>
+        <v>5.528624045549504e-29</v>
       </c>
       <c r="I16" t="n">
         <v>1.291185267029882e-24</v>
@@ -1129,6 +1176,9 @@
           <t>n&gt;=10</t>
         </is>
       </c>
+      <c r="L16" t="b">
+        <v>1</v>
+      </c>
     </row>
     <row r="17">
       <c r="A17" t="inlineStr">
@@ -1172,6 +1222,9 @@
           <t>n&gt;=10</t>
         </is>
       </c>
+      <c r="L17" t="b">
+        <v>1</v>
+      </c>
     </row>
     <row r="18">
       <c r="A18" t="inlineStr">
@@ -1215,6 +1268,9 @@
           <t>n&gt;=10</t>
         </is>
       </c>
+      <c r="L18" t="b">
+        <v>1</v>
+      </c>
     </row>
     <row r="19">
       <c r="A19" t="inlineStr">
@@ -1258,6 +1314,9 @@
           <t>n&gt;=10</t>
         </is>
       </c>
+      <c r="L19" t="b">
+        <v>1</v>
+      </c>
     </row>
     <row r="20">
       <c r="A20" t="inlineStr">
@@ -1301,6 +1360,9 @@
           <t>n&gt;=10</t>
         </is>
       </c>
+      <c r="L20" t="b">
+        <v>1</v>
+      </c>
     </row>
     <row r="21">
       <c r="A21" t="inlineStr">
@@ -1344,6 +1406,9 @@
           <t>n&gt;=10</t>
         </is>
       </c>
+      <c r="L21" t="b">
+        <v>1</v>
+      </c>
     </row>
     <row r="22">
       <c r="A22" t="inlineStr">
@@ -1387,6 +1452,9 @@
           <t>n&gt;=10</t>
         </is>
       </c>
+      <c r="L22" t="b">
+        <v>1</v>
+      </c>
     </row>
     <row r="23">
       <c r="A23" t="inlineStr">
@@ -1417,7 +1485,7 @@
         <v>-0.8153544382751436</v>
       </c>
       <c r="H23" t="n">
-        <v>2.075636238096951e-10</v>
+        <v>2.07563623809695e-10</v>
       </c>
       <c r="I23" t="n">
         <v>2.130793419975699e-07</v>
@@ -1430,6 +1498,9 @@
           <t>n&gt;=10</t>
         </is>
       </c>
+      <c r="L23" t="b">
+        <v>1</v>
+      </c>
     </row>
     <row r="24">
       <c r="A24" t="inlineStr">
@@ -1473,6 +1544,9 @@
           <t>n&gt;=10</t>
         </is>
       </c>
+      <c r="L24" t="b">
+        <v>1</v>
+      </c>
     </row>
     <row r="25">
       <c r="A25" t="inlineStr">
@@ -1516,6 +1590,9 @@
           <t>n&gt;=10</t>
         </is>
       </c>
+      <c r="L25" t="b">
+        <v>1</v>
+      </c>
     </row>
     <row r="26">
       <c r="A26" t="inlineStr">
@@ -1559,6 +1636,9 @@
           <t>low sample size (n&lt;10)</t>
         </is>
       </c>
+      <c r="L26" t="b">
+        <v>1</v>
+      </c>
     </row>
     <row r="27">
       <c r="A27" t="inlineStr">
@@ -1602,6 +1682,9 @@
           <t>n&gt;=10</t>
         </is>
       </c>
+      <c r="L27" t="b">
+        <v>1</v>
+      </c>
     </row>
     <row r="28">
       <c r="A28" t="inlineStr">
@@ -1645,6 +1728,9 @@
           <t>n&gt;=10</t>
         </is>
       </c>
+      <c r="L28" t="b">
+        <v>1</v>
+      </c>
     </row>
     <row r="29">
       <c r="A29" t="inlineStr">
@@ -1675,7 +1761,7 @@
         <v>-0.7717732730149428</v>
       </c>
       <c r="H29" t="n">
-        <v>7.866237070193035e-29</v>
+        <v>7.866237070193034e-29</v>
       </c>
       <c r="I29" t="n">
         <v>1.749642161596922e-24</v>
@@ -1688,6 +1774,9 @@
           <t>n&gt;=10</t>
         </is>
       </c>
+      <c r="L29" t="b">
+        <v>1</v>
+      </c>
     </row>
     <row r="30">
       <c r="A30" t="inlineStr">
@@ -1731,6 +1820,9 @@
           <t>n&gt;=10</t>
         </is>
       </c>
+      <c r="L30" t="b">
+        <v>1</v>
+      </c>
     </row>
     <row r="31">
       <c r="A31" t="inlineStr">
@@ -1774,6 +1866,9 @@
           <t>n&gt;=10</t>
         </is>
       </c>
+      <c r="L31" t="b">
+        <v>1</v>
+      </c>
     </row>
     <row r="32">
       <c r="A32" t="inlineStr">
@@ -1817,6 +1912,9 @@
           <t>n&gt;=10</t>
         </is>
       </c>
+      <c r="L32" t="b">
+        <v>1</v>
+      </c>
     </row>
     <row r="33">
       <c r="A33" t="inlineStr">
@@ -1860,6 +1958,9 @@
           <t>n&gt;=10</t>
         </is>
       </c>
+      <c r="L33" t="b">
+        <v>1</v>
+      </c>
     </row>
     <row r="34">
       <c r="A34" t="inlineStr">
@@ -1903,6 +2004,9 @@
           <t>n&gt;=10</t>
         </is>
       </c>
+      <c r="L34" t="b">
+        <v>1</v>
+      </c>
     </row>
     <row r="35">
       <c r="A35" t="inlineStr">
@@ -1933,7 +2037,7 @@
         <v>-0.7315352899151317</v>
       </c>
       <c r="H35" t="n">
-        <v>1.205557157838033e-29</v>
+        <v>1.205557157838034e-29</v>
       </c>
       <c r="I35" t="n">
         <v>3.128360546731804e-25</v>
@@ -1946,6 +2050,9 @@
           <t>n&gt;=10</t>
         </is>
       </c>
+      <c r="L35" t="b">
+        <v>1</v>
+      </c>
     </row>
     <row r="36">
       <c r="A36" t="inlineStr">
@@ -1989,6 +2096,9 @@
           <t>n&gt;=10</t>
         </is>
       </c>
+      <c r="L36" t="b">
+        <v>1</v>
+      </c>
     </row>
     <row r="37">
       <c r="A37" t="inlineStr">
@@ -2032,6 +2142,9 @@
           <t>n&gt;=10</t>
         </is>
       </c>
+      <c r="L37" t="b">
+        <v>1</v>
+      </c>
     </row>
     <row r="38">
       <c r="A38" t="inlineStr">
@@ -2075,6 +2188,9 @@
           <t>n&gt;=10</t>
         </is>
       </c>
+      <c r="L38" t="b">
+        <v>1</v>
+      </c>
     </row>
     <row r="39">
       <c r="A39" t="inlineStr">
@@ -2118,6 +2234,9 @@
           <t>n&gt;=10</t>
         </is>
       </c>
+      <c r="L39" t="b">
+        <v>1</v>
+      </c>
     </row>
     <row r="40">
       <c r="A40" t="inlineStr">
@@ -2161,6 +2280,9 @@
           <t>n&gt;=10</t>
         </is>
       </c>
+      <c r="L40" t="b">
+        <v>1</v>
+      </c>
     </row>
     <row r="41">
       <c r="A41" t="inlineStr">
@@ -2204,6 +2326,9 @@
           <t>n&gt;=10</t>
         </is>
       </c>
+      <c r="L41" t="b">
+        <v>1</v>
+      </c>
     </row>
     <row r="42">
       <c r="A42" t="inlineStr">
@@ -2247,6 +2372,9 @@
           <t>n&gt;=10</t>
         </is>
       </c>
+      <c r="L42" t="b">
+        <v>1</v>
+      </c>
     </row>
     <row r="43">
       <c r="A43" t="inlineStr">
@@ -2290,6 +2418,9 @@
           <t>n&gt;=10</t>
         </is>
       </c>
+      <c r="L43" t="b">
+        <v>0</v>
+      </c>
     </row>
     <row r="44">
       <c r="A44" t="inlineStr">
@@ -2333,6 +2464,9 @@
           <t>n&gt;=10</t>
         </is>
       </c>
+      <c r="L44" t="b">
+        <v>1</v>
+      </c>
     </row>
     <row r="45">
       <c r="A45" t="inlineStr">
@@ -2376,6 +2510,9 @@
           <t>n&gt;=10</t>
         </is>
       </c>
+      <c r="L45" t="b">
+        <v>1</v>
+      </c>
     </row>
     <row r="46">
       <c r="A46" t="inlineStr">
@@ -2419,6 +2556,9 @@
           <t>n&gt;=10</t>
         </is>
       </c>
+      <c r="L46" t="b">
+        <v>1</v>
+      </c>
     </row>
     <row r="47">
       <c r="A47" t="inlineStr">
@@ -2462,6 +2602,9 @@
           <t>n&gt;=10</t>
         </is>
       </c>
+      <c r="L47" t="b">
+        <v>1</v>
+      </c>
     </row>
     <row r="48">
       <c r="A48" t="inlineStr">
@@ -2505,6 +2648,9 @@
           <t>n&gt;=10</t>
         </is>
       </c>
+      <c r="L48" t="b">
+        <v>1</v>
+      </c>
     </row>
     <row r="49">
       <c r="A49" t="inlineStr">
@@ -2548,6 +2694,9 @@
           <t>n&gt;=10</t>
         </is>
       </c>
+      <c r="L49" t="b">
+        <v>1</v>
+      </c>
     </row>
     <row r="50">
       <c r="A50" t="inlineStr">
@@ -2591,6 +2740,9 @@
           <t>n&gt;=10</t>
         </is>
       </c>
+      <c r="L50" t="b">
+        <v>1</v>
+      </c>
     </row>
     <row r="51">
       <c r="A51" t="inlineStr">
@@ -2634,6 +2786,9 @@
           <t>n&gt;=10</t>
         </is>
       </c>
+      <c r="L51" t="b">
+        <v>1</v>
+      </c>
     </row>
     <row r="52">
       <c r="A52" t="inlineStr">
@@ -2677,6 +2832,9 @@
           <t>n&gt;=10</t>
         </is>
       </c>
+      <c r="L52" t="b">
+        <v>1</v>
+      </c>
     </row>
     <row r="53">
       <c r="A53" t="inlineStr">
@@ -2720,6 +2878,9 @@
           <t>n&gt;=10</t>
         </is>
       </c>
+      <c r="L53" t="b">
+        <v>1</v>
+      </c>
     </row>
     <row r="54">
       <c r="A54" t="inlineStr">
@@ -2763,6 +2924,9 @@
           <t>n&gt;=10</t>
         </is>
       </c>
+      <c r="L54" t="b">
+        <v>1</v>
+      </c>
     </row>
     <row r="55">
       <c r="A55" t="inlineStr">
@@ -2806,6 +2970,9 @@
           <t>n&gt;=10</t>
         </is>
       </c>
+      <c r="L55" t="b">
+        <v>1</v>
+      </c>
     </row>
     <row r="56">
       <c r="A56" t="inlineStr">
@@ -2849,6 +3016,9 @@
           <t>n&gt;=10</t>
         </is>
       </c>
+      <c r="L56" t="b">
+        <v>1</v>
+      </c>
     </row>
     <row r="57">
       <c r="A57" t="inlineStr">
@@ -2892,6 +3062,9 @@
           <t>n&gt;=10</t>
         </is>
       </c>
+      <c r="L57" t="b">
+        <v>1</v>
+      </c>
     </row>
     <row r="58">
       <c r="A58" t="inlineStr">
@@ -2935,6 +3108,9 @@
           <t>n&gt;=10</t>
         </is>
       </c>
+      <c r="L58" t="b">
+        <v>1</v>
+      </c>
     </row>
     <row r="59">
       <c r="A59" t="inlineStr">
@@ -2978,6 +3154,9 @@
           <t>n&gt;=10</t>
         </is>
       </c>
+      <c r="L59" t="b">
+        <v>1</v>
+      </c>
     </row>
     <row r="60">
       <c r="A60" t="inlineStr">
@@ -3021,6 +3200,9 @@
           <t>n&gt;=10</t>
         </is>
       </c>
+      <c r="L60" t="b">
+        <v>1</v>
+      </c>
     </row>
     <row r="61">
       <c r="A61" t="inlineStr">
@@ -3064,6 +3246,9 @@
           <t>n&gt;=10</t>
         </is>
       </c>
+      <c r="L61" t="b">
+        <v>1</v>
+      </c>
     </row>
     <row r="62">
       <c r="A62" t="inlineStr">
@@ -3107,6 +3292,9 @@
           <t>n&gt;=10</t>
         </is>
       </c>
+      <c r="L62" t="b">
+        <v>0</v>
+      </c>
     </row>
     <row r="63">
       <c r="A63" t="inlineStr">
@@ -3150,6 +3338,9 @@
           <t>n&gt;=10</t>
         </is>
       </c>
+      <c r="L63" t="b">
+        <v>1</v>
+      </c>
     </row>
     <row r="64">
       <c r="A64" t="inlineStr">
@@ -3193,6 +3384,9 @@
           <t>n&gt;=10</t>
         </is>
       </c>
+      <c r="L64" t="b">
+        <v>1</v>
+      </c>
     </row>
     <row r="65">
       <c r="A65" t="inlineStr">
@@ -3236,6 +3430,9 @@
           <t>n&gt;=10</t>
         </is>
       </c>
+      <c r="L65" t="b">
+        <v>1</v>
+      </c>
     </row>
     <row r="66">
       <c r="A66" t="inlineStr">
@@ -3279,6 +3476,9 @@
           <t>n&gt;=10</t>
         </is>
       </c>
+      <c r="L66" t="b">
+        <v>1</v>
+      </c>
     </row>
     <row r="67">
       <c r="A67" t="inlineStr">
@@ -3322,6 +3522,9 @@
           <t>n&gt;=10</t>
         </is>
       </c>
+      <c r="L67" t="b">
+        <v>1</v>
+      </c>
     </row>
     <row r="68">
       <c r="A68" t="inlineStr">
@@ -3365,6 +3568,9 @@
           <t>n&gt;=10</t>
         </is>
       </c>
+      <c r="L68" t="b">
+        <v>1</v>
+      </c>
     </row>
     <row r="69">
       <c r="A69" t="inlineStr">
@@ -3408,6 +3614,9 @@
           <t>n&gt;=10</t>
         </is>
       </c>
+      <c r="L69" t="b">
+        <v>0</v>
+      </c>
     </row>
     <row r="70">
       <c r="A70" t="inlineStr">
@@ -3451,6 +3660,9 @@
           <t>n&gt;=10</t>
         </is>
       </c>
+      <c r="L70" t="b">
+        <v>1</v>
+      </c>
     </row>
     <row r="71">
       <c r="A71" t="inlineStr">
@@ -3494,6 +3706,9 @@
           <t>n&gt;=10</t>
         </is>
       </c>
+      <c r="L71" t="b">
+        <v>1</v>
+      </c>
     </row>
     <row r="72">
       <c r="A72" t="inlineStr">
@@ -3537,6 +3752,9 @@
           <t>n&gt;=10</t>
         </is>
       </c>
+      <c r="L72" t="b">
+        <v>1</v>
+      </c>
     </row>
     <row r="73">
       <c r="A73" t="inlineStr">
@@ -3580,6 +3798,9 @@
           <t>n&gt;=10</t>
         </is>
       </c>
+      <c r="L73" t="b">
+        <v>1</v>
+      </c>
     </row>
     <row r="74">
       <c r="A74" t="inlineStr">
@@ -3623,6 +3844,9 @@
           <t>n&gt;=10</t>
         </is>
       </c>
+      <c r="L74" t="b">
+        <v>1</v>
+      </c>
     </row>
     <row r="75">
       <c r="A75" t="inlineStr">
@@ -3666,6 +3890,9 @@
           <t>n&gt;=10</t>
         </is>
       </c>
+      <c r="L75" t="b">
+        <v>1</v>
+      </c>
     </row>
     <row r="76">
       <c r="A76" t="inlineStr">
@@ -3709,6 +3936,9 @@
           <t>n&gt;=10</t>
         </is>
       </c>
+      <c r="L76" t="b">
+        <v>1</v>
+      </c>
     </row>
     <row r="77">
       <c r="A77" t="inlineStr">
@@ -3752,6 +3982,9 @@
           <t>n&gt;=10</t>
         </is>
       </c>
+      <c r="L77" t="b">
+        <v>1</v>
+      </c>
     </row>
     <row r="78">
       <c r="A78" t="inlineStr">
@@ -3795,6 +4028,9 @@
           <t>n&gt;=10</t>
         </is>
       </c>
+      <c r="L78" t="b">
+        <v>1</v>
+      </c>
     </row>
     <row r="79">
       <c r="A79" t="inlineStr">
@@ -3838,6 +4074,9 @@
           <t>n&gt;=10</t>
         </is>
       </c>
+      <c r="L79" t="b">
+        <v>1</v>
+      </c>
     </row>
     <row r="80">
       <c r="A80" t="inlineStr">
@@ -3881,6 +4120,9 @@
           <t>n&gt;=10</t>
         </is>
       </c>
+      <c r="L80" t="b">
+        <v>1</v>
+      </c>
     </row>
     <row r="81">
       <c r="A81" t="inlineStr">
@@ -3924,6 +4166,9 @@
           <t>n&gt;=10</t>
         </is>
       </c>
+      <c r="L81" t="b">
+        <v>1</v>
+      </c>
     </row>
     <row r="82">
       <c r="A82" t="inlineStr">
@@ -3967,6 +4212,9 @@
           <t>n&gt;=10</t>
         </is>
       </c>
+      <c r="L82" t="b">
+        <v>1</v>
+      </c>
     </row>
     <row r="83">
       <c r="A83" t="inlineStr">
@@ -4010,6 +4258,9 @@
           <t>n&gt;=10</t>
         </is>
       </c>
+      <c r="L83" t="b">
+        <v>1</v>
+      </c>
     </row>
     <row r="84">
       <c r="A84" t="inlineStr">
@@ -4053,6 +4304,9 @@
           <t>n&gt;=10</t>
         </is>
       </c>
+      <c r="L84" t="b">
+        <v>1</v>
+      </c>
     </row>
     <row r="85">
       <c r="A85" t="inlineStr">
@@ -4086,7 +4340,7 @@
         <v>2.47733188297244e-13</v>
       </c>
       <c r="I85" t="n">
-        <v>4.987669942023617e-10</v>
+        <v>4.987669942023616e-10</v>
       </c>
       <c r="J85" t="b">
         <v>1</v>
@@ -4095,6 +4349,9 @@
         <is>
           <t>n&gt;=10</t>
         </is>
+      </c>
+      <c r="L85" t="b">
+        <v>1</v>
       </c>
     </row>
     <row r="86">
@@ -4139,6 +4396,9 @@
           <t>n&gt;=10</t>
         </is>
       </c>
+      <c r="L86" t="b">
+        <v>1</v>
+      </c>
     </row>
     <row r="87">
       <c r="A87" t="inlineStr">
@@ -4182,6 +4442,9 @@
           <t>n&gt;=10</t>
         </is>
       </c>
+      <c r="L87" t="b">
+        <v>1</v>
+      </c>
     </row>
     <row r="88">
       <c r="A88" t="inlineStr">
@@ -4225,6 +4488,9 @@
           <t>n&gt;=10</t>
         </is>
       </c>
+      <c r="L88" t="b">
+        <v>0</v>
+      </c>
     </row>
     <row r="89">
       <c r="A89" t="inlineStr">
@@ -4268,6 +4534,9 @@
           <t>n&gt;=10</t>
         </is>
       </c>
+      <c r="L89" t="b">
+        <v>1</v>
+      </c>
     </row>
     <row r="90">
       <c r="A90" t="inlineStr">
@@ -4311,6 +4580,9 @@
           <t>n&gt;=10</t>
         </is>
       </c>
+      <c r="L90" t="b">
+        <v>1</v>
+      </c>
     </row>
     <row r="91">
       <c r="A91" t="inlineStr">
@@ -4354,6 +4626,9 @@
           <t>n&gt;=10</t>
         </is>
       </c>
+      <c r="L91" t="b">
+        <v>1</v>
+      </c>
     </row>
     <row r="92">
       <c r="A92" t="inlineStr">
@@ -4397,6 +4672,9 @@
           <t>n&gt;=10</t>
         </is>
       </c>
+      <c r="L92" t="b">
+        <v>0</v>
+      </c>
     </row>
     <row r="93">
       <c r="A93" t="inlineStr">
@@ -4440,6 +4718,9 @@
           <t>n&gt;=10</t>
         </is>
       </c>
+      <c r="L93" t="b">
+        <v>1</v>
+      </c>
     </row>
     <row r="94">
       <c r="A94" t="inlineStr">
@@ -4483,6 +4764,9 @@
           <t>n&gt;=10</t>
         </is>
       </c>
+      <c r="L94" t="b">
+        <v>0</v>
+      </c>
     </row>
     <row r="95">
       <c r="A95" t="inlineStr">
@@ -4525,6 +4809,9 @@
         <is>
           <t>n&gt;=10</t>
         </is>
+      </c>
+      <c r="L95" t="b">
+        <v>1</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
revision6_checks.py: matched co-dependency null from all genes, bootstrap intervals, comparison-group medians, APC/BRAF genotype, quantile-matched 22Q1 threshold, adherent-only comparison; S2 Table columns
Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/figures/supporting_information/S2_Table.xlsx
+++ b/figures/supporting_information/S2_Table.xlsx
@@ -425,7 +425,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:L95"/>
+  <dimension ref="A1:T95"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -489,6 +489,46 @@
           <t>Retained with one model per patient</t>
         </is>
       </c>
+      <c r="M1" s="1" t="inlineStr">
+        <is>
+          <t>Selectivity, bootstrap 95% CI low</t>
+        </is>
+      </c>
+      <c r="N1" s="1" t="inlineStr">
+        <is>
+          <t>Selectivity, bootstrap 95% CI high</t>
+        </is>
+      </c>
+      <c r="O1" s="1" t="inlineStr">
+        <is>
+          <t>Bootstrap fraction with selectivity &lt; -0.5</t>
+        </is>
+      </c>
+      <c r="P1" s="1" t="inlineStr">
+        <is>
+          <t>Median Chronos, all other lines</t>
+        </is>
+      </c>
+      <c r="Q1" s="1" t="inlineStr">
+        <is>
+          <t>Other eligible lineages with median &lt; -1</t>
+        </is>
+      </c>
+      <c r="R1" s="1" t="inlineStr">
+        <is>
+          <t>Fraction of cancer lines with data for the gene</t>
+        </is>
+      </c>
+      <c r="S1" s="1" t="inlineStr">
+        <is>
+          <t>Selectivity against adherent lines of other lineages (non-blood pairs)</t>
+        </is>
+      </c>
+      <c r="T1" s="1" t="inlineStr">
+        <is>
+          <t>Partial gene coverage (&lt; 50% of lines)</t>
+        </is>
+      </c>
     </row>
     <row r="2">
       <c r="A2" t="inlineStr">
@@ -535,6 +575,30 @@
       <c r="L2" t="b">
         <v>1</v>
       </c>
+      <c r="M2" t="n">
+        <v>-1.906805716960861</v>
+      </c>
+      <c r="N2" t="n">
+        <v>-1.363999375487942</v>
+      </c>
+      <c r="O2" t="n">
+        <v>1</v>
+      </c>
+      <c r="P2" t="n">
+        <v>-0.5027912706731148</v>
+      </c>
+      <c r="Q2" t="n">
+        <v>1</v>
+      </c>
+      <c r="R2" t="n">
+        <v>1</v>
+      </c>
+      <c r="S2" t="n">
+        <v>-1.584452650068515</v>
+      </c>
+      <c r="T2" t="b">
+        <v>0</v>
+      </c>
     </row>
     <row r="3">
       <c r="A3" t="inlineStr">
@@ -581,6 +645,30 @@
       <c r="L3" t="b">
         <v>1</v>
       </c>
+      <c r="M3" t="n">
+        <v>-1.662227347736795</v>
+      </c>
+      <c r="N3" t="n">
+        <v>-1.126609743863654</v>
+      </c>
+      <c r="O3" t="n">
+        <v>1</v>
+      </c>
+      <c r="P3" t="n">
+        <v>-0.2953696861005563</v>
+      </c>
+      <c r="Q3" t="n">
+        <v>1</v>
+      </c>
+      <c r="R3" t="n">
+        <v>1</v>
+      </c>
+      <c r="S3" t="n">
+        <v>-1.365346268416268</v>
+      </c>
+      <c r="T3" t="b">
+        <v>0</v>
+      </c>
     </row>
     <row r="4">
       <c r="A4" t="inlineStr">
@@ -627,6 +715,30 @@
       <c r="L4" t="b">
         <v>1</v>
       </c>
+      <c r="M4" t="n">
+        <v>-1.556707242659497</v>
+      </c>
+      <c r="N4" t="n">
+        <v>-0.6778479788938805</v>
+      </c>
+      <c r="O4" t="n">
+        <v>0.988</v>
+      </c>
+      <c r="P4" t="n">
+        <v>-0.1599547715406944</v>
+      </c>
+      <c r="Q4" t="n">
+        <v>0</v>
+      </c>
+      <c r="R4" t="n">
+        <v>1</v>
+      </c>
+      <c r="S4" t="n">
+        <v>-1.266030939868908</v>
+      </c>
+      <c r="T4" t="b">
+        <v>0</v>
+      </c>
     </row>
     <row r="5">
       <c r="A5" t="inlineStr">
@@ -673,6 +785,30 @@
       <c r="L5" t="b">
         <v>1</v>
       </c>
+      <c r="M5" t="n">
+        <v>-2.136194848897806</v>
+      </c>
+      <c r="N5" t="n">
+        <v>-0.0340679715719917</v>
+      </c>
+      <c r="O5" t="n">
+        <v>0.952</v>
+      </c>
+      <c r="P5" t="n">
+        <v>-0.1225957134497577</v>
+      </c>
+      <c r="Q5" t="n">
+        <v>0</v>
+      </c>
+      <c r="R5" t="n">
+        <v>1</v>
+      </c>
+      <c r="S5" t="n">
+        <v>-1.23404302816103</v>
+      </c>
+      <c r="T5" t="b">
+        <v>0</v>
+      </c>
     </row>
     <row r="6">
       <c r="A6" t="inlineStr">
@@ -719,6 +855,30 @@
       <c r="L6" t="b">
         <v>1</v>
       </c>
+      <c r="M6" t="n">
+        <v>-1.400498035486563</v>
+      </c>
+      <c r="N6" t="n">
+        <v>-0.7722021415362592</v>
+      </c>
+      <c r="O6" t="n">
+        <v>1</v>
+      </c>
+      <c r="P6" t="n">
+        <v>-0.4199775996261109</v>
+      </c>
+      <c r="Q6" t="n">
+        <v>3</v>
+      </c>
+      <c r="R6" t="n">
+        <v>1</v>
+      </c>
+      <c r="S6" t="n">
+        <v>-1.125878754445281</v>
+      </c>
+      <c r="T6" t="b">
+        <v>0</v>
+      </c>
     </row>
     <row r="7">
       <c r="A7" t="inlineStr">
@@ -765,6 +925,30 @@
       <c r="L7" t="b">
         <v>1</v>
       </c>
+      <c r="M7" t="n">
+        <v>-1.300993063677379</v>
+      </c>
+      <c r="N7" t="n">
+        <v>-0.8164514005408364</v>
+      </c>
+      <c r="O7" t="n">
+        <v>1</v>
+      </c>
+      <c r="P7" t="n">
+        <v>-0.1329652794742778</v>
+      </c>
+      <c r="Q7" t="n">
+        <v>1</v>
+      </c>
+      <c r="R7" t="n">
+        <v>1</v>
+      </c>
+      <c r="S7" t="n">
+        <v>-1.109792710320845</v>
+      </c>
+      <c r="T7" t="b">
+        <v>0</v>
+      </c>
     </row>
     <row r="8">
       <c r="A8" t="inlineStr">
@@ -811,6 +995,30 @@
       <c r="L8" t="b">
         <v>1</v>
       </c>
+      <c r="M8" t="n">
+        <v>-1.549150473460425</v>
+      </c>
+      <c r="N8" t="n">
+        <v>-0.6449981322261785</v>
+      </c>
+      <c r="O8" t="n">
+        <v>0.996</v>
+      </c>
+      <c r="P8" t="n">
+        <v>-0.5563753664767225</v>
+      </c>
+      <c r="Q8" t="n">
+        <v>3</v>
+      </c>
+      <c r="R8" t="n">
+        <v>1</v>
+      </c>
+      <c r="S8" t="n">
+        <v>-1.058221316126808</v>
+      </c>
+      <c r="T8" t="b">
+        <v>0</v>
+      </c>
     </row>
     <row r="9">
       <c r="A9" t="inlineStr">
@@ -857,6 +1065,28 @@
       <c r="L9" t="b">
         <v>1</v>
       </c>
+      <c r="M9" t="n">
+        <v>-1.324288863240755</v>
+      </c>
+      <c r="N9" t="n">
+        <v>-0.9912270020046864</v>
+      </c>
+      <c r="O9" t="n">
+        <v>1</v>
+      </c>
+      <c r="P9" t="n">
+        <v>-0.2931148543955476</v>
+      </c>
+      <c r="Q9" t="n">
+        <v>0</v>
+      </c>
+      <c r="R9" t="n">
+        <v>1</v>
+      </c>
+      <c r="S9" t="inlineStr"/>
+      <c r="T9" t="b">
+        <v>0</v>
+      </c>
     </row>
     <row r="10">
       <c r="A10" t="inlineStr">
@@ -903,6 +1133,28 @@
       <c r="L10" t="b">
         <v>1</v>
       </c>
+      <c r="M10" t="n">
+        <v>-1.390782242700744</v>
+      </c>
+      <c r="N10" t="n">
+        <v>-0.8512741288732499</v>
+      </c>
+      <c r="O10" t="n">
+        <v>1</v>
+      </c>
+      <c r="P10" t="n">
+        <v>-0.1457668424501607</v>
+      </c>
+      <c r="Q10" t="n">
+        <v>0</v>
+      </c>
+      <c r="R10" t="n">
+        <v>1</v>
+      </c>
+      <c r="S10" t="inlineStr"/>
+      <c r="T10" t="b">
+        <v>0</v>
+      </c>
     </row>
     <row r="11">
       <c r="A11" t="inlineStr">
@@ -949,6 +1201,30 @@
       <c r="L11" t="b">
         <v>0</v>
       </c>
+      <c r="M11" t="n">
+        <v>-1.955273996353375</v>
+      </c>
+      <c r="N11" t="n">
+        <v>-0.1196608610778677</v>
+      </c>
+      <c r="O11" t="n">
+        <v>0.6850000000000001</v>
+      </c>
+      <c r="P11" t="n">
+        <v>-0.32316123250174</v>
+      </c>
+      <c r="Q11" t="n">
+        <v>0</v>
+      </c>
+      <c r="R11" t="n">
+        <v>1</v>
+      </c>
+      <c r="S11" t="n">
+        <v>-1.02620617371</v>
+      </c>
+      <c r="T11" t="b">
+        <v>0</v>
+      </c>
     </row>
     <row r="12">
       <c r="A12" t="inlineStr">
@@ -995,6 +1271,30 @@
       <c r="L12" t="b">
         <v>1</v>
       </c>
+      <c r="M12" t="n">
+        <v>-1.328607260254524</v>
+      </c>
+      <c r="N12" t="n">
+        <v>-0.4424338935593439</v>
+      </c>
+      <c r="O12" t="n">
+        <v>0.958</v>
+      </c>
+      <c r="P12" t="n">
+        <v>-0.1057483436988376</v>
+      </c>
+      <c r="Q12" t="n">
+        <v>0</v>
+      </c>
+      <c r="R12" t="n">
+        <v>1</v>
+      </c>
+      <c r="S12" t="n">
+        <v>-1.009824469373484</v>
+      </c>
+      <c r="T12" t="b">
+        <v>0</v>
+      </c>
     </row>
     <row r="13">
       <c r="A13" t="inlineStr">
@@ -1041,6 +1341,30 @@
       <c r="L13" t="b">
         <v>1</v>
       </c>
+      <c r="M13" t="n">
+        <v>-1.151286526457582</v>
+      </c>
+      <c r="N13" t="n">
+        <v>-0.6934279565962019</v>
+      </c>
+      <c r="O13" t="n">
+        <v>0.996</v>
+      </c>
+      <c r="P13" t="n">
+        <v>-0.08542755800437569</v>
+      </c>
+      <c r="Q13" t="n">
+        <v>0</v>
+      </c>
+      <c r="R13" t="n">
+        <v>1</v>
+      </c>
+      <c r="S13" t="n">
+        <v>-1.006015403525742</v>
+      </c>
+      <c r="T13" t="b">
+        <v>0</v>
+      </c>
     </row>
     <row r="14">
       <c r="A14" t="inlineStr">
@@ -1087,6 +1411,30 @@
       <c r="L14" t="b">
         <v>1</v>
       </c>
+      <c r="M14" t="n">
+        <v>-1.281197306098525</v>
+      </c>
+      <c r="N14" t="n">
+        <v>-0.704137304957687</v>
+      </c>
+      <c r="O14" t="n">
+        <v>1</v>
+      </c>
+      <c r="P14" t="n">
+        <v>-0.1141629380048705</v>
+      </c>
+      <c r="Q14" t="n">
+        <v>0</v>
+      </c>
+      <c r="R14" t="n">
+        <v>1</v>
+      </c>
+      <c r="S14" t="n">
+        <v>-0.9881551348459824</v>
+      </c>
+      <c r="T14" t="b">
+        <v>0</v>
+      </c>
     </row>
     <row r="15">
       <c r="A15" t="inlineStr">
@@ -1133,6 +1481,28 @@
       <c r="L15" t="b">
         <v>1</v>
       </c>
+      <c r="M15" t="n">
+        <v>-1.107085600511549</v>
+      </c>
+      <c r="N15" t="n">
+        <v>-0.8722832816809946</v>
+      </c>
+      <c r="O15" t="n">
+        <v>1</v>
+      </c>
+      <c r="P15" t="n">
+        <v>-0.2443062206903385</v>
+      </c>
+      <c r="Q15" t="n">
+        <v>0</v>
+      </c>
+      <c r="R15" t="n">
+        <v>1</v>
+      </c>
+      <c r="S15" t="inlineStr"/>
+      <c r="T15" t="b">
+        <v>0</v>
+      </c>
     </row>
     <row r="16">
       <c r="A16" t="inlineStr">
@@ -1179,6 +1549,28 @@
       <c r="L16" t="b">
         <v>1</v>
       </c>
+      <c r="M16" t="n">
+        <v>-1.257985425138047</v>
+      </c>
+      <c r="N16" t="n">
+        <v>-0.4185608110422276</v>
+      </c>
+      <c r="O16" t="n">
+        <v>0.9389999999999999</v>
+      </c>
+      <c r="P16" t="n">
+        <v>-0.096767740013727</v>
+      </c>
+      <c r="Q16" t="n">
+        <v>0</v>
+      </c>
+      <c r="R16" t="n">
+        <v>1</v>
+      </c>
+      <c r="S16" t="inlineStr"/>
+      <c r="T16" t="b">
+        <v>0</v>
+      </c>
     </row>
     <row r="17">
       <c r="A17" t="inlineStr">
@@ -1225,6 +1617,30 @@
       <c r="L17" t="b">
         <v>1</v>
       </c>
+      <c r="M17" t="n">
+        <v>-1.121709171053386</v>
+      </c>
+      <c r="N17" t="n">
+        <v>-0.6910590319353629</v>
+      </c>
+      <c r="O17" t="n">
+        <v>0.999</v>
+      </c>
+      <c r="P17" t="n">
+        <v>-1.04655249993445</v>
+      </c>
+      <c r="Q17" t="n">
+        <v>16</v>
+      </c>
+      <c r="R17" t="n">
+        <v>1</v>
+      </c>
+      <c r="S17" t="n">
+        <v>-0.7529375255075197</v>
+      </c>
+      <c r="T17" t="b">
+        <v>0</v>
+      </c>
     </row>
     <row r="18">
       <c r="A18" t="inlineStr">
@@ -1271,6 +1687,30 @@
       <c r="L18" t="b">
         <v>1</v>
       </c>
+      <c r="M18" t="n">
+        <v>-1.118830499690903</v>
+      </c>
+      <c r="N18" t="n">
+        <v>-0.4455358349683622</v>
+      </c>
+      <c r="O18" t="n">
+        <v>0.958</v>
+      </c>
+      <c r="P18" t="n">
+        <v>-0.4829437816216086</v>
+      </c>
+      <c r="Q18" t="n">
+        <v>6</v>
+      </c>
+      <c r="R18" t="n">
+        <v>1</v>
+      </c>
+      <c r="S18" t="n">
+        <v>-0.7785534884072509</v>
+      </c>
+      <c r="T18" t="b">
+        <v>0</v>
+      </c>
     </row>
     <row r="19">
       <c r="A19" t="inlineStr">
@@ -1317,6 +1757,30 @@
       <c r="L19" t="b">
         <v>1</v>
       </c>
+      <c r="M19" t="n">
+        <v>-1.409108204869249</v>
+      </c>
+      <c r="N19" t="n">
+        <v>-0.3776306398983961</v>
+      </c>
+      <c r="O19" t="n">
+        <v>0.834</v>
+      </c>
+      <c r="P19" t="n">
+        <v>-0.6597209731187603</v>
+      </c>
+      <c r="Q19" t="n">
+        <v>0</v>
+      </c>
+      <c r="R19" t="n">
+        <v>1</v>
+      </c>
+      <c r="S19" t="n">
+        <v>-0.9059054274829854</v>
+      </c>
+      <c r="T19" t="b">
+        <v>0</v>
+      </c>
     </row>
     <row r="20">
       <c r="A20" t="inlineStr">
@@ -1363,6 +1827,30 @@
       <c r="L20" t="b">
         <v>1</v>
       </c>
+      <c r="M20" t="n">
+        <v>-1.102160435514065</v>
+      </c>
+      <c r="N20" t="n">
+        <v>-0.3640754126948947</v>
+      </c>
+      <c r="O20" t="n">
+        <v>0.965</v>
+      </c>
+      <c r="P20" t="n">
+        <v>-0.4160707239969616</v>
+      </c>
+      <c r="Q20" t="n">
+        <v>3</v>
+      </c>
+      <c r="R20" t="n">
+        <v>1</v>
+      </c>
+      <c r="S20" t="n">
+        <v>-0.8639862304996127</v>
+      </c>
+      <c r="T20" t="b">
+        <v>0</v>
+      </c>
     </row>
     <row r="21">
       <c r="A21" t="inlineStr">
@@ -1409,6 +1897,30 @@
       <c r="L21" t="b">
         <v>1</v>
       </c>
+      <c r="M21" t="n">
+        <v>-1.214369382284079</v>
+      </c>
+      <c r="N21" t="n">
+        <v>-0.186825387565905</v>
+      </c>
+      <c r="O21" t="n">
+        <v>0.875</v>
+      </c>
+      <c r="P21" t="n">
+        <v>-0.4186339007710089</v>
+      </c>
+      <c r="Q21" t="n">
+        <v>3</v>
+      </c>
+      <c r="R21" t="n">
+        <v>1</v>
+      </c>
+      <c r="S21" t="n">
+        <v>-0.8511794949700303</v>
+      </c>
+      <c r="T21" t="b">
+        <v>0</v>
+      </c>
     </row>
     <row r="22">
       <c r="A22" t="inlineStr">
@@ -1455,6 +1967,30 @@
       <c r="L22" t="b">
         <v>1</v>
       </c>
+      <c r="M22" t="n">
+        <v>-1.085955196916328</v>
+      </c>
+      <c r="N22" t="n">
+        <v>-0.4611772746409619</v>
+      </c>
+      <c r="O22" t="n">
+        <v>0.901</v>
+      </c>
+      <c r="P22" t="n">
+        <v>-0.7740374797538534</v>
+      </c>
+      <c r="Q22" t="n">
+        <v>5</v>
+      </c>
+      <c r="R22" t="n">
+        <v>1</v>
+      </c>
+      <c r="S22" t="n">
+        <v>-0.8198661214223878</v>
+      </c>
+      <c r="T22" t="b">
+        <v>0</v>
+      </c>
     </row>
     <row r="23">
       <c r="A23" t="inlineStr">
@@ -1501,6 +2037,30 @@
       <c r="L23" t="b">
         <v>1</v>
       </c>
+      <c r="M23" t="n">
+        <v>-1.025757133269352</v>
+      </c>
+      <c r="N23" t="n">
+        <v>-0.3025941633086956</v>
+      </c>
+      <c r="O23" t="n">
+        <v>0.863</v>
+      </c>
+      <c r="P23" t="n">
+        <v>-0.414666013664794</v>
+      </c>
+      <c r="Q23" t="n">
+        <v>3</v>
+      </c>
+      <c r="R23" t="n">
+        <v>1</v>
+      </c>
+      <c r="S23" t="n">
+        <v>-0.8114075168145537</v>
+      </c>
+      <c r="T23" t="b">
+        <v>0</v>
+      </c>
     </row>
     <row r="24">
       <c r="A24" t="inlineStr">
@@ -1547,6 +2107,28 @@
       <c r="L24" t="b">
         <v>1</v>
       </c>
+      <c r="M24" t="n">
+        <v>-0.8935893324096084</v>
+      </c>
+      <c r="N24" t="n">
+        <v>-0.7088831852765213</v>
+      </c>
+      <c r="O24" t="n">
+        <v>1</v>
+      </c>
+      <c r="P24" t="n">
+        <v>-0.2973934471262233</v>
+      </c>
+      <c r="Q24" t="n">
+        <v>0</v>
+      </c>
+      <c r="R24" t="n">
+        <v>1</v>
+      </c>
+      <c r="S24" t="inlineStr"/>
+      <c r="T24" t="b">
+        <v>0</v>
+      </c>
     </row>
     <row r="25">
       <c r="A25" t="inlineStr">
@@ -1593,6 +2175,28 @@
       <c r="L25" t="b">
         <v>1</v>
       </c>
+      <c r="M25" t="n">
+        <v>-1.044007379909569</v>
+      </c>
+      <c r="N25" t="n">
+        <v>-0.4754491883069735</v>
+      </c>
+      <c r="O25" t="n">
+        <v>0.9330000000000001</v>
+      </c>
+      <c r="P25" t="n">
+        <v>-0.4420862368788819</v>
+      </c>
+      <c r="Q25" t="n">
+        <v>2</v>
+      </c>
+      <c r="R25" t="n">
+        <v>1</v>
+      </c>
+      <c r="S25" t="inlineStr"/>
+      <c r="T25" t="b">
+        <v>0</v>
+      </c>
     </row>
     <row r="26">
       <c r="A26" t="inlineStr">
@@ -1639,6 +2243,28 @@
       <c r="L26" t="b">
         <v>1</v>
       </c>
+      <c r="M26" t="n">
+        <v>-1.016873625440496</v>
+      </c>
+      <c r="N26" t="n">
+        <v>-0.3271779690315874</v>
+      </c>
+      <c r="O26" t="n">
+        <v>0.874</v>
+      </c>
+      <c r="P26" t="n">
+        <v>-0.6452072614166818</v>
+      </c>
+      <c r="Q26" t="n">
+        <v>1</v>
+      </c>
+      <c r="R26" t="n">
+        <v>0.0620805369127516</v>
+      </c>
+      <c r="S26" t="inlineStr"/>
+      <c r="T26" t="b">
+        <v>1</v>
+      </c>
     </row>
     <row r="27">
       <c r="A27" t="inlineStr">
@@ -1685,6 +2311,28 @@
       <c r="L27" t="b">
         <v>1</v>
       </c>
+      <c r="M27" t="n">
+        <v>-0.8458188419611679</v>
+      </c>
+      <c r="N27" t="n">
+        <v>-0.7287101235189486</v>
+      </c>
+      <c r="O27" t="n">
+        <v>1</v>
+      </c>
+      <c r="P27" t="n">
+        <v>-0.2969030721089515</v>
+      </c>
+      <c r="Q27" t="n">
+        <v>1</v>
+      </c>
+      <c r="R27" t="n">
+        <v>1</v>
+      </c>
+      <c r="S27" t="inlineStr"/>
+      <c r="T27" t="b">
+        <v>0</v>
+      </c>
     </row>
     <row r="28">
       <c r="A28" t="inlineStr">
@@ -1731,6 +2379,30 @@
       <c r="L28" t="b">
         <v>1</v>
       </c>
+      <c r="M28" t="n">
+        <v>-0.9467674591839504</v>
+      </c>
+      <c r="N28" t="n">
+        <v>-0.6161600962252058</v>
+      </c>
+      <c r="O28" t="n">
+        <v>0.999</v>
+      </c>
+      <c r="P28" t="n">
+        <v>-0.7422117172167758</v>
+      </c>
+      <c r="Q28" t="n">
+        <v>6</v>
+      </c>
+      <c r="R28" t="n">
+        <v>1</v>
+      </c>
+      <c r="S28" t="n">
+        <v>-0.8191204755982007</v>
+      </c>
+      <c r="T28" t="b">
+        <v>0</v>
+      </c>
     </row>
     <row r="29">
       <c r="A29" t="inlineStr">
@@ -1777,6 +2449,28 @@
       <c r="L29" t="b">
         <v>1</v>
       </c>
+      <c r="M29" t="n">
+        <v>-0.9811918580826304</v>
+      </c>
+      <c r="N29" t="n">
+        <v>-0.6917674466057018</v>
+      </c>
+      <c r="O29" t="n">
+        <v>1</v>
+      </c>
+      <c r="P29" t="n">
+        <v>-0.4242902412865484</v>
+      </c>
+      <c r="Q29" t="n">
+        <v>2</v>
+      </c>
+      <c r="R29" t="n">
+        <v>1</v>
+      </c>
+      <c r="S29" t="inlineStr"/>
+      <c r="T29" t="b">
+        <v>0</v>
+      </c>
     </row>
     <row r="30">
       <c r="A30" t="inlineStr">
@@ -1823,6 +2517,30 @@
       <c r="L30" t="b">
         <v>1</v>
       </c>
+      <c r="M30" t="n">
+        <v>-1.124047138521464</v>
+      </c>
+      <c r="N30" t="n">
+        <v>-0.2390371319950871</v>
+      </c>
+      <c r="O30" t="n">
+        <v>0.879</v>
+      </c>
+      <c r="P30" t="n">
+        <v>-0.6993277480985273</v>
+      </c>
+      <c r="Q30" t="n">
+        <v>3</v>
+      </c>
+      <c r="R30" t="n">
+        <v>1</v>
+      </c>
+      <c r="S30" t="n">
+        <v>-0.839977473932463</v>
+      </c>
+      <c r="T30" t="b">
+        <v>0</v>
+      </c>
     </row>
     <row r="31">
       <c r="A31" t="inlineStr">
@@ -1869,6 +2587,28 @@
       <c r="L31" t="b">
         <v>1</v>
       </c>
+      <c r="M31" t="n">
+        <v>-0.8718543246219286</v>
+      </c>
+      <c r="N31" t="n">
+        <v>-0.6666177584605667</v>
+      </c>
+      <c r="O31" t="n">
+        <v>1</v>
+      </c>
+      <c r="P31" t="n">
+        <v>-0.6649898271888</v>
+      </c>
+      <c r="Q31" t="n">
+        <v>3</v>
+      </c>
+      <c r="R31" t="n">
+        <v>1</v>
+      </c>
+      <c r="S31" t="inlineStr"/>
+      <c r="T31" t="b">
+        <v>0</v>
+      </c>
     </row>
     <row r="32">
       <c r="A32" t="inlineStr">
@@ -1915,6 +2655,30 @@
       <c r="L32" t="b">
         <v>1</v>
       </c>
+      <c r="M32" t="n">
+        <v>-0.8722347225595037</v>
+      </c>
+      <c r="N32" t="n">
+        <v>-0.5977436026047905</v>
+      </c>
+      <c r="O32" t="n">
+        <v>1</v>
+      </c>
+      <c r="P32" t="n">
+        <v>-0.469949191719441</v>
+      </c>
+      <c r="Q32" t="n">
+        <v>6</v>
+      </c>
+      <c r="R32" t="n">
+        <v>1</v>
+      </c>
+      <c r="S32" t="n">
+        <v>-0.6084736820451923</v>
+      </c>
+      <c r="T32" t="b">
+        <v>0</v>
+      </c>
     </row>
     <row r="33">
       <c r="A33" t="inlineStr">
@@ -1961,6 +2725,28 @@
       <c r="L33" t="b">
         <v>1</v>
       </c>
+      <c r="M33" t="n">
+        <v>-0.8407937567604921</v>
+      </c>
+      <c r="N33" t="n">
+        <v>-0.5978451340904132</v>
+      </c>
+      <c r="O33" t="n">
+        <v>1</v>
+      </c>
+      <c r="P33" t="n">
+        <v>-0.8353018438376421</v>
+      </c>
+      <c r="Q33" t="n">
+        <v>8</v>
+      </c>
+      <c r="R33" t="n">
+        <v>1</v>
+      </c>
+      <c r="S33" t="inlineStr"/>
+      <c r="T33" t="b">
+        <v>0</v>
+      </c>
     </row>
     <row r="34">
       <c r="A34" t="inlineStr">
@@ -2007,6 +2793,28 @@
       <c r="L34" t="b">
         <v>1</v>
       </c>
+      <c r="M34" t="n">
+        <v>-0.9176013519077216</v>
+      </c>
+      <c r="N34" t="n">
+        <v>-0.6432621992866175</v>
+      </c>
+      <c r="O34" t="n">
+        <v>1</v>
+      </c>
+      <c r="P34" t="n">
+        <v>-0.3103096117101562</v>
+      </c>
+      <c r="Q34" t="n">
+        <v>1</v>
+      </c>
+      <c r="R34" t="n">
+        <v>1</v>
+      </c>
+      <c r="S34" t="inlineStr"/>
+      <c r="T34" t="b">
+        <v>0</v>
+      </c>
     </row>
     <row r="35">
       <c r="A35" t="inlineStr">
@@ -2053,6 +2861,28 @@
       <c r="L35" t="b">
         <v>1</v>
       </c>
+      <c r="M35" t="n">
+        <v>-0.8250703777805477</v>
+      </c>
+      <c r="N35" t="n">
+        <v>-0.5744135085334444</v>
+      </c>
+      <c r="O35" t="n">
+        <v>1</v>
+      </c>
+      <c r="P35" t="n">
+        <v>-0.3974415725073837</v>
+      </c>
+      <c r="Q35" t="n">
+        <v>1</v>
+      </c>
+      <c r="R35" t="n">
+        <v>1</v>
+      </c>
+      <c r="S35" t="inlineStr"/>
+      <c r="T35" t="b">
+        <v>0</v>
+      </c>
     </row>
     <row r="36">
       <c r="A36" t="inlineStr">
@@ -2099,6 +2929,28 @@
       <c r="L36" t="b">
         <v>1</v>
       </c>
+      <c r="M36" t="n">
+        <v>-0.8401401258990273</v>
+      </c>
+      <c r="N36" t="n">
+        <v>-0.5381750748842614</v>
+      </c>
+      <c r="O36" t="n">
+        <v>0.994</v>
+      </c>
+      <c r="P36" t="n">
+        <v>-0.9640618079384859</v>
+      </c>
+      <c r="Q36" t="n">
+        <v>8</v>
+      </c>
+      <c r="R36" t="n">
+        <v>1</v>
+      </c>
+      <c r="S36" t="inlineStr"/>
+      <c r="T36" t="b">
+        <v>0</v>
+      </c>
     </row>
     <row r="37">
       <c r="A37" t="inlineStr">
@@ -2145,6 +2997,30 @@
       <c r="L37" t="b">
         <v>1</v>
       </c>
+      <c r="M37" t="n">
+        <v>-0.9538492226665428</v>
+      </c>
+      <c r="N37" t="n">
+        <v>-0.3794946059674365</v>
+      </c>
+      <c r="O37" t="n">
+        <v>0.9429999999999999</v>
+      </c>
+      <c r="P37" t="n">
+        <v>-1.044696539322223</v>
+      </c>
+      <c r="Q37" t="n">
+        <v>16</v>
+      </c>
+      <c r="R37" t="n">
+        <v>1</v>
+      </c>
+      <c r="S37" t="n">
+        <v>-0.5544090465874651</v>
+      </c>
+      <c r="T37" t="b">
+        <v>0</v>
+      </c>
     </row>
     <row r="38">
       <c r="A38" t="inlineStr">
@@ -2191,6 +3067,28 @@
       <c r="L38" t="b">
         <v>1</v>
       </c>
+      <c r="M38" t="n">
+        <v>-1.119731924003487</v>
+      </c>
+      <c r="N38" t="n">
+        <v>-0.3953221815802298</v>
+      </c>
+      <c r="O38" t="n">
+        <v>0.9409999999999999</v>
+      </c>
+      <c r="P38" t="n">
+        <v>-0.7929491880436018</v>
+      </c>
+      <c r="Q38" t="n">
+        <v>1</v>
+      </c>
+      <c r="R38" t="n">
+        <v>0.2642617449664429</v>
+      </c>
+      <c r="S38" t="inlineStr"/>
+      <c r="T38" t="b">
+        <v>1</v>
+      </c>
     </row>
     <row r="39">
       <c r="A39" t="inlineStr">
@@ -2237,6 +3135,28 @@
       <c r="L39" t="b">
         <v>1</v>
       </c>
+      <c r="M39" t="n">
+        <v>-0.8052953054982561</v>
+      </c>
+      <c r="N39" t="n">
+        <v>-0.5818918334160008</v>
+      </c>
+      <c r="O39" t="n">
+        <v>0.997</v>
+      </c>
+      <c r="P39" t="n">
+        <v>-0.9184347638906504</v>
+      </c>
+      <c r="Q39" t="n">
+        <v>8</v>
+      </c>
+      <c r="R39" t="n">
+        <v>1</v>
+      </c>
+      <c r="S39" t="inlineStr"/>
+      <c r="T39" t="b">
+        <v>0</v>
+      </c>
     </row>
     <row r="40">
       <c r="A40" t="inlineStr">
@@ -2283,6 +3203,28 @@
       <c r="L40" t="b">
         <v>1</v>
       </c>
+      <c r="M40" t="n">
+        <v>-0.8304330544232009</v>
+      </c>
+      <c r="N40" t="n">
+        <v>-0.5410985577939629</v>
+      </c>
+      <c r="O40" t="n">
+        <v>1</v>
+      </c>
+      <c r="P40" t="n">
+        <v>-0.2902772721273366</v>
+      </c>
+      <c r="Q40" t="n">
+        <v>0</v>
+      </c>
+      <c r="R40" t="n">
+        <v>1</v>
+      </c>
+      <c r="S40" t="inlineStr"/>
+      <c r="T40" t="b">
+        <v>0</v>
+      </c>
     </row>
     <row r="41">
       <c r="A41" t="inlineStr">
@@ -2329,6 +3271,30 @@
       <c r="L41" t="b">
         <v>1</v>
       </c>
+      <c r="M41" t="n">
+        <v>-0.9655658334931724</v>
+      </c>
+      <c r="N41" t="n">
+        <v>-0.4925378929892742</v>
+      </c>
+      <c r="O41" t="n">
+        <v>0.973</v>
+      </c>
+      <c r="P41" t="n">
+        <v>-0.9615977554022876</v>
+      </c>
+      <c r="Q41" t="n">
+        <v>13</v>
+      </c>
+      <c r="R41" t="n">
+        <v>1</v>
+      </c>
+      <c r="S41" t="n">
+        <v>-0.6853701508326836</v>
+      </c>
+      <c r="T41" t="b">
+        <v>0</v>
+      </c>
     </row>
     <row r="42">
       <c r="A42" t="inlineStr">
@@ -2375,6 +3341,30 @@
       <c r="L42" t="b">
         <v>1</v>
       </c>
+      <c r="M42" t="n">
+        <v>-1.057595610458858</v>
+      </c>
+      <c r="N42" t="n">
+        <v>-0.5136514845713118</v>
+      </c>
+      <c r="O42" t="n">
+        <v>0.976</v>
+      </c>
+      <c r="P42" t="n">
+        <v>-0.5027572416194172</v>
+      </c>
+      <c r="Q42" t="n">
+        <v>1</v>
+      </c>
+      <c r="R42" t="n">
+        <v>1</v>
+      </c>
+      <c r="S42" t="n">
+        <v>-0.7085207064429841</v>
+      </c>
+      <c r="T42" t="b">
+        <v>0</v>
+      </c>
     </row>
     <row r="43">
       <c r="A43" t="inlineStr">
@@ -2421,6 +3411,30 @@
       <c r="L43" t="b">
         <v>0</v>
       </c>
+      <c r="M43" t="n">
+        <v>-1.447797438543193</v>
+      </c>
+      <c r="N43" t="n">
+        <v>-0.081084273042486</v>
+      </c>
+      <c r="O43" t="n">
+        <v>0.64</v>
+      </c>
+      <c r="P43" t="n">
+        <v>-0.3054095560530782</v>
+      </c>
+      <c r="Q43" t="n">
+        <v>1</v>
+      </c>
+      <c r="R43" t="n">
+        <v>1</v>
+      </c>
+      <c r="S43" t="n">
+        <v>-0.6942113049282915</v>
+      </c>
+      <c r="T43" t="b">
+        <v>0</v>
+      </c>
     </row>
     <row r="44">
       <c r="A44" t="inlineStr">
@@ -2467,6 +3481,28 @@
       <c r="L44" t="b">
         <v>1</v>
       </c>
+      <c r="M44" t="n">
+        <v>-0.8214357078073892</v>
+      </c>
+      <c r="N44" t="n">
+        <v>-0.5377239584877787</v>
+      </c>
+      <c r="O44" t="n">
+        <v>0.996</v>
+      </c>
+      <c r="P44" t="n">
+        <v>-0.9220808889510006</v>
+      </c>
+      <c r="Q44" t="n">
+        <v>8</v>
+      </c>
+      <c r="R44" t="n">
+        <v>1</v>
+      </c>
+      <c r="S44" t="inlineStr"/>
+      <c r="T44" t="b">
+        <v>0</v>
+      </c>
     </row>
     <row r="45">
       <c r="A45" t="inlineStr">
@@ -2513,6 +3549,30 @@
       <c r="L45" t="b">
         <v>1</v>
       </c>
+      <c r="M45" t="n">
+        <v>-0.8752541218961688</v>
+      </c>
+      <c r="N45" t="n">
+        <v>-0.4036012834856441</v>
+      </c>
+      <c r="O45" t="n">
+        <v>0.876</v>
+      </c>
+      <c r="P45" t="n">
+        <v>-0.7587150702997643</v>
+      </c>
+      <c r="Q45" t="n">
+        <v>6</v>
+      </c>
+      <c r="R45" t="n">
+        <v>1</v>
+      </c>
+      <c r="S45" t="n">
+        <v>-0.7130512657411576</v>
+      </c>
+      <c r="T45" t="b">
+        <v>0</v>
+      </c>
     </row>
     <row r="46">
       <c r="A46" t="inlineStr">
@@ -2559,6 +3619,30 @@
       <c r="L46" t="b">
         <v>1</v>
       </c>
+      <c r="M46" t="n">
+        <v>-0.8506304350029201</v>
+      </c>
+      <c r="N46" t="n">
+        <v>-0.3647592205178758</v>
+      </c>
+      <c r="O46" t="n">
+        <v>0.838</v>
+      </c>
+      <c r="P46" t="n">
+        <v>-0.970955013648747</v>
+      </c>
+      <c r="Q46" t="n">
+        <v>13</v>
+      </c>
+      <c r="R46" t="n">
+        <v>1</v>
+      </c>
+      <c r="S46" t="n">
+        <v>-0.6843641186634508</v>
+      </c>
+      <c r="T46" t="b">
+        <v>0</v>
+      </c>
     </row>
     <row r="47">
       <c r="A47" t="inlineStr">
@@ -2605,6 +3689,28 @@
       <c r="L47" t="b">
         <v>1</v>
       </c>
+      <c r="M47" t="n">
+        <v>-0.837392782689817</v>
+      </c>
+      <c r="N47" t="n">
+        <v>-0.4394183769208078</v>
+      </c>
+      <c r="O47" t="n">
+        <v>0.965</v>
+      </c>
+      <c r="P47" t="n">
+        <v>-1.754984539582456</v>
+      </c>
+      <c r="Q47" t="n">
+        <v>14</v>
+      </c>
+      <c r="R47" t="n">
+        <v>0.3196308724832215</v>
+      </c>
+      <c r="S47" t="inlineStr"/>
+      <c r="T47" t="b">
+        <v>1</v>
+      </c>
     </row>
     <row r="48">
       <c r="A48" t="inlineStr">
@@ -2651,6 +3757,30 @@
       <c r="L48" t="b">
         <v>1</v>
       </c>
+      <c r="M48" t="n">
+        <v>-0.8618205521704326</v>
+      </c>
+      <c r="N48" t="n">
+        <v>-0.3435800696406638</v>
+      </c>
+      <c r="O48" t="n">
+        <v>0.805</v>
+      </c>
+      <c r="P48" t="n">
+        <v>-0.4649200784404343</v>
+      </c>
+      <c r="Q48" t="n">
+        <v>3</v>
+      </c>
+      <c r="R48" t="n">
+        <v>1</v>
+      </c>
+      <c r="S48" t="n">
+        <v>-0.6988467703448962</v>
+      </c>
+      <c r="T48" t="b">
+        <v>0</v>
+      </c>
     </row>
     <row r="49">
       <c r="A49" t="inlineStr">
@@ -2697,6 +3827,28 @@
       <c r="L49" t="b">
         <v>1</v>
       </c>
+      <c r="M49" t="n">
+        <v>-0.7826395003841041</v>
+      </c>
+      <c r="N49" t="n">
+        <v>-0.5317305548437105</v>
+      </c>
+      <c r="O49" t="n">
+        <v>0.997</v>
+      </c>
+      <c r="P49" t="n">
+        <v>-0.4154892781807939</v>
+      </c>
+      <c r="Q49" t="n">
+        <v>0</v>
+      </c>
+      <c r="R49" t="n">
+        <v>1</v>
+      </c>
+      <c r="S49" t="inlineStr"/>
+      <c r="T49" t="b">
+        <v>0</v>
+      </c>
     </row>
     <row r="50">
       <c r="A50" t="inlineStr">
@@ -2743,6 +3895,28 @@
       <c r="L50" t="b">
         <v>1</v>
       </c>
+      <c r="M50" t="n">
+        <v>-0.7805665963298993</v>
+      </c>
+      <c r="N50" t="n">
+        <v>-0.5700772057451743</v>
+      </c>
+      <c r="O50" t="n">
+        <v>1</v>
+      </c>
+      <c r="P50" t="n">
+        <v>-0.4318221903668604</v>
+      </c>
+      <c r="Q50" t="n">
+        <v>2</v>
+      </c>
+      <c r="R50" t="n">
+        <v>1</v>
+      </c>
+      <c r="S50" t="inlineStr"/>
+      <c r="T50" t="b">
+        <v>0</v>
+      </c>
     </row>
     <row r="51">
       <c r="A51" t="inlineStr">
@@ -2789,6 +3963,28 @@
       <c r="L51" t="b">
         <v>1</v>
       </c>
+      <c r="M51" t="n">
+        <v>-1.066934176872252</v>
+      </c>
+      <c r="N51" t="n">
+        <v>-0.2349879569704975</v>
+      </c>
+      <c r="O51" t="n">
+        <v>0.606</v>
+      </c>
+      <c r="P51" t="n">
+        <v>-0.4950326289911044</v>
+      </c>
+      <c r="Q51" t="n">
+        <v>2</v>
+      </c>
+      <c r="R51" t="n">
+        <v>1</v>
+      </c>
+      <c r="S51" t="inlineStr"/>
+      <c r="T51" t="b">
+        <v>0</v>
+      </c>
     </row>
     <row r="52">
       <c r="A52" t="inlineStr">
@@ -2835,6 +4031,30 @@
       <c r="L52" t="b">
         <v>1</v>
       </c>
+      <c r="M52" t="n">
+        <v>-0.7521731603149857</v>
+      </c>
+      <c r="N52" t="n">
+        <v>-0.4335330572060192</v>
+      </c>
+      <c r="O52" t="n">
+        <v>0.8120000000000001</v>
+      </c>
+      <c r="P52" t="n">
+        <v>-0.4772688689809301</v>
+      </c>
+      <c r="Q52" t="n">
+        <v>6</v>
+      </c>
+      <c r="R52" t="n">
+        <v>1</v>
+      </c>
+      <c r="S52" t="n">
+        <v>-0.5102568936273411</v>
+      </c>
+      <c r="T52" t="b">
+        <v>0</v>
+      </c>
     </row>
     <row r="53">
       <c r="A53" t="inlineStr">
@@ -2881,6 +4101,28 @@
       <c r="L53" t="b">
         <v>1</v>
       </c>
+      <c r="M53" t="n">
+        <v>-0.7597274327306256</v>
+      </c>
+      <c r="N53" t="n">
+        <v>-0.4433893452902123</v>
+      </c>
+      <c r="O53" t="n">
+        <v>0.886</v>
+      </c>
+      <c r="P53" t="n">
+        <v>-0.456353994894077</v>
+      </c>
+      <c r="Q53" t="n">
+        <v>3</v>
+      </c>
+      <c r="R53" t="n">
+        <v>1</v>
+      </c>
+      <c r="S53" t="inlineStr"/>
+      <c r="T53" t="b">
+        <v>0</v>
+      </c>
     </row>
     <row r="54">
       <c r="A54" t="inlineStr">
@@ -2927,6 +4169,30 @@
       <c r="L54" t="b">
         <v>1</v>
       </c>
+      <c r="M54" t="n">
+        <v>-0.7676422338212127</v>
+      </c>
+      <c r="N54" t="n">
+        <v>-0.1917091229553515</v>
+      </c>
+      <c r="O54" t="n">
+        <v>0.847</v>
+      </c>
+      <c r="P54" t="n">
+        <v>-1.009174357385265</v>
+      </c>
+      <c r="Q54" t="n">
+        <v>14</v>
+      </c>
+      <c r="R54" t="n">
+        <v>1</v>
+      </c>
+      <c r="S54" t="n">
+        <v>-0.5534113933631437</v>
+      </c>
+      <c r="T54" t="b">
+        <v>0</v>
+      </c>
     </row>
     <row r="55">
       <c r="A55" t="inlineStr">
@@ -2973,6 +4239,28 @@
       <c r="L55" t="b">
         <v>1</v>
       </c>
+      <c r="M55" t="n">
+        <v>-0.7545744076150935</v>
+      </c>
+      <c r="N55" t="n">
+        <v>-0.4838582521566146</v>
+      </c>
+      <c r="O55" t="n">
+        <v>0.958</v>
+      </c>
+      <c r="P55" t="n">
+        <v>-1.219763215298996</v>
+      </c>
+      <c r="Q55" t="n">
+        <v>18</v>
+      </c>
+      <c r="R55" t="n">
+        <v>1</v>
+      </c>
+      <c r="S55" t="inlineStr"/>
+      <c r="T55" t="b">
+        <v>0</v>
+      </c>
     </row>
     <row r="56">
       <c r="A56" t="inlineStr">
@@ -3019,6 +4307,28 @@
       <c r="L56" t="b">
         <v>1</v>
       </c>
+      <c r="M56" t="n">
+        <v>-0.7693098965234377</v>
+      </c>
+      <c r="N56" t="n">
+        <v>-0.4363069856633109</v>
+      </c>
+      <c r="O56" t="n">
+        <v>0.855</v>
+      </c>
+      <c r="P56" t="n">
+        <v>-0.6377520950803345</v>
+      </c>
+      <c r="Q56" t="n">
+        <v>3</v>
+      </c>
+      <c r="R56" t="n">
+        <v>1</v>
+      </c>
+      <c r="S56" t="inlineStr"/>
+      <c r="T56" t="b">
+        <v>0</v>
+      </c>
     </row>
     <row r="57">
       <c r="A57" t="inlineStr">
@@ -3065,6 +4375,30 @@
       <c r="L57" t="b">
         <v>1</v>
       </c>
+      <c r="M57" t="n">
+        <v>-0.9061007896168644</v>
+      </c>
+      <c r="N57" t="n">
+        <v>-0.4866043441003803</v>
+      </c>
+      <c r="O57" t="n">
+        <v>0.963</v>
+      </c>
+      <c r="P57" t="n">
+        <v>-1.182437996028832</v>
+      </c>
+      <c r="Q57" t="n">
+        <v>15</v>
+      </c>
+      <c r="R57" t="n">
+        <v>1</v>
+      </c>
+      <c r="S57" t="n">
+        <v>-0.6378285813571751</v>
+      </c>
+      <c r="T57" t="b">
+        <v>0</v>
+      </c>
     </row>
     <row r="58">
       <c r="A58" t="inlineStr">
@@ -3111,6 +4445,28 @@
       <c r="L58" t="b">
         <v>1</v>
       </c>
+      <c r="M58" t="n">
+        <v>-0.7217296836950619</v>
+      </c>
+      <c r="N58" t="n">
+        <v>-0.4783898814941205</v>
+      </c>
+      <c r="O58" t="n">
+        <v>0.946</v>
+      </c>
+      <c r="P58" t="n">
+        <v>-0.5915929876991849</v>
+      </c>
+      <c r="Q58" t="n">
+        <v>2</v>
+      </c>
+      <c r="R58" t="n">
+        <v>1</v>
+      </c>
+      <c r="S58" t="inlineStr"/>
+      <c r="T58" t="b">
+        <v>0</v>
+      </c>
     </row>
     <row r="59">
       <c r="A59" t="inlineStr">
@@ -3157,6 +4513,28 @@
       <c r="L59" t="b">
         <v>1</v>
       </c>
+      <c r="M59" t="n">
+        <v>-0.7299876992184966</v>
+      </c>
+      <c r="N59" t="n">
+        <v>-0.5452644424643805</v>
+      </c>
+      <c r="O59" t="n">
+        <v>1</v>
+      </c>
+      <c r="P59" t="n">
+        <v>-0.5680187756846773</v>
+      </c>
+      <c r="Q59" t="n">
+        <v>0</v>
+      </c>
+      <c r="R59" t="n">
+        <v>1</v>
+      </c>
+      <c r="S59" t="inlineStr"/>
+      <c r="T59" t="b">
+        <v>0</v>
+      </c>
     </row>
     <row r="60">
       <c r="A60" t="inlineStr">
@@ -3203,6 +4581,30 @@
       <c r="L60" t="b">
         <v>1</v>
       </c>
+      <c r="M60" t="n">
+        <v>-0.7491699143876224</v>
+      </c>
+      <c r="N60" t="n">
+        <v>-0.4139509924826077</v>
+      </c>
+      <c r="O60" t="n">
+        <v>0.894</v>
+      </c>
+      <c r="P60" t="n">
+        <v>-0.4651918858192855</v>
+      </c>
+      <c r="Q60" t="n">
+        <v>6</v>
+      </c>
+      <c r="R60" t="n">
+        <v>1</v>
+      </c>
+      <c r="S60" t="n">
+        <v>-0.4817934716278975</v>
+      </c>
+      <c r="T60" t="b">
+        <v>0</v>
+      </c>
     </row>
     <row r="61">
       <c r="A61" t="inlineStr">
@@ -3249,6 +4651,28 @@
       <c r="L61" t="b">
         <v>1</v>
       </c>
+      <c r="M61" t="n">
+        <v>-0.8204516027977049</v>
+      </c>
+      <c r="N61" t="n">
+        <v>-0.4644032069316101</v>
+      </c>
+      <c r="O61" t="n">
+        <v>0.946</v>
+      </c>
+      <c r="P61" t="n">
+        <v>-0.8778886753161558</v>
+      </c>
+      <c r="Q61" t="n">
+        <v>8</v>
+      </c>
+      <c r="R61" t="n">
+        <v>1</v>
+      </c>
+      <c r="S61" t="inlineStr"/>
+      <c r="T61" t="b">
+        <v>0</v>
+      </c>
     </row>
     <row r="62">
       <c r="A62" t="inlineStr">
@@ -3295,6 +4719,30 @@
       <c r="L62" t="b">
         <v>0</v>
       </c>
+      <c r="M62" t="n">
+        <v>-0.7335893514548196</v>
+      </c>
+      <c r="N62" t="n">
+        <v>-0.1710950615397271</v>
+      </c>
+      <c r="O62" t="n">
+        <v>0.575</v>
+      </c>
+      <c r="P62" t="n">
+        <v>-0.4750442478522227</v>
+      </c>
+      <c r="Q62" t="n">
+        <v>3</v>
+      </c>
+      <c r="R62" t="n">
+        <v>1</v>
+      </c>
+      <c r="S62" t="n">
+        <v>-0.6394145232712816</v>
+      </c>
+      <c r="T62" t="b">
+        <v>0</v>
+      </c>
     </row>
     <row r="63">
       <c r="A63" t="inlineStr">
@@ -3341,6 +4789,28 @@
       <c r="L63" t="b">
         <v>1</v>
       </c>
+      <c r="M63" t="n">
+        <v>-0.8305863697062951</v>
+      </c>
+      <c r="N63" t="n">
+        <v>-0.4377336438965211</v>
+      </c>
+      <c r="O63" t="n">
+        <v>0.819</v>
+      </c>
+      <c r="P63" t="n">
+        <v>-0.6939021837154955</v>
+      </c>
+      <c r="Q63" t="n">
+        <v>3</v>
+      </c>
+      <c r="R63" t="n">
+        <v>1</v>
+      </c>
+      <c r="S63" t="inlineStr"/>
+      <c r="T63" t="b">
+        <v>0</v>
+      </c>
     </row>
     <row r="64">
       <c r="A64" t="inlineStr">
@@ -3387,6 +4857,30 @@
       <c r="L64" t="b">
         <v>1</v>
       </c>
+      <c r="M64" t="n">
+        <v>-0.7225023787452054</v>
+      </c>
+      <c r="N64" t="n">
+        <v>-0.2532098835550042</v>
+      </c>
+      <c r="O64" t="n">
+        <v>0.74</v>
+      </c>
+      <c r="P64" t="n">
+        <v>-0.4949438962435852</v>
+      </c>
+      <c r="Q64" t="n">
+        <v>6</v>
+      </c>
+      <c r="R64" t="n">
+        <v>1</v>
+      </c>
+      <c r="S64" t="n">
+        <v>-0.4490834435442543</v>
+      </c>
+      <c r="T64" t="b">
+        <v>0</v>
+      </c>
     </row>
     <row r="65">
       <c r="A65" t="inlineStr">
@@ -3433,6 +4927,30 @@
       <c r="L65" t="b">
         <v>1</v>
       </c>
+      <c r="M65" t="n">
+        <v>-0.7384487414982182</v>
+      </c>
+      <c r="N65" t="n">
+        <v>-0.3472954840722806</v>
+      </c>
+      <c r="O65" t="n">
+        <v>0.735</v>
+      </c>
+      <c r="P65" t="n">
+        <v>-0.8310646926615343</v>
+      </c>
+      <c r="Q65" t="n">
+        <v>5</v>
+      </c>
+      <c r="R65" t="n">
+        <v>1</v>
+      </c>
+      <c r="S65" t="n">
+        <v>-0.5404735083025476</v>
+      </c>
+      <c r="T65" t="b">
+        <v>0</v>
+      </c>
     </row>
     <row r="66">
       <c r="A66" t="inlineStr">
@@ -3479,6 +4997,30 @@
       <c r="L66" t="b">
         <v>1</v>
       </c>
+      <c r="M66" t="n">
+        <v>-0.8435696405856929</v>
+      </c>
+      <c r="N66" t="n">
+        <v>-0.09265848043050209</v>
+      </c>
+      <c r="O66" t="n">
+        <v>0.584</v>
+      </c>
+      <c r="P66" t="n">
+        <v>-1.06384655210062</v>
+      </c>
+      <c r="Q66" t="n">
+        <v>16</v>
+      </c>
+      <c r="R66" t="n">
+        <v>1</v>
+      </c>
+      <c r="S66" t="n">
+        <v>-0.406612366159008</v>
+      </c>
+      <c r="T66" t="b">
+        <v>0</v>
+      </c>
     </row>
     <row r="67">
       <c r="A67" t="inlineStr">
@@ -3525,6 +5067,28 @@
       <c r="L67" t="b">
         <v>1</v>
       </c>
+      <c r="M67" t="n">
+        <v>-0.7122927174204319</v>
+      </c>
+      <c r="N67" t="n">
+        <v>-0.4735504085420971</v>
+      </c>
+      <c r="O67" t="n">
+        <v>0.931</v>
+      </c>
+      <c r="P67" t="n">
+        <v>-0.5409572235254618</v>
+      </c>
+      <c r="Q67" t="n">
+        <v>1</v>
+      </c>
+      <c r="R67" t="n">
+        <v>1</v>
+      </c>
+      <c r="S67" t="inlineStr"/>
+      <c r="T67" t="b">
+        <v>0</v>
+      </c>
     </row>
     <row r="68">
       <c r="A68" t="inlineStr">
@@ -3571,6 +5135,30 @@
       <c r="L68" t="b">
         <v>1</v>
       </c>
+      <c r="M68" t="n">
+        <v>-0.6736098746110847</v>
+      </c>
+      <c r="N68" t="n">
+        <v>-0.4713960457356391</v>
+      </c>
+      <c r="O68" t="n">
+        <v>0.923</v>
+      </c>
+      <c r="P68" t="n">
+        <v>-0.9761144912429176</v>
+      </c>
+      <c r="Q68" t="n">
+        <v>14</v>
+      </c>
+      <c r="R68" t="n">
+        <v>1</v>
+      </c>
+      <c r="S68" t="n">
+        <v>-0.4843902512385207</v>
+      </c>
+      <c r="T68" t="b">
+        <v>0</v>
+      </c>
     </row>
     <row r="69">
       <c r="A69" t="inlineStr">
@@ -3617,6 +5205,28 @@
       <c r="L69" t="b">
         <v>0</v>
       </c>
+      <c r="M69" t="n">
+        <v>-0.6950954092693049</v>
+      </c>
+      <c r="N69" t="n">
+        <v>-0.4837325009461344</v>
+      </c>
+      <c r="O69" t="n">
+        <v>0.954</v>
+      </c>
+      <c r="P69" t="n">
+        <v>-0.4159778058357058</v>
+      </c>
+      <c r="Q69" t="n">
+        <v>1</v>
+      </c>
+      <c r="R69" t="n">
+        <v>1</v>
+      </c>
+      <c r="S69" t="inlineStr"/>
+      <c r="T69" t="b">
+        <v>0</v>
+      </c>
     </row>
     <row r="70">
       <c r="A70" t="inlineStr">
@@ -3663,6 +5273,28 @@
       <c r="L70" t="b">
         <v>1</v>
       </c>
+      <c r="M70" t="n">
+        <v>-0.7084230011000947</v>
+      </c>
+      <c r="N70" t="n">
+        <v>-0.3374591100481385</v>
+      </c>
+      <c r="O70" t="n">
+        <v>0.792</v>
+      </c>
+      <c r="P70" t="n">
+        <v>-0.7700393589149928</v>
+      </c>
+      <c r="Q70" t="n">
+        <v>1</v>
+      </c>
+      <c r="R70" t="n">
+        <v>1</v>
+      </c>
+      <c r="S70" t="inlineStr"/>
+      <c r="T70" t="b">
+        <v>0</v>
+      </c>
     </row>
     <row r="71">
       <c r="A71" t="inlineStr">
@@ -3709,6 +5341,30 @@
       <c r="L71" t="b">
         <v>1</v>
       </c>
+      <c r="M71" t="n">
+        <v>-0.6854998612799186</v>
+      </c>
+      <c r="N71" t="n">
+        <v>-0.2313425649150735</v>
+      </c>
+      <c r="O71" t="n">
+        <v>0.803</v>
+      </c>
+      <c r="P71" t="n">
+        <v>-0.9909197173410114</v>
+      </c>
+      <c r="Q71" t="n">
+        <v>14</v>
+      </c>
+      <c r="R71" t="n">
+        <v>1</v>
+      </c>
+      <c r="S71" t="n">
+        <v>-0.4743769149008274</v>
+      </c>
+      <c r="T71" t="b">
+        <v>0</v>
+      </c>
     </row>
     <row r="72">
       <c r="A72" t="inlineStr">
@@ -3755,6 +5411,30 @@
       <c r="L72" t="b">
         <v>1</v>
       </c>
+      <c r="M72" t="n">
+        <v>-0.7077959773264803</v>
+      </c>
+      <c r="N72" t="n">
+        <v>-0.3109452979599228</v>
+      </c>
+      <c r="O72" t="n">
+        <v>0.632</v>
+      </c>
+      <c r="P72" t="n">
+        <v>-1.189531973051574</v>
+      </c>
+      <c r="Q72" t="n">
+        <v>15</v>
+      </c>
+      <c r="R72" t="n">
+        <v>1</v>
+      </c>
+      <c r="S72" t="n">
+        <v>-0.5897492988825257</v>
+      </c>
+      <c r="T72" t="b">
+        <v>0</v>
+      </c>
     </row>
     <row r="73">
       <c r="A73" t="inlineStr">
@@ -3801,6 +5481,30 @@
       <c r="L73" t="b">
         <v>1</v>
       </c>
+      <c r="M73" t="n">
+        <v>-0.8678307527384331</v>
+      </c>
+      <c r="N73" t="n">
+        <v>-0.3104891458577039</v>
+      </c>
+      <c r="O73" t="n">
+        <v>0.731</v>
+      </c>
+      <c r="P73" t="n">
+        <v>-1.058968043208771</v>
+      </c>
+      <c r="Q73" t="n">
+        <v>16</v>
+      </c>
+      <c r="R73" t="n">
+        <v>1</v>
+      </c>
+      <c r="S73" t="n">
+        <v>-0.4048867379553922</v>
+      </c>
+      <c r="T73" t="b">
+        <v>0</v>
+      </c>
     </row>
     <row r="74">
       <c r="A74" t="inlineStr">
@@ -3847,6 +5551,28 @@
       <c r="L74" t="b">
         <v>1</v>
       </c>
+      <c r="M74" t="n">
+        <v>-0.7459926882485236</v>
+      </c>
+      <c r="N74" t="n">
+        <v>-0.3464257388563686</v>
+      </c>
+      <c r="O74" t="n">
+        <v>0.681</v>
+      </c>
+      <c r="P74" t="n">
+        <v>-0.6141710462256644</v>
+      </c>
+      <c r="Q74" t="n">
+        <v>2</v>
+      </c>
+      <c r="R74" t="n">
+        <v>1</v>
+      </c>
+      <c r="S74" t="inlineStr"/>
+      <c r="T74" t="b">
+        <v>0</v>
+      </c>
     </row>
     <row r="75">
       <c r="A75" t="inlineStr">
@@ -3893,6 +5619,30 @@
       <c r="L75" t="b">
         <v>1</v>
       </c>
+      <c r="M75" t="n">
+        <v>-0.850621167994563</v>
+      </c>
+      <c r="N75" t="n">
+        <v>-0.2956165191085919</v>
+      </c>
+      <c r="O75" t="n">
+        <v>0.712</v>
+      </c>
+      <c r="P75" t="n">
+        <v>-0.7441689212853471</v>
+      </c>
+      <c r="Q75" t="n">
+        <v>6</v>
+      </c>
+      <c r="R75" t="n">
+        <v>1</v>
+      </c>
+      <c r="S75" t="n">
+        <v>-0.5798443315788967</v>
+      </c>
+      <c r="T75" t="b">
+        <v>0</v>
+      </c>
     </row>
     <row r="76">
       <c r="A76" t="inlineStr">
@@ -3939,6 +5689,28 @@
       <c r="L76" t="b">
         <v>1</v>
       </c>
+      <c r="M76" t="n">
+        <v>-0.8630561011225075</v>
+      </c>
+      <c r="N76" t="n">
+        <v>-0.1670960129342065</v>
+      </c>
+      <c r="O76" t="n">
+        <v>0.642</v>
+      </c>
+      <c r="P76" t="n">
+        <v>-0.9589585590633402</v>
+      </c>
+      <c r="Q76" t="n">
+        <v>8</v>
+      </c>
+      <c r="R76" t="n">
+        <v>1</v>
+      </c>
+      <c r="S76" t="inlineStr"/>
+      <c r="T76" t="b">
+        <v>0</v>
+      </c>
     </row>
     <row r="77">
       <c r="A77" t="inlineStr">
@@ -3985,6 +5757,28 @@
       <c r="L77" t="b">
         <v>1</v>
       </c>
+      <c r="M77" t="n">
+        <v>-0.7432844232363466</v>
+      </c>
+      <c r="N77" t="n">
+        <v>-0.4600846131745957</v>
+      </c>
+      <c r="O77" t="n">
+        <v>0.843</v>
+      </c>
+      <c r="P77" t="n">
+        <v>-0.4691977800529071</v>
+      </c>
+      <c r="Q77" t="n">
+        <v>3</v>
+      </c>
+      <c r="R77" t="n">
+        <v>1</v>
+      </c>
+      <c r="S77" t="inlineStr"/>
+      <c r="T77" t="b">
+        <v>0</v>
+      </c>
     </row>
     <row r="78">
       <c r="A78" t="inlineStr">
@@ -4031,6 +5825,28 @@
       <c r="L78" t="b">
         <v>1</v>
       </c>
+      <c r="M78" t="n">
+        <v>-0.734990333079965</v>
+      </c>
+      <c r="N78" t="n">
+        <v>-0.3991601415683706</v>
+      </c>
+      <c r="O78" t="n">
+        <v>0.846</v>
+      </c>
+      <c r="P78" t="n">
+        <v>-0.6710493548952888</v>
+      </c>
+      <c r="Q78" t="n">
+        <v>0</v>
+      </c>
+      <c r="R78" t="n">
+        <v>1</v>
+      </c>
+      <c r="S78" t="inlineStr"/>
+      <c r="T78" t="b">
+        <v>0</v>
+      </c>
     </row>
     <row r="79">
       <c r="A79" t="inlineStr">
@@ -4077,6 +5893,28 @@
       <c r="L79" t="b">
         <v>1</v>
       </c>
+      <c r="M79" t="n">
+        <v>-0.6485528235135485</v>
+      </c>
+      <c r="N79" t="n">
+        <v>-0.4769130515209499</v>
+      </c>
+      <c r="O79" t="n">
+        <v>0.917</v>
+      </c>
+      <c r="P79" t="n">
+        <v>-0.7236148533772427</v>
+      </c>
+      <c r="Q79" t="n">
+        <v>3</v>
+      </c>
+      <c r="R79" t="n">
+        <v>0.9026845637583892</v>
+      </c>
+      <c r="S79" t="inlineStr"/>
+      <c r="T79" t="b">
+        <v>0</v>
+      </c>
     </row>
     <row r="80">
       <c r="A80" t="inlineStr">
@@ -4123,6 +5961,30 @@
       <c r="L80" t="b">
         <v>1</v>
       </c>
+      <c r="M80" t="n">
+        <v>-0.9004090958901174</v>
+      </c>
+      <c r="N80" t="n">
+        <v>-0.3337823191990164</v>
+      </c>
+      <c r="O80" t="n">
+        <v>0.582</v>
+      </c>
+      <c r="P80" t="n">
+        <v>-0.7002909381313732</v>
+      </c>
+      <c r="Q80" t="n">
+        <v>0</v>
+      </c>
+      <c r="R80" t="n">
+        <v>0.9026845637583892</v>
+      </c>
+      <c r="S80" t="n">
+        <v>-0.5617379284295128</v>
+      </c>
+      <c r="T80" t="b">
+        <v>0</v>
+      </c>
     </row>
     <row r="81">
       <c r="A81" t="inlineStr">
@@ -4169,6 +6031,28 @@
       <c r="L81" t="b">
         <v>1</v>
       </c>
+      <c r="M81" t="n">
+        <v>-0.6677625111073029</v>
+      </c>
+      <c r="N81" t="n">
+        <v>-0.3909101633017942</v>
+      </c>
+      <c r="O81" t="n">
+        <v>0.6840000000000001</v>
+      </c>
+      <c r="P81" t="n">
+        <v>-0.4552411097740529</v>
+      </c>
+      <c r="Q81" t="n">
+        <v>2</v>
+      </c>
+      <c r="R81" t="n">
+        <v>1</v>
+      </c>
+      <c r="S81" t="inlineStr"/>
+      <c r="T81" t="b">
+        <v>0</v>
+      </c>
     </row>
     <row r="82">
       <c r="A82" t="inlineStr">
@@ -4215,6 +6099,30 @@
       <c r="L82" t="b">
         <v>1</v>
       </c>
+      <c r="M82" t="n">
+        <v>-0.6697943419612395</v>
+      </c>
+      <c r="N82" t="n">
+        <v>-0.2803263694340062</v>
+      </c>
+      <c r="O82" t="n">
+        <v>0.781</v>
+      </c>
+      <c r="P82" t="n">
+        <v>-1.456821326791018</v>
+      </c>
+      <c r="Q82" t="n">
+        <v>24</v>
+      </c>
+      <c r="R82" t="n">
+        <v>1</v>
+      </c>
+      <c r="S82" t="n">
+        <v>-0.5617644506954811</v>
+      </c>
+      <c r="T82" t="b">
+        <v>0</v>
+      </c>
     </row>
     <row r="83">
       <c r="A83" t="inlineStr">
@@ -4261,6 +6169,30 @@
       <c r="L83" t="b">
         <v>1</v>
       </c>
+      <c r="M83" t="n">
+        <v>-0.6916068254937691</v>
+      </c>
+      <c r="N83" t="n">
+        <v>-0.2872578771007067</v>
+      </c>
+      <c r="O83" t="n">
+        <v>0.669</v>
+      </c>
+      <c r="P83" t="n">
+        <v>-0.4772688689809301</v>
+      </c>
+      <c r="Q83" t="n">
+        <v>6</v>
+      </c>
+      <c r="R83" t="n">
+        <v>1</v>
+      </c>
+      <c r="S83" t="n">
+        <v>-0.4073241307819252</v>
+      </c>
+      <c r="T83" t="b">
+        <v>0</v>
+      </c>
     </row>
     <row r="84">
       <c r="A84" t="inlineStr">
@@ -4307,6 +6239,30 @@
       <c r="L84" t="b">
         <v>1</v>
       </c>
+      <c r="M84" t="n">
+        <v>-0.7733371867448966</v>
+      </c>
+      <c r="N84" t="n">
+        <v>-0.1322203737464279</v>
+      </c>
+      <c r="O84" t="n">
+        <v>0.605</v>
+      </c>
+      <c r="P84" t="n">
+        <v>-0.9747880250253556</v>
+      </c>
+      <c r="Q84" t="n">
+        <v>13</v>
+      </c>
+      <c r="R84" t="n">
+        <v>1</v>
+      </c>
+      <c r="S84" t="n">
+        <v>-0.53314579239117</v>
+      </c>
+      <c r="T84" t="b">
+        <v>0</v>
+      </c>
     </row>
     <row r="85">
       <c r="A85" t="inlineStr">
@@ -4353,6 +6309,28 @@
       <c r="L85" t="b">
         <v>1</v>
       </c>
+      <c r="M85" t="n">
+        <v>-0.7653741797779482</v>
+      </c>
+      <c r="N85" t="n">
+        <v>-0.4190137050592593</v>
+      </c>
+      <c r="O85" t="n">
+        <v>0.699</v>
+      </c>
+      <c r="P85" t="n">
+        <v>-1.182795965679451</v>
+      </c>
+      <c r="Q85" t="n">
+        <v>21</v>
+      </c>
+      <c r="R85" t="n">
+        <v>1</v>
+      </c>
+      <c r="S85" t="inlineStr"/>
+      <c r="T85" t="b">
+        <v>0</v>
+      </c>
     </row>
     <row r="86">
       <c r="A86" t="inlineStr">
@@ -4399,6 +6377,30 @@
       <c r="L86" t="b">
         <v>1</v>
       </c>
+      <c r="M86" t="n">
+        <v>-0.8806600041171775</v>
+      </c>
+      <c r="N86" t="n">
+        <v>-0.1742101372114658</v>
+      </c>
+      <c r="O86" t="n">
+        <v>0.5669999999999999</v>
+      </c>
+      <c r="P86" t="n">
+        <v>-0.5251149736546507</v>
+      </c>
+      <c r="Q86" t="n">
+        <v>0</v>
+      </c>
+      <c r="R86" t="n">
+        <v>1</v>
+      </c>
+      <c r="S86" t="n">
+        <v>-0.4539997444361936</v>
+      </c>
+      <c r="T86" t="b">
+        <v>0</v>
+      </c>
     </row>
     <row r="87">
       <c r="A87" t="inlineStr">
@@ -4445,6 +6447,30 @@
       <c r="L87" t="b">
         <v>1</v>
       </c>
+      <c r="M87" t="n">
+        <v>-0.8207411326910962</v>
+      </c>
+      <c r="N87" t="n">
+        <v>-0.3560907905115967</v>
+      </c>
+      <c r="O87" t="n">
+        <v>0.606</v>
+      </c>
+      <c r="P87" t="n">
+        <v>-0.5537695112593262</v>
+      </c>
+      <c r="Q87" t="n">
+        <v>3</v>
+      </c>
+      <c r="R87" t="n">
+        <v>1</v>
+      </c>
+      <c r="S87" t="n">
+        <v>-0.5055087453173113</v>
+      </c>
+      <c r="T87" t="b">
+        <v>0</v>
+      </c>
     </row>
     <row r="88">
       <c r="A88" t="inlineStr">
@@ -4491,6 +6517,30 @@
       <c r="L88" t="b">
         <v>0</v>
       </c>
+      <c r="M88" t="n">
+        <v>-0.6098065088354274</v>
+      </c>
+      <c r="N88" t="n">
+        <v>0.0231870738582407</v>
+      </c>
+      <c r="O88" t="n">
+        <v>0.589</v>
+      </c>
+      <c r="P88" t="n">
+        <v>-0.6080014481446055</v>
+      </c>
+      <c r="Q88" t="n">
+        <v>0</v>
+      </c>
+      <c r="R88" t="n">
+        <v>1</v>
+      </c>
+      <c r="S88" t="n">
+        <v>-0.5170352709021244</v>
+      </c>
+      <c r="T88" t="b">
+        <v>0</v>
+      </c>
     </row>
     <row r="89">
       <c r="A89" t="inlineStr">
@@ -4537,6 +6587,28 @@
       <c r="L89" t="b">
         <v>1</v>
       </c>
+      <c r="M89" t="n">
+        <v>-0.7534908760912196</v>
+      </c>
+      <c r="N89" t="n">
+        <v>-0.4200435982261164</v>
+      </c>
+      <c r="O89" t="n">
+        <v>0.655</v>
+      </c>
+      <c r="P89" t="n">
+        <v>-0.4961789658482341</v>
+      </c>
+      <c r="Q89" t="n">
+        <v>0</v>
+      </c>
+      <c r="R89" t="n">
+        <v>1</v>
+      </c>
+      <c r="S89" t="inlineStr"/>
+      <c r="T89" t="b">
+        <v>0</v>
+      </c>
     </row>
     <row r="90">
       <c r="A90" t="inlineStr">
@@ -4583,6 +6655,28 @@
       <c r="L90" t="b">
         <v>1</v>
       </c>
+      <c r="M90" t="n">
+        <v>-0.6118334084450665</v>
+      </c>
+      <c r="N90" t="n">
+        <v>-0.4253548853018783</v>
+      </c>
+      <c r="O90" t="n">
+        <v>0.613</v>
+      </c>
+      <c r="P90" t="n">
+        <v>-1.162026585608163</v>
+      </c>
+      <c r="Q90" t="n">
+        <v>21</v>
+      </c>
+      <c r="R90" t="n">
+        <v>1</v>
+      </c>
+      <c r="S90" t="inlineStr"/>
+      <c r="T90" t="b">
+        <v>0</v>
+      </c>
     </row>
     <row r="91">
       <c r="A91" t="inlineStr">
@@ -4629,6 +6723,28 @@
       <c r="L91" t="b">
         <v>1</v>
       </c>
+      <c r="M91" t="n">
+        <v>-0.7745214460586115</v>
+      </c>
+      <c r="N91" t="n">
+        <v>-0.2908308640670951</v>
+      </c>
+      <c r="O91" t="n">
+        <v>0.573</v>
+      </c>
+      <c r="P91" t="n">
+        <v>-0.5667966172426316</v>
+      </c>
+      <c r="Q91" t="n">
+        <v>1</v>
+      </c>
+      <c r="R91" t="n">
+        <v>1</v>
+      </c>
+      <c r="S91" t="inlineStr"/>
+      <c r="T91" t="b">
+        <v>0</v>
+      </c>
     </row>
     <row r="92">
       <c r="A92" t="inlineStr">
@@ -4675,6 +6791,30 @@
       <c r="L92" t="b">
         <v>0</v>
       </c>
+      <c r="M92" t="n">
+        <v>-0.8028037616571958</v>
+      </c>
+      <c r="N92" t="n">
+        <v>-0.3220984670333131</v>
+      </c>
+      <c r="O92" t="n">
+        <v>0.517</v>
+      </c>
+      <c r="P92" t="n">
+        <v>-0.6542727483753684</v>
+      </c>
+      <c r="Q92" t="n">
+        <v>2</v>
+      </c>
+      <c r="R92" t="n">
+        <v>1</v>
+      </c>
+      <c r="S92" t="n">
+        <v>-0.4996294356564459</v>
+      </c>
+      <c r="T92" t="b">
+        <v>0</v>
+      </c>
     </row>
     <row r="93">
       <c r="A93" t="inlineStr">
@@ -4721,6 +6861,30 @@
       <c r="L93" t="b">
         <v>1</v>
       </c>
+      <c r="M93" t="n">
+        <v>-0.6747577637351226</v>
+      </c>
+      <c r="N93" t="n">
+        <v>-0.2037950168336169</v>
+      </c>
+      <c r="O93" t="n">
+        <v>0.599</v>
+      </c>
+      <c r="P93" t="n">
+        <v>-2.059879851833106</v>
+      </c>
+      <c r="Q93" t="n">
+        <v>23</v>
+      </c>
+      <c r="R93" t="n">
+        <v>1</v>
+      </c>
+      <c r="S93" t="n">
+        <v>-0.5385624683457566</v>
+      </c>
+      <c r="T93" t="b">
+        <v>0</v>
+      </c>
     </row>
     <row r="94">
       <c r="A94" t="inlineStr">
@@ -4767,6 +6931,30 @@
       <c r="L94" t="b">
         <v>0</v>
       </c>
+      <c r="M94" t="n">
+        <v>-0.7604133481293013</v>
+      </c>
+      <c r="N94" t="n">
+        <v>-0.064487287996132</v>
+      </c>
+      <c r="O94" t="n">
+        <v>0.574</v>
+      </c>
+      <c r="P94" t="n">
+        <v>-0.9523414259356812</v>
+      </c>
+      <c r="Q94" t="n">
+        <v>10</v>
+      </c>
+      <c r="R94" t="n">
+        <v>1</v>
+      </c>
+      <c r="S94" t="n">
+        <v>-0.482779094591359</v>
+      </c>
+      <c r="T94" t="b">
+        <v>0</v>
+      </c>
     </row>
     <row r="95">
       <c r="A95" t="inlineStr">
@@ -4812,6 +7000,30 @@
       </c>
       <c r="L95" t="b">
         <v>1</v>
+      </c>
+      <c r="M95" t="n">
+        <v>-0.7193690362274225</v>
+      </c>
+      <c r="N95" t="n">
+        <v>-0.2077253644823453</v>
+      </c>
+      <c r="O95" t="n">
+        <v>0.496</v>
+      </c>
+      <c r="P95" t="n">
+        <v>-0.9849297289819704</v>
+      </c>
+      <c r="Q95" t="n">
+        <v>8</v>
+      </c>
+      <c r="R95" t="n">
+        <v>1</v>
+      </c>
+      <c r="S95" t="n">
+        <v>-0.6471033843918669</v>
+      </c>
+      <c r="T95" t="b">
+        <v>0</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
revision6_checks.py: genotype framework as for KRAS (other variants excluded), bowel CTNNB1 groups, lineage coefficient adjusted for genotype, both 22Q1 thresholds quantile-matched, adherent-only test with BH; S2 Table
Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/figures/supporting_information/S2_Table.xlsx
+++ b/figures/supporting_information/S2_Table.xlsx
@@ -425,7 +425,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:T95"/>
+  <dimension ref="A1:U95"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -526,6 +526,11 @@
       </c>
       <c r="T1" s="1" t="inlineStr">
         <is>
+          <t>q against adherent lines (BH over 52 non-blood pairs)</t>
+        </is>
+      </c>
+      <c r="U1" s="1" t="inlineStr">
+        <is>
           <t>Partial gene coverage (&lt; 50% of lines)</t>
         </is>
       </c>
@@ -596,7 +601,10 @@
       <c r="S2" t="n">
         <v>-1.584452650068515</v>
       </c>
-      <c r="T2" t="b">
+      <c r="T2" t="n">
+        <v>1.84431017707983e-20</v>
+      </c>
+      <c r="U2" t="b">
         <v>0</v>
       </c>
     </row>
@@ -666,7 +674,10 @@
       <c r="S3" t="n">
         <v>-1.365346268416268</v>
       </c>
-      <c r="T3" t="b">
+      <c r="T3" t="n">
+        <v>5.53554329001041e-27</v>
+      </c>
+      <c r="U3" t="b">
         <v>0</v>
       </c>
     </row>
@@ -736,7 +747,10 @@
       <c r="S4" t="n">
         <v>-1.266030939868908</v>
       </c>
-      <c r="T4" t="b">
+      <c r="T4" t="n">
+        <v>9.665821965631267e-10</v>
+      </c>
+      <c r="U4" t="b">
         <v>0</v>
       </c>
     </row>
@@ -806,7 +820,10 @@
       <c r="S5" t="n">
         <v>-1.23404302816103</v>
       </c>
-      <c r="T5" t="b">
+      <c r="T5" t="n">
+        <v>0.0003041829646107</v>
+      </c>
+      <c r="U5" t="b">
         <v>0</v>
       </c>
     </row>
@@ -876,7 +893,10 @@
       <c r="S6" t="n">
         <v>-1.125878754445281</v>
       </c>
-      <c r="T6" t="b">
+      <c r="T6" t="n">
+        <v>1.86645150924334e-05</v>
+      </c>
+      <c r="U6" t="b">
         <v>0</v>
       </c>
     </row>
@@ -946,7 +966,10 @@
       <c r="S7" t="n">
         <v>-1.109792710320845</v>
       </c>
-      <c r="T7" t="b">
+      <c r="T7" t="n">
+        <v>1.817185583753147e-23</v>
+      </c>
+      <c r="U7" t="b">
         <v>0</v>
       </c>
     </row>
@@ -1016,7 +1039,10 @@
       <c r="S8" t="n">
         <v>-1.058221316126808</v>
       </c>
-      <c r="T8" t="b">
+      <c r="T8" t="n">
+        <v>6.032349262893444e-09</v>
+      </c>
+      <c r="U8" t="b">
         <v>0</v>
       </c>
     </row>
@@ -1084,7 +1110,8 @@
         <v>1</v>
       </c>
       <c r="S9" t="inlineStr"/>
-      <c r="T9" t="b">
+      <c r="T9" t="inlineStr"/>
+      <c r="U9" t="b">
         <v>0</v>
       </c>
     </row>
@@ -1152,7 +1179,8 @@
         <v>1</v>
       </c>
       <c r="S10" t="inlineStr"/>
-      <c r="T10" t="b">
+      <c r="T10" t="inlineStr"/>
+      <c r="U10" t="b">
         <v>0</v>
       </c>
     </row>
@@ -1222,7 +1250,10 @@
       <c r="S11" t="n">
         <v>-1.02620617371</v>
       </c>
-      <c r="T11" t="b">
+      <c r="T11" t="n">
+        <v>0.0006352892138615001</v>
+      </c>
+      <c r="U11" t="b">
         <v>0</v>
       </c>
     </row>
@@ -1292,7 +1323,10 @@
       <c r="S12" t="n">
         <v>-1.009824469373484</v>
       </c>
-      <c r="T12" t="b">
+      <c r="T12" t="n">
+        <v>1.772025227875256e-12</v>
+      </c>
+      <c r="U12" t="b">
         <v>0</v>
       </c>
     </row>
@@ -1362,7 +1396,10 @@
       <c r="S13" t="n">
         <v>-1.006015403525742</v>
       </c>
-      <c r="T13" t="b">
+      <c r="T13" t="n">
+        <v>1.330946155599137e-22</v>
+      </c>
+      <c r="U13" t="b">
         <v>0</v>
       </c>
     </row>
@@ -1432,7 +1469,10 @@
       <c r="S14" t="n">
         <v>-0.9881551348459824</v>
       </c>
-      <c r="T14" t="b">
+      <c r="T14" t="n">
+        <v>2.694633675129323e-09</v>
+      </c>
+      <c r="U14" t="b">
         <v>0</v>
       </c>
     </row>
@@ -1500,7 +1540,8 @@
         <v>1</v>
       </c>
       <c r="S15" t="inlineStr"/>
-      <c r="T15" t="b">
+      <c r="T15" t="inlineStr"/>
+      <c r="U15" t="b">
         <v>0</v>
       </c>
     </row>
@@ -1568,7 +1609,8 @@
         <v>1</v>
       </c>
       <c r="S16" t="inlineStr"/>
-      <c r="T16" t="b">
+      <c r="T16" t="inlineStr"/>
+      <c r="U16" t="b">
         <v>0</v>
       </c>
     </row>
@@ -1638,7 +1680,10 @@
       <c r="S17" t="n">
         <v>-0.7529375255075197</v>
       </c>
-      <c r="T17" t="b">
+      <c r="T17" t="n">
+        <v>9.750687781536828e-06</v>
+      </c>
+      <c r="U17" t="b">
         <v>0</v>
       </c>
     </row>
@@ -1708,7 +1753,10 @@
       <c r="S18" t="n">
         <v>-0.7785534884072509</v>
       </c>
-      <c r="T18" t="b">
+      <c r="T18" t="n">
+        <v>7.485381074359769e-07</v>
+      </c>
+      <c r="U18" t="b">
         <v>0</v>
       </c>
     </row>
@@ -1778,7 +1826,10 @@
       <c r="S19" t="n">
         <v>-0.9059054274829854</v>
       </c>
-      <c r="T19" t="b">
+      <c r="T19" t="n">
+        <v>2.773996537359419e-06</v>
+      </c>
+      <c r="U19" t="b">
         <v>0</v>
       </c>
     </row>
@@ -1848,7 +1899,10 @@
       <c r="S20" t="n">
         <v>-0.8639862304996127</v>
       </c>
-      <c r="T20" t="b">
+      <c r="T20" t="n">
+        <v>1.51471202581867e-08</v>
+      </c>
+      <c r="U20" t="b">
         <v>0</v>
       </c>
     </row>
@@ -1918,7 +1972,10 @@
       <c r="S21" t="n">
         <v>-0.8511794949700303</v>
       </c>
-      <c r="T21" t="b">
+      <c r="T21" t="n">
+        <v>6.63859289517095e-05</v>
+      </c>
+      <c r="U21" t="b">
         <v>0</v>
       </c>
     </row>
@@ -1988,7 +2045,10 @@
       <c r="S22" t="n">
         <v>-0.8198661214223878</v>
       </c>
-      <c r="T22" t="b">
+      <c r="T22" t="n">
+        <v>0.0003204506415732</v>
+      </c>
+      <c r="U22" t="b">
         <v>0</v>
       </c>
     </row>
@@ -2058,7 +2118,10 @@
       <c r="S23" t="n">
         <v>-0.8114075168145537</v>
       </c>
-      <c r="T23" t="b">
+      <c r="T23" t="n">
+        <v>2.461360486887062e-09</v>
+      </c>
+      <c r="U23" t="b">
         <v>0</v>
       </c>
     </row>
@@ -2126,7 +2189,8 @@
         <v>1</v>
       </c>
       <c r="S24" t="inlineStr"/>
-      <c r="T24" t="b">
+      <c r="T24" t="inlineStr"/>
+      <c r="U24" t="b">
         <v>0</v>
       </c>
     </row>
@@ -2194,7 +2258,8 @@
         <v>1</v>
       </c>
       <c r="S25" t="inlineStr"/>
-      <c r="T25" t="b">
+      <c r="T25" t="inlineStr"/>
+      <c r="U25" t="b">
         <v>0</v>
       </c>
     </row>
@@ -2262,7 +2327,8 @@
         <v>0.0620805369127516</v>
       </c>
       <c r="S26" t="inlineStr"/>
-      <c r="T26" t="b">
+      <c r="T26" t="inlineStr"/>
+      <c r="U26" t="b">
         <v>1</v>
       </c>
     </row>
@@ -2330,7 +2396,8 @@
         <v>1</v>
       </c>
       <c r="S27" t="inlineStr"/>
-      <c r="T27" t="b">
+      <c r="T27" t="inlineStr"/>
+      <c r="U27" t="b">
         <v>0</v>
       </c>
     </row>
@@ -2400,7 +2467,10 @@
       <c r="S28" t="n">
         <v>-0.8191204755982007</v>
       </c>
-      <c r="T28" t="b">
+      <c r="T28" t="n">
+        <v>2.28231083225573e-10</v>
+      </c>
+      <c r="U28" t="b">
         <v>0</v>
       </c>
     </row>
@@ -2468,7 +2538,8 @@
         <v>1</v>
       </c>
       <c r="S29" t="inlineStr"/>
-      <c r="T29" t="b">
+      <c r="T29" t="inlineStr"/>
+      <c r="U29" t="b">
         <v>0</v>
       </c>
     </row>
@@ -2538,7 +2609,10 @@
       <c r="S30" t="n">
         <v>-0.839977473932463</v>
       </c>
-      <c r="T30" t="b">
+      <c r="T30" t="n">
+        <v>4.094998870284325e-06</v>
+      </c>
+      <c r="U30" t="b">
         <v>0</v>
       </c>
     </row>
@@ -2606,7 +2680,8 @@
         <v>1</v>
       </c>
       <c r="S31" t="inlineStr"/>
-      <c r="T31" t="b">
+      <c r="T31" t="inlineStr"/>
+      <c r="U31" t="b">
         <v>0</v>
       </c>
     </row>
@@ -2676,7 +2751,10 @@
       <c r="S32" t="n">
         <v>-0.6084736820451923</v>
       </c>
-      <c r="T32" t="b">
+      <c r="T32" t="n">
+        <v>1.550800447577399e-10</v>
+      </c>
+      <c r="U32" t="b">
         <v>0</v>
       </c>
     </row>
@@ -2744,7 +2822,8 @@
         <v>1</v>
       </c>
       <c r="S33" t="inlineStr"/>
-      <c r="T33" t="b">
+      <c r="T33" t="inlineStr"/>
+      <c r="U33" t="b">
         <v>0</v>
       </c>
     </row>
@@ -2812,7 +2891,8 @@
         <v>1</v>
       </c>
       <c r="S34" t="inlineStr"/>
-      <c r="T34" t="b">
+      <c r="T34" t="inlineStr"/>
+      <c r="U34" t="b">
         <v>0</v>
       </c>
     </row>
@@ -2880,7 +2960,8 @@
         <v>1</v>
       </c>
       <c r="S35" t="inlineStr"/>
-      <c r="T35" t="b">
+      <c r="T35" t="inlineStr"/>
+      <c r="U35" t="b">
         <v>0</v>
       </c>
     </row>
@@ -2948,7 +3029,8 @@
         <v>1</v>
       </c>
       <c r="S36" t="inlineStr"/>
-      <c r="T36" t="b">
+      <c r="T36" t="inlineStr"/>
+      <c r="U36" t="b">
         <v>0</v>
       </c>
     </row>
@@ -3018,7 +3100,10 @@
       <c r="S37" t="n">
         <v>-0.5544090465874651</v>
       </c>
-      <c r="T37" t="b">
+      <c r="T37" t="n">
+        <v>5.21302707072996e-05</v>
+      </c>
+      <c r="U37" t="b">
         <v>0</v>
       </c>
     </row>
@@ -3086,7 +3171,8 @@
         <v>0.2642617449664429</v>
       </c>
       <c r="S38" t="inlineStr"/>
-      <c r="T38" t="b">
+      <c r="T38" t="inlineStr"/>
+      <c r="U38" t="b">
         <v>1</v>
       </c>
     </row>
@@ -3154,7 +3240,8 @@
         <v>1</v>
       </c>
       <c r="S39" t="inlineStr"/>
-      <c r="T39" t="b">
+      <c r="T39" t="inlineStr"/>
+      <c r="U39" t="b">
         <v>0</v>
       </c>
     </row>
@@ -3222,7 +3309,8 @@
         <v>1</v>
       </c>
       <c r="S40" t="inlineStr"/>
-      <c r="T40" t="b">
+      <c r="T40" t="inlineStr"/>
+      <c r="U40" t="b">
         <v>0</v>
       </c>
     </row>
@@ -3292,7 +3380,10 @@
       <c r="S41" t="n">
         <v>-0.6853701508326836</v>
       </c>
-      <c r="T41" t="b">
+      <c r="T41" t="n">
+        <v>2.323961430000939e-09</v>
+      </c>
+      <c r="U41" t="b">
         <v>0</v>
       </c>
     </row>
@@ -3362,7 +3453,10 @@
       <c r="S42" t="n">
         <v>-0.7085207064429841</v>
       </c>
-      <c r="T42" t="b">
+      <c r="T42" t="n">
+        <v>2.017026423084941e-12</v>
+      </c>
+      <c r="U42" t="b">
         <v>0</v>
       </c>
     </row>
@@ -3432,7 +3526,10 @@
       <c r="S43" t="n">
         <v>-0.6942113049282915</v>
       </c>
-      <c r="T43" t="b">
+      <c r="T43" t="n">
+        <v>0.0001607163364952</v>
+      </c>
+      <c r="U43" t="b">
         <v>0</v>
       </c>
     </row>
@@ -3500,7 +3597,8 @@
         <v>1</v>
       </c>
       <c r="S44" t="inlineStr"/>
-      <c r="T44" t="b">
+      <c r="T44" t="inlineStr"/>
+      <c r="U44" t="b">
         <v>0</v>
       </c>
     </row>
@@ -3570,7 +3668,10 @@
       <c r="S45" t="n">
         <v>-0.7130512657411576</v>
       </c>
-      <c r="T45" t="b">
+      <c r="T45" t="n">
+        <v>5.702644016334722e-05</v>
+      </c>
+      <c r="U45" t="b">
         <v>0</v>
       </c>
     </row>
@@ -3640,7 +3741,10 @@
       <c r="S46" t="n">
         <v>-0.6843641186634508</v>
       </c>
-      <c r="T46" t="b">
+      <c r="T46" t="n">
+        <v>2.548991064761546e-07</v>
+      </c>
+      <c r="U46" t="b">
         <v>0</v>
       </c>
     </row>
@@ -3708,7 +3812,8 @@
         <v>0.3196308724832215</v>
       </c>
       <c r="S47" t="inlineStr"/>
-      <c r="T47" t="b">
+      <c r="T47" t="inlineStr"/>
+      <c r="U47" t="b">
         <v>1</v>
       </c>
     </row>
@@ -3778,7 +3883,10 @@
       <c r="S48" t="n">
         <v>-0.6988467703448962</v>
       </c>
-      <c r="T48" t="b">
+      <c r="T48" t="n">
+        <v>2.721511447344206e-05</v>
+      </c>
+      <c r="U48" t="b">
         <v>0</v>
       </c>
     </row>
@@ -3846,7 +3954,8 @@
         <v>1</v>
       </c>
       <c r="S49" t="inlineStr"/>
-      <c r="T49" t="b">
+      <c r="T49" t="inlineStr"/>
+      <c r="U49" t="b">
         <v>0</v>
       </c>
     </row>
@@ -3914,7 +4023,8 @@
         <v>1</v>
       </c>
       <c r="S50" t="inlineStr"/>
-      <c r="T50" t="b">
+      <c r="T50" t="inlineStr"/>
+      <c r="U50" t="b">
         <v>0</v>
       </c>
     </row>
@@ -3982,7 +4092,8 @@
         <v>1</v>
       </c>
       <c r="S51" t="inlineStr"/>
-      <c r="T51" t="b">
+      <c r="T51" t="inlineStr"/>
+      <c r="U51" t="b">
         <v>0</v>
       </c>
     </row>
@@ -4052,7 +4163,10 @@
       <c r="S52" t="n">
         <v>-0.5102568936273411</v>
       </c>
-      <c r="T52" t="b">
+      <c r="T52" t="n">
+        <v>2.929676306635483e-05</v>
+      </c>
+      <c r="U52" t="b">
         <v>0</v>
       </c>
     </row>
@@ -4120,7 +4234,8 @@
         <v>1</v>
       </c>
       <c r="S53" t="inlineStr"/>
-      <c r="T53" t="b">
+      <c r="T53" t="inlineStr"/>
+      <c r="U53" t="b">
         <v>0</v>
       </c>
     </row>
@@ -4190,7 +4305,10 @@
       <c r="S54" t="n">
         <v>-0.5534113933631437</v>
       </c>
-      <c r="T54" t="b">
+      <c r="T54" t="n">
+        <v>0.0011012533721359</v>
+      </c>
+      <c r="U54" t="b">
         <v>0</v>
       </c>
     </row>
@@ -4258,7 +4376,8 @@
         <v>1</v>
       </c>
       <c r="S55" t="inlineStr"/>
-      <c r="T55" t="b">
+      <c r="T55" t="inlineStr"/>
+      <c r="U55" t="b">
         <v>0</v>
       </c>
     </row>
@@ -4326,7 +4445,8 @@
         <v>1</v>
       </c>
       <c r="S56" t="inlineStr"/>
-      <c r="T56" t="b">
+      <c r="T56" t="inlineStr"/>
+      <c r="U56" t="b">
         <v>0</v>
       </c>
     </row>
@@ -4396,7 +4516,10 @@
       <c r="S57" t="n">
         <v>-0.6378285813571751</v>
       </c>
-      <c r="T57" t="b">
+      <c r="T57" t="n">
+        <v>6.24070329558384e-11</v>
+      </c>
+      <c r="U57" t="b">
         <v>0</v>
       </c>
     </row>
@@ -4464,7 +4587,8 @@
         <v>1</v>
       </c>
       <c r="S58" t="inlineStr"/>
-      <c r="T58" t="b">
+      <c r="T58" t="inlineStr"/>
+      <c r="U58" t="b">
         <v>0</v>
       </c>
     </row>
@@ -4532,7 +4656,8 @@
         <v>1</v>
       </c>
       <c r="S59" t="inlineStr"/>
-      <c r="T59" t="b">
+      <c r="T59" t="inlineStr"/>
+      <c r="U59" t="b">
         <v>0</v>
       </c>
     </row>
@@ -4602,7 +4727,10 @@
       <c r="S60" t="n">
         <v>-0.4817934716278975</v>
       </c>
-      <c r="T60" t="b">
+      <c r="T60" t="n">
+        <v>7.485381074359769e-07</v>
+      </c>
+      <c r="U60" t="b">
         <v>0</v>
       </c>
     </row>
@@ -4670,7 +4798,8 @@
         <v>1</v>
       </c>
       <c r="S61" t="inlineStr"/>
-      <c r="T61" t="b">
+      <c r="T61" t="inlineStr"/>
+      <c r="U61" t="b">
         <v>0</v>
       </c>
     </row>
@@ -4740,7 +4869,10 @@
       <c r="S62" t="n">
         <v>-0.6394145232712816</v>
       </c>
-      <c r="T62" t="b">
+      <c r="T62" t="n">
+        <v>0.0003143970681586</v>
+      </c>
+      <c r="U62" t="b">
         <v>0</v>
       </c>
     </row>
@@ -4808,7 +4940,8 @@
         <v>1</v>
       </c>
       <c r="S63" t="inlineStr"/>
-      <c r="T63" t="b">
+      <c r="T63" t="inlineStr"/>
+      <c r="U63" t="b">
         <v>0</v>
       </c>
     </row>
@@ -4878,7 +5011,10 @@
       <c r="S64" t="n">
         <v>-0.4490834435442543</v>
       </c>
-      <c r="T64" t="b">
+      <c r="T64" t="n">
+        <v>0.0063128685715897</v>
+      </c>
+      <c r="U64" t="b">
         <v>0</v>
       </c>
     </row>
@@ -4948,7 +5084,10 @@
       <c r="S65" t="n">
         <v>-0.5404735083025476</v>
       </c>
-      <c r="T65" t="b">
+      <c r="T65" t="n">
+        <v>4.377795310824934e-06</v>
+      </c>
+      <c r="U65" t="b">
         <v>0</v>
       </c>
     </row>
@@ -5018,7 +5157,10 @@
       <c r="S66" t="n">
         <v>-0.406612366159008</v>
       </c>
-      <c r="T66" t="b">
+      <c r="T66" t="n">
+        <v>0.0101388932809592</v>
+      </c>
+      <c r="U66" t="b">
         <v>0</v>
       </c>
     </row>
@@ -5086,7 +5228,8 @@
         <v>1</v>
       </c>
       <c r="S67" t="inlineStr"/>
-      <c r="T67" t="b">
+      <c r="T67" t="inlineStr"/>
+      <c r="U67" t="b">
         <v>0</v>
       </c>
     </row>
@@ -5156,7 +5299,10 @@
       <c r="S68" t="n">
         <v>-0.4843902512385207</v>
       </c>
-      <c r="T68" t="b">
+      <c r="T68" t="n">
+        <v>9.665821965631267e-10</v>
+      </c>
+      <c r="U68" t="b">
         <v>0</v>
       </c>
     </row>
@@ -5224,7 +5370,8 @@
         <v>1</v>
       </c>
       <c r="S69" t="inlineStr"/>
-      <c r="T69" t="b">
+      <c r="T69" t="inlineStr"/>
+      <c r="U69" t="b">
         <v>0</v>
       </c>
     </row>
@@ -5292,7 +5439,8 @@
         <v>1</v>
       </c>
       <c r="S70" t="inlineStr"/>
-      <c r="T70" t="b">
+      <c r="T70" t="inlineStr"/>
+      <c r="U70" t="b">
         <v>0</v>
       </c>
     </row>
@@ -5362,7 +5510,10 @@
       <c r="S71" t="n">
         <v>-0.4743769149008274</v>
       </c>
-      <c r="T71" t="b">
+      <c r="T71" t="n">
+        <v>2.806305324557342e-05</v>
+      </c>
+      <c r="U71" t="b">
         <v>0</v>
       </c>
     </row>
@@ -5432,7 +5583,10 @@
       <c r="S72" t="n">
         <v>-0.5897492988825257</v>
       </c>
-      <c r="T72" t="b">
+      <c r="T72" t="n">
+        <v>2.674217199348652e-07</v>
+      </c>
+      <c r="U72" t="b">
         <v>0</v>
       </c>
     </row>
@@ -5502,7 +5656,10 @@
       <c r="S73" t="n">
         <v>-0.4048867379553922</v>
       </c>
-      <c r="T73" t="b">
+      <c r="T73" t="n">
+        <v>0.0025987128700893</v>
+      </c>
+      <c r="U73" t="b">
         <v>0</v>
       </c>
     </row>
@@ -5570,7 +5727,8 @@
         <v>1</v>
       </c>
       <c r="S74" t="inlineStr"/>
-      <c r="T74" t="b">
+      <c r="T74" t="inlineStr"/>
+      <c r="U74" t="b">
         <v>0</v>
       </c>
     </row>
@@ -5640,7 +5798,10 @@
       <c r="S75" t="n">
         <v>-0.5798443315788967</v>
       </c>
-      <c r="T75" t="b">
+      <c r="T75" t="n">
+        <v>1.007538783362769e-06</v>
+      </c>
+      <c r="U75" t="b">
         <v>0</v>
       </c>
     </row>
@@ -5708,7 +5869,8 @@
         <v>1</v>
       </c>
       <c r="S76" t="inlineStr"/>
-      <c r="T76" t="b">
+      <c r="T76" t="inlineStr"/>
+      <c r="U76" t="b">
         <v>0</v>
       </c>
     </row>
@@ -5776,7 +5938,8 @@
         <v>1</v>
       </c>
       <c r="S77" t="inlineStr"/>
-      <c r="T77" t="b">
+      <c r="T77" t="inlineStr"/>
+      <c r="U77" t="b">
         <v>0</v>
       </c>
     </row>
@@ -5844,7 +6007,8 @@
         <v>1</v>
       </c>
       <c r="S78" t="inlineStr"/>
-      <c r="T78" t="b">
+      <c r="T78" t="inlineStr"/>
+      <c r="U78" t="b">
         <v>0</v>
       </c>
     </row>
@@ -5912,7 +6076,8 @@
         <v>0.9026845637583892</v>
       </c>
       <c r="S79" t="inlineStr"/>
-      <c r="T79" t="b">
+      <c r="T79" t="inlineStr"/>
+      <c r="U79" t="b">
         <v>0</v>
       </c>
     </row>
@@ -5982,7 +6147,10 @@
       <c r="S80" t="n">
         <v>-0.5617379284295128</v>
       </c>
-      <c r="T80" t="b">
+      <c r="T80" t="n">
+        <v>2.548991064761546e-07</v>
+      </c>
+      <c r="U80" t="b">
         <v>0</v>
       </c>
     </row>
@@ -6050,7 +6218,8 @@
         <v>1</v>
       </c>
       <c r="S81" t="inlineStr"/>
-      <c r="T81" t="b">
+      <c r="T81" t="inlineStr"/>
+      <c r="U81" t="b">
         <v>0</v>
       </c>
     </row>
@@ -6120,7 +6289,10 @@
       <c r="S82" t="n">
         <v>-0.5617644506954811</v>
       </c>
-      <c r="T82" t="b">
+      <c r="T82" t="n">
+        <v>2.038848754406467e-05</v>
+      </c>
+      <c r="U82" t="b">
         <v>0</v>
       </c>
     </row>
@@ -6190,7 +6362,10 @@
       <c r="S83" t="n">
         <v>-0.4073241307819252</v>
       </c>
-      <c r="T83" t="b">
+      <c r="T83" t="n">
+        <v>0.000223370626048</v>
+      </c>
+      <c r="U83" t="b">
         <v>0</v>
       </c>
     </row>
@@ -6260,7 +6435,10 @@
       <c r="S84" t="n">
         <v>-0.53314579239117</v>
       </c>
-      <c r="T84" t="b">
+      <c r="T84" t="n">
+        <v>0.0004260732876121</v>
+      </c>
+      <c r="U84" t="b">
         <v>0</v>
       </c>
     </row>
@@ -6328,7 +6506,8 @@
         <v>1</v>
       </c>
       <c r="S85" t="inlineStr"/>
-      <c r="T85" t="b">
+      <c r="T85" t="inlineStr"/>
+      <c r="U85" t="b">
         <v>0</v>
       </c>
     </row>
@@ -6398,7 +6577,10 @@
       <c r="S86" t="n">
         <v>-0.4539997444361936</v>
       </c>
-      <c r="T86" t="b">
+      <c r="T86" t="n">
+        <v>0.0005835530108741</v>
+      </c>
+      <c r="U86" t="b">
         <v>0</v>
       </c>
     </row>
@@ -6468,7 +6650,10 @@
       <c r="S87" t="n">
         <v>-0.5055087453173113</v>
       </c>
-      <c r="T87" t="b">
+      <c r="T87" t="n">
+        <v>7.485381074359769e-07</v>
+      </c>
+      <c r="U87" t="b">
         <v>0</v>
       </c>
     </row>
@@ -6538,7 +6723,10 @@
       <c r="S88" t="n">
         <v>-0.5170352709021244</v>
       </c>
-      <c r="T88" t="b">
+      <c r="T88" t="n">
+        <v>0.0005281361209666</v>
+      </c>
+      <c r="U88" t="b">
         <v>0</v>
       </c>
     </row>
@@ -6606,7 +6794,8 @@
         <v>1</v>
       </c>
       <c r="S89" t="inlineStr"/>
-      <c r="T89" t="b">
+      <c r="T89" t="inlineStr"/>
+      <c r="U89" t="b">
         <v>0</v>
       </c>
     </row>
@@ -6674,7 +6863,8 @@
         <v>1</v>
       </c>
       <c r="S90" t="inlineStr"/>
-      <c r="T90" t="b">
+      <c r="T90" t="inlineStr"/>
+      <c r="U90" t="b">
         <v>0</v>
       </c>
     </row>
@@ -6742,7 +6932,8 @@
         <v>1</v>
       </c>
       <c r="S91" t="inlineStr"/>
-      <c r="T91" t="b">
+      <c r="T91" t="inlineStr"/>
+      <c r="U91" t="b">
         <v>0</v>
       </c>
     </row>
@@ -6812,7 +7003,10 @@
       <c r="S92" t="n">
         <v>-0.4996294356564459</v>
       </c>
-      <c r="T92" t="b">
+      <c r="T92" t="n">
+        <v>5.017080770875738e-09</v>
+      </c>
+      <c r="U92" t="b">
         <v>0</v>
       </c>
     </row>
@@ -6882,7 +7076,10 @@
       <c r="S93" t="n">
         <v>-0.5385624683457566</v>
       </c>
-      <c r="T93" t="b">
+      <c r="T93" t="n">
+        <v>4.138322123820952e-07</v>
+      </c>
+      <c r="U93" t="b">
         <v>0</v>
       </c>
     </row>
@@ -6952,7 +7149,10 @@
       <c r="S94" t="n">
         <v>-0.482779094591359</v>
       </c>
-      <c r="T94" t="b">
+      <c r="T94" t="n">
+        <v>0.0010118338796103</v>
+      </c>
+      <c r="U94" t="b">
         <v>0</v>
       </c>
     </row>
@@ -7022,7 +7222,10 @@
       <c r="S95" t="n">
         <v>-0.6471033843918669</v>
       </c>
-      <c r="T95" t="b">
+      <c r="T95" t="n">
+        <v>1.56053294854902e-07</v>
+      </c>
+      <c r="U95" t="b">
         <v>0</v>
       </c>
     </row>

</xml_diff>

<commit_message>
confidence_tiers.py: confidence tiers of the prioritised pairs from existing checks; S2 Table columns
Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/figures/supporting_information/S2_Table.xlsx
+++ b/figures/supporting_information/S2_Table.xlsx
@@ -425,7 +425,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:U95"/>
+  <dimension ref="A1:AB95"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -534,6 +534,41 @@
           <t>Partial gene coverage (&lt; 50% of lines)</t>
         </is>
       </c>
+      <c r="V1" s="1" t="inlineStr">
+        <is>
+          <t>Confidence tier</t>
+        </is>
+      </c>
+      <c r="W1" s="1" t="inlineStr">
+        <is>
+          <t>Evidence: bootstrap interval below -0.5</t>
+        </is>
+      </c>
+      <c r="X1" s="1" t="inlineStr">
+        <is>
+          <t>Evidence: one model per patient</t>
+        </is>
+      </c>
+      <c r="Y1" s="1" t="inlineStr">
+        <is>
+          <t>Evidence: 22Q1</t>
+        </is>
+      </c>
+      <c r="Z1" s="1" t="inlineStr">
+        <is>
+          <t>Evidence: culture format</t>
+        </is>
+      </c>
+      <c r="AA1" s="1" t="inlineStr">
+        <is>
+          <t>Evidence: independent replication (Project Score)</t>
+        </is>
+      </c>
+      <c r="AB1" s="1" t="inlineStr">
+        <is>
+          <t>Selectivity without suspension lines in the comparison group</t>
+        </is>
+      </c>
     </row>
     <row r="2">
       <c r="A2" t="inlineStr">
@@ -607,6 +642,39 @@
       <c r="U2" t="b">
         <v>0</v>
       </c>
+      <c r="V2" t="inlineStr">
+        <is>
+          <t>high</t>
+        </is>
+      </c>
+      <c r="W2" t="inlineStr">
+        <is>
+          <t>pass</t>
+        </is>
+      </c>
+      <c r="X2" t="inlineStr">
+        <is>
+          <t>pass</t>
+        </is>
+      </c>
+      <c r="Y2" t="inlineStr">
+        <is>
+          <t>pass</t>
+        </is>
+      </c>
+      <c r="Z2" t="inlineStr">
+        <is>
+          <t>pass</t>
+        </is>
+      </c>
+      <c r="AA2" t="inlineStr">
+        <is>
+          <t>pass</t>
+        </is>
+      </c>
+      <c r="AB2" t="n">
+        <v>-1.58201152192072</v>
+      </c>
     </row>
     <row r="3">
       <c r="A3" t="inlineStr">
@@ -680,6 +748,39 @@
       <c r="U3" t="b">
         <v>0</v>
       </c>
+      <c r="V3" t="inlineStr">
+        <is>
+          <t>high</t>
+        </is>
+      </c>
+      <c r="W3" t="inlineStr">
+        <is>
+          <t>pass</t>
+        </is>
+      </c>
+      <c r="X3" t="inlineStr">
+        <is>
+          <t>pass</t>
+        </is>
+      </c>
+      <c r="Y3" t="inlineStr">
+        <is>
+          <t>pass</t>
+        </is>
+      </c>
+      <c r="Z3" t="inlineStr">
+        <is>
+          <t>pass</t>
+        </is>
+      </c>
+      <c r="AA3" t="inlineStr">
+        <is>
+          <t>uninformative</t>
+        </is>
+      </c>
+      <c r="AB3" t="n">
+        <v>-1.365346268416268</v>
+      </c>
     </row>
     <row r="4">
       <c r="A4" t="inlineStr">
@@ -753,6 +854,39 @@
       <c r="U4" t="b">
         <v>0</v>
       </c>
+      <c r="V4" t="inlineStr">
+        <is>
+          <t>high</t>
+        </is>
+      </c>
+      <c r="W4" t="inlineStr">
+        <is>
+          <t>pass</t>
+        </is>
+      </c>
+      <c r="X4" t="inlineStr">
+        <is>
+          <t>pass</t>
+        </is>
+      </c>
+      <c r="Y4" t="inlineStr">
+        <is>
+          <t>pass</t>
+        </is>
+      </c>
+      <c r="Z4" t="inlineStr">
+        <is>
+          <t>pass</t>
+        </is>
+      </c>
+      <c r="AA4" t="inlineStr">
+        <is>
+          <t>uninformative</t>
+        </is>
+      </c>
+      <c r="AB4" t="n">
+        <v>-1.26224975866103</v>
+      </c>
     </row>
     <row r="5">
       <c r="A5" t="inlineStr">
@@ -826,6 +960,39 @@
       <c r="U5" t="b">
         <v>0</v>
       </c>
+      <c r="V5" t="inlineStr">
+        <is>
+          <t>low</t>
+        </is>
+      </c>
+      <c r="W5" t="inlineStr">
+        <is>
+          <t>fail</t>
+        </is>
+      </c>
+      <c r="X5" t="inlineStr">
+        <is>
+          <t>pass</t>
+        </is>
+      </c>
+      <c r="Y5" t="inlineStr">
+        <is>
+          <t>uninformative</t>
+        </is>
+      </c>
+      <c r="Z5" t="inlineStr">
+        <is>
+          <t>pass</t>
+        </is>
+      </c>
+      <c r="AA5" t="inlineStr">
+        <is>
+          <t>uninformative</t>
+        </is>
+      </c>
+      <c r="AB5" t="n">
+        <v>-1.238492317464168</v>
+      </c>
     </row>
     <row r="6">
       <c r="A6" t="inlineStr">
@@ -899,6 +1066,39 @@
       <c r="U6" t="b">
         <v>0</v>
       </c>
+      <c r="V6" t="inlineStr">
+        <is>
+          <t>high</t>
+        </is>
+      </c>
+      <c r="W6" t="inlineStr">
+        <is>
+          <t>pass</t>
+        </is>
+      </c>
+      <c r="X6" t="inlineStr">
+        <is>
+          <t>pass</t>
+        </is>
+      </c>
+      <c r="Y6" t="inlineStr">
+        <is>
+          <t>pass</t>
+        </is>
+      </c>
+      <c r="Z6" t="inlineStr">
+        <is>
+          <t>pass</t>
+        </is>
+      </c>
+      <c r="AA6" t="inlineStr">
+        <is>
+          <t>uninformative</t>
+        </is>
+      </c>
+      <c r="AB6" t="n">
+        <v>-1.125345804313242</v>
+      </c>
     </row>
     <row r="7">
       <c r="A7" t="inlineStr">
@@ -972,6 +1172,39 @@
       <c r="U7" t="b">
         <v>0</v>
       </c>
+      <c r="V7" t="inlineStr">
+        <is>
+          <t>medium</t>
+        </is>
+      </c>
+      <c r="W7" t="inlineStr">
+        <is>
+          <t>pass</t>
+        </is>
+      </c>
+      <c r="X7" t="inlineStr">
+        <is>
+          <t>pass</t>
+        </is>
+      </c>
+      <c r="Y7" t="inlineStr">
+        <is>
+          <t>pass</t>
+        </is>
+      </c>
+      <c r="Z7" t="inlineStr">
+        <is>
+          <t>pass</t>
+        </is>
+      </c>
+      <c r="AA7" t="inlineStr">
+        <is>
+          <t>fail</t>
+        </is>
+      </c>
+      <c r="AB7" t="n">
+        <v>-1.113757459659644</v>
+      </c>
     </row>
     <row r="8">
       <c r="A8" t="inlineStr">
@@ -1045,6 +1278,39 @@
       <c r="U8" t="b">
         <v>0</v>
       </c>
+      <c r="V8" t="inlineStr">
+        <is>
+          <t>high</t>
+        </is>
+      </c>
+      <c r="W8" t="inlineStr">
+        <is>
+          <t>pass</t>
+        </is>
+      </c>
+      <c r="X8" t="inlineStr">
+        <is>
+          <t>pass</t>
+        </is>
+      </c>
+      <c r="Y8" t="inlineStr">
+        <is>
+          <t>pass</t>
+        </is>
+      </c>
+      <c r="Z8" t="inlineStr">
+        <is>
+          <t>pass</t>
+        </is>
+      </c>
+      <c r="AA8" t="inlineStr">
+        <is>
+          <t>uninformative</t>
+        </is>
+      </c>
+      <c r="AB8" t="n">
+        <v>-1.072469868432948</v>
+      </c>
     </row>
     <row r="9">
       <c r="A9" t="inlineStr">
@@ -1114,6 +1380,39 @@
       <c r="U9" t="b">
         <v>0</v>
       </c>
+      <c r="V9" t="inlineStr">
+        <is>
+          <t>high</t>
+        </is>
+      </c>
+      <c r="W9" t="inlineStr">
+        <is>
+          <t>pass</t>
+        </is>
+      </c>
+      <c r="X9" t="inlineStr">
+        <is>
+          <t>pass</t>
+        </is>
+      </c>
+      <c r="Y9" t="inlineStr">
+        <is>
+          <t>pass</t>
+        </is>
+      </c>
+      <c r="Z9" t="inlineStr">
+        <is>
+          <t>pass</t>
+        </is>
+      </c>
+      <c r="AA9" t="inlineStr">
+        <is>
+          <t>uninformative</t>
+        </is>
+      </c>
+      <c r="AB9" t="n">
+        <v>-1.072872853944649</v>
+      </c>
     </row>
     <row r="10">
       <c r="A10" t="inlineStr">
@@ -1183,6 +1482,39 @@
       <c r="U10" t="b">
         <v>0</v>
       </c>
+      <c r="V10" t="inlineStr">
+        <is>
+          <t>high</t>
+        </is>
+      </c>
+      <c r="W10" t="inlineStr">
+        <is>
+          <t>pass</t>
+        </is>
+      </c>
+      <c r="X10" t="inlineStr">
+        <is>
+          <t>pass</t>
+        </is>
+      </c>
+      <c r="Y10" t="inlineStr">
+        <is>
+          <t>pass</t>
+        </is>
+      </c>
+      <c r="Z10" t="inlineStr">
+        <is>
+          <t>pass</t>
+        </is>
+      </c>
+      <c r="AA10" t="inlineStr">
+        <is>
+          <t>uninformative</t>
+        </is>
+      </c>
+      <c r="AB10" t="n">
+        <v>-1.082806882382966</v>
+      </c>
     </row>
     <row r="11">
       <c r="A11" t="inlineStr">
@@ -1256,6 +1588,39 @@
       <c r="U11" t="b">
         <v>0</v>
       </c>
+      <c r="V11" t="inlineStr">
+        <is>
+          <t>low</t>
+        </is>
+      </c>
+      <c r="W11" t="inlineStr">
+        <is>
+          <t>fail</t>
+        </is>
+      </c>
+      <c r="X11" t="inlineStr">
+        <is>
+          <t>fail</t>
+        </is>
+      </c>
+      <c r="Y11" t="inlineStr">
+        <is>
+          <t>pass</t>
+        </is>
+      </c>
+      <c r="Z11" t="inlineStr">
+        <is>
+          <t>pass</t>
+        </is>
+      </c>
+      <c r="AA11" t="inlineStr">
+        <is>
+          <t>uninformative</t>
+        </is>
+      </c>
+      <c r="AB11" t="n">
+        <v>-1.031480749922119</v>
+      </c>
     </row>
     <row r="12">
       <c r="A12" t="inlineStr">
@@ -1329,6 +1694,39 @@
       <c r="U12" t="b">
         <v>0</v>
       </c>
+      <c r="V12" t="inlineStr">
+        <is>
+          <t>medium</t>
+        </is>
+      </c>
+      <c r="W12" t="inlineStr">
+        <is>
+          <t>fail</t>
+        </is>
+      </c>
+      <c r="X12" t="inlineStr">
+        <is>
+          <t>pass</t>
+        </is>
+      </c>
+      <c r="Y12" t="inlineStr">
+        <is>
+          <t>pass</t>
+        </is>
+      </c>
+      <c r="Z12" t="inlineStr">
+        <is>
+          <t>pass</t>
+        </is>
+      </c>
+      <c r="AA12" t="inlineStr">
+        <is>
+          <t>uninformative</t>
+        </is>
+      </c>
+      <c r="AB12" t="n">
+        <v>-1.012640543351392</v>
+      </c>
     </row>
     <row r="13">
       <c r="A13" t="inlineStr">
@@ -1402,6 +1800,39 @@
       <c r="U13" t="b">
         <v>0</v>
       </c>
+      <c r="V13" t="inlineStr">
+        <is>
+          <t>high</t>
+        </is>
+      </c>
+      <c r="W13" t="inlineStr">
+        <is>
+          <t>pass</t>
+        </is>
+      </c>
+      <c r="X13" t="inlineStr">
+        <is>
+          <t>pass</t>
+        </is>
+      </c>
+      <c r="Y13" t="inlineStr">
+        <is>
+          <t>pass</t>
+        </is>
+      </c>
+      <c r="Z13" t="inlineStr">
+        <is>
+          <t>pass</t>
+        </is>
+      </c>
+      <c r="AA13" t="inlineStr">
+        <is>
+          <t>uninformative</t>
+        </is>
+      </c>
+      <c r="AB13" t="n">
+        <v>-1.004424871336947</v>
+      </c>
     </row>
     <row r="14">
       <c r="A14" t="inlineStr">
@@ -1475,6 +1906,39 @@
       <c r="U14" t="b">
         <v>0</v>
       </c>
+      <c r="V14" t="inlineStr">
+        <is>
+          <t>high</t>
+        </is>
+      </c>
+      <c r="W14" t="inlineStr">
+        <is>
+          <t>pass</t>
+        </is>
+      </c>
+      <c r="X14" t="inlineStr">
+        <is>
+          <t>pass</t>
+        </is>
+      </c>
+      <c r="Y14" t="inlineStr">
+        <is>
+          <t>pass</t>
+        </is>
+      </c>
+      <c r="Z14" t="inlineStr">
+        <is>
+          <t>pass</t>
+        </is>
+      </c>
+      <c r="AA14" t="inlineStr">
+        <is>
+          <t>uninformative</t>
+        </is>
+      </c>
+      <c r="AB14" t="n">
+        <v>-0.9882905978980336</v>
+      </c>
     </row>
     <row r="15">
       <c r="A15" t="inlineStr">
@@ -1544,6 +2008,39 @@
       <c r="U15" t="b">
         <v>0</v>
       </c>
+      <c r="V15" t="inlineStr">
+        <is>
+          <t>high</t>
+        </is>
+      </c>
+      <c r="W15" t="inlineStr">
+        <is>
+          <t>pass</t>
+        </is>
+      </c>
+      <c r="X15" t="inlineStr">
+        <is>
+          <t>pass</t>
+        </is>
+      </c>
+      <c r="Y15" t="inlineStr">
+        <is>
+          <t>pass</t>
+        </is>
+      </c>
+      <c r="Z15" t="inlineStr">
+        <is>
+          <t>pass</t>
+        </is>
+      </c>
+      <c r="AA15" t="inlineStr">
+        <is>
+          <t>pass</t>
+        </is>
+      </c>
+      <c r="AB15" t="n">
+        <v>-0.9639799440870452</v>
+      </c>
     </row>
     <row r="16">
       <c r="A16" t="inlineStr">
@@ -1613,6 +2110,39 @@
       <c r="U16" t="b">
         <v>0</v>
       </c>
+      <c r="V16" t="inlineStr">
+        <is>
+          <t>low</t>
+        </is>
+      </c>
+      <c r="W16" t="inlineStr">
+        <is>
+          <t>fail</t>
+        </is>
+      </c>
+      <c r="X16" t="inlineStr">
+        <is>
+          <t>pass</t>
+        </is>
+      </c>
+      <c r="Y16" t="inlineStr">
+        <is>
+          <t>pass</t>
+        </is>
+      </c>
+      <c r="Z16" t="inlineStr">
+        <is>
+          <t>pass</t>
+        </is>
+      </c>
+      <c r="AA16" t="inlineStr">
+        <is>
+          <t>fail</t>
+        </is>
+      </c>
+      <c r="AB16" t="n">
+        <v>-0.9432738793226464</v>
+      </c>
     </row>
     <row r="17">
       <c r="A17" t="inlineStr">
@@ -1686,6 +2216,39 @@
       <c r="U17" t="b">
         <v>0</v>
       </c>
+      <c r="V17" t="inlineStr">
+        <is>
+          <t>high</t>
+        </is>
+      </c>
+      <c r="W17" t="inlineStr">
+        <is>
+          <t>pass</t>
+        </is>
+      </c>
+      <c r="X17" t="inlineStr">
+        <is>
+          <t>pass</t>
+        </is>
+      </c>
+      <c r="Y17" t="inlineStr">
+        <is>
+          <t>pass</t>
+        </is>
+      </c>
+      <c r="Z17" t="inlineStr">
+        <is>
+          <t>pass</t>
+        </is>
+      </c>
+      <c r="AA17" t="inlineStr">
+        <is>
+          <t>pass</t>
+        </is>
+      </c>
+      <c r="AB17" t="n">
+        <v>-0.7701057966378611</v>
+      </c>
     </row>
     <row r="18">
       <c r="A18" t="inlineStr">
@@ -1759,6 +2322,39 @@
       <c r="U18" t="b">
         <v>0</v>
       </c>
+      <c r="V18" t="inlineStr">
+        <is>
+          <t>medium</t>
+        </is>
+      </c>
+      <c r="W18" t="inlineStr">
+        <is>
+          <t>fail</t>
+        </is>
+      </c>
+      <c r="X18" t="inlineStr">
+        <is>
+          <t>pass</t>
+        </is>
+      </c>
+      <c r="Y18" t="inlineStr">
+        <is>
+          <t>pass</t>
+        </is>
+      </c>
+      <c r="Z18" t="inlineStr">
+        <is>
+          <t>pass</t>
+        </is>
+      </c>
+      <c r="AA18" t="inlineStr">
+        <is>
+          <t>uninformative</t>
+        </is>
+      </c>
+      <c r="AB18" t="n">
+        <v>-0.8094174294517624</v>
+      </c>
     </row>
     <row r="19">
       <c r="A19" t="inlineStr">
@@ -1832,6 +2428,39 @@
       <c r="U19" t="b">
         <v>0</v>
       </c>
+      <c r="V19" t="inlineStr">
+        <is>
+          <t>medium</t>
+        </is>
+      </c>
+      <c r="W19" t="inlineStr">
+        <is>
+          <t>fail</t>
+        </is>
+      </c>
+      <c r="X19" t="inlineStr">
+        <is>
+          <t>pass</t>
+        </is>
+      </c>
+      <c r="Y19" t="inlineStr">
+        <is>
+          <t>pass</t>
+        </is>
+      </c>
+      <c r="Z19" t="inlineStr">
+        <is>
+          <t>pass</t>
+        </is>
+      </c>
+      <c r="AA19" t="inlineStr">
+        <is>
+          <t>uninformative</t>
+        </is>
+      </c>
+      <c r="AB19" t="n">
+        <v>-0.8991478476896867</v>
+      </c>
     </row>
     <row r="20">
       <c r="A20" t="inlineStr">
@@ -1905,6 +2534,39 @@
       <c r="U20" t="b">
         <v>0</v>
       </c>
+      <c r="V20" t="inlineStr">
+        <is>
+          <t>medium</t>
+        </is>
+      </c>
+      <c r="W20" t="inlineStr">
+        <is>
+          <t>fail</t>
+        </is>
+      </c>
+      <c r="X20" t="inlineStr">
+        <is>
+          <t>pass</t>
+        </is>
+      </c>
+      <c r="Y20" t="inlineStr">
+        <is>
+          <t>pass</t>
+        </is>
+      </c>
+      <c r="Z20" t="inlineStr">
+        <is>
+          <t>pass</t>
+        </is>
+      </c>
+      <c r="AA20" t="inlineStr">
+        <is>
+          <t>uninformative</t>
+        </is>
+      </c>
+      <c r="AB20" t="n">
+        <v>-0.8633316194200893</v>
+      </c>
     </row>
     <row r="21">
       <c r="A21" t="inlineStr">
@@ -1978,6 +2640,39 @@
       <c r="U21" t="b">
         <v>0</v>
       </c>
+      <c r="V21" t="inlineStr">
+        <is>
+          <t>medium</t>
+        </is>
+      </c>
+      <c r="W21" t="inlineStr">
+        <is>
+          <t>fail</t>
+        </is>
+      </c>
+      <c r="X21" t="inlineStr">
+        <is>
+          <t>pass</t>
+        </is>
+      </c>
+      <c r="Y21" t="inlineStr">
+        <is>
+          <t>pass</t>
+        </is>
+      </c>
+      <c r="Z21" t="inlineStr">
+        <is>
+          <t>pass</t>
+        </is>
+      </c>
+      <c r="AA21" t="inlineStr">
+        <is>
+          <t>uninformative</t>
+        </is>
+      </c>
+      <c r="AB21" t="n">
+        <v>-0.850555099680339</v>
+      </c>
     </row>
     <row r="22">
       <c r="A22" t="inlineStr">
@@ -2051,6 +2746,39 @@
       <c r="U22" t="b">
         <v>0</v>
       </c>
+      <c r="V22" t="inlineStr">
+        <is>
+          <t>medium</t>
+        </is>
+      </c>
+      <c r="W22" t="inlineStr">
+        <is>
+          <t>fail</t>
+        </is>
+      </c>
+      <c r="X22" t="inlineStr">
+        <is>
+          <t>pass</t>
+        </is>
+      </c>
+      <c r="Y22" t="inlineStr">
+        <is>
+          <t>pass</t>
+        </is>
+      </c>
+      <c r="Z22" t="inlineStr">
+        <is>
+          <t>pass</t>
+        </is>
+      </c>
+      <c r="AA22" t="inlineStr">
+        <is>
+          <t>uninformative</t>
+        </is>
+      </c>
+      <c r="AB22" t="n">
+        <v>-0.8294961143416411</v>
+      </c>
     </row>
     <row r="23">
       <c r="A23" t="inlineStr">
@@ -2124,6 +2852,39 @@
       <c r="U23" t="b">
         <v>0</v>
       </c>
+      <c r="V23" t="inlineStr">
+        <is>
+          <t>medium</t>
+        </is>
+      </c>
+      <c r="W23" t="inlineStr">
+        <is>
+          <t>fail</t>
+        </is>
+      </c>
+      <c r="X23" t="inlineStr">
+        <is>
+          <t>pass</t>
+        </is>
+      </c>
+      <c r="Y23" t="inlineStr">
+        <is>
+          <t>pass</t>
+        </is>
+      </c>
+      <c r="Z23" t="inlineStr">
+        <is>
+          <t>pass</t>
+        </is>
+      </c>
+      <c r="AA23" t="inlineStr">
+        <is>
+          <t>uninformative</t>
+        </is>
+      </c>
+      <c r="AB23" t="n">
+        <v>-0.8114075168145537</v>
+      </c>
     </row>
     <row r="24">
       <c r="A24" t="inlineStr">
@@ -2193,6 +2954,39 @@
       <c r="U24" t="b">
         <v>0</v>
       </c>
+      <c r="V24" t="inlineStr">
+        <is>
+          <t>high</t>
+        </is>
+      </c>
+      <c r="W24" t="inlineStr">
+        <is>
+          <t>pass</t>
+        </is>
+      </c>
+      <c r="X24" t="inlineStr">
+        <is>
+          <t>pass</t>
+        </is>
+      </c>
+      <c r="Y24" t="inlineStr">
+        <is>
+          <t>pass</t>
+        </is>
+      </c>
+      <c r="Z24" t="inlineStr">
+        <is>
+          <t>pass</t>
+        </is>
+      </c>
+      <c r="AA24" t="inlineStr">
+        <is>
+          <t>pass</t>
+        </is>
+      </c>
+      <c r="AB24" t="n">
+        <v>-0.8205412491305067</v>
+      </c>
     </row>
     <row r="25">
       <c r="A25" t="inlineStr">
@@ -2262,6 +3056,39 @@
       <c r="U25" t="b">
         <v>0</v>
       </c>
+      <c r="V25" t="inlineStr">
+        <is>
+          <t>medium</t>
+        </is>
+      </c>
+      <c r="W25" t="inlineStr">
+        <is>
+          <t>fail</t>
+        </is>
+      </c>
+      <c r="X25" t="inlineStr">
+        <is>
+          <t>pass</t>
+        </is>
+      </c>
+      <c r="Y25" t="inlineStr">
+        <is>
+          <t>pass</t>
+        </is>
+      </c>
+      <c r="Z25" t="inlineStr">
+        <is>
+          <t>pass</t>
+        </is>
+      </c>
+      <c r="AA25" t="inlineStr">
+        <is>
+          <t>uninformative</t>
+        </is>
+      </c>
+      <c r="AB25" t="n">
+        <v>-0.8322255705482856</v>
+      </c>
     </row>
     <row r="26">
       <c r="A26" t="inlineStr">
@@ -2331,6 +3158,39 @@
       <c r="U26" t="b">
         <v>1</v>
       </c>
+      <c r="V26" t="inlineStr">
+        <is>
+          <t>low</t>
+        </is>
+      </c>
+      <c r="W26" t="inlineStr">
+        <is>
+          <t>fail</t>
+        </is>
+      </c>
+      <c r="X26" t="inlineStr">
+        <is>
+          <t>pass</t>
+        </is>
+      </c>
+      <c r="Y26" t="inlineStr">
+        <is>
+          <t>uninformative</t>
+        </is>
+      </c>
+      <c r="Z26" t="inlineStr">
+        <is>
+          <t>uninformative</t>
+        </is>
+      </c>
+      <c r="AA26" t="inlineStr">
+        <is>
+          <t>uninformative</t>
+        </is>
+      </c>
+      <c r="AB26" t="n">
+        <v>-0.8447951576685384</v>
+      </c>
     </row>
     <row r="27">
       <c r="A27" t="inlineStr">
@@ -2400,6 +3260,39 @@
       <c r="U27" t="b">
         <v>0</v>
       </c>
+      <c r="V27" t="inlineStr">
+        <is>
+          <t>medium</t>
+        </is>
+      </c>
+      <c r="W27" t="inlineStr">
+        <is>
+          <t>pass</t>
+        </is>
+      </c>
+      <c r="X27" t="inlineStr">
+        <is>
+          <t>pass</t>
+        </is>
+      </c>
+      <c r="Y27" t="inlineStr">
+        <is>
+          <t>pass</t>
+        </is>
+      </c>
+      <c r="Z27" t="inlineStr">
+        <is>
+          <t>fail</t>
+        </is>
+      </c>
+      <c r="AA27" t="inlineStr">
+        <is>
+          <t>pass</t>
+        </is>
+      </c>
+      <c r="AB27" t="n">
+        <v>-0.7995231952144938</v>
+      </c>
     </row>
     <row r="28">
       <c r="A28" t="inlineStr">
@@ -2473,6 +3366,39 @@
       <c r="U28" t="b">
         <v>0</v>
       </c>
+      <c r="V28" t="inlineStr">
+        <is>
+          <t>high</t>
+        </is>
+      </c>
+      <c r="W28" t="inlineStr">
+        <is>
+          <t>pass</t>
+        </is>
+      </c>
+      <c r="X28" t="inlineStr">
+        <is>
+          <t>pass</t>
+        </is>
+      </c>
+      <c r="Y28" t="inlineStr">
+        <is>
+          <t>pass</t>
+        </is>
+      </c>
+      <c r="Z28" t="inlineStr">
+        <is>
+          <t>pass</t>
+        </is>
+      </c>
+      <c r="AA28" t="inlineStr">
+        <is>
+          <t>pass</t>
+        </is>
+      </c>
+      <c r="AB28" t="n">
+        <v>-0.7963184334088669</v>
+      </c>
     </row>
     <row r="29">
       <c r="A29" t="inlineStr">
@@ -2542,6 +3468,39 @@
       <c r="U29" t="b">
         <v>0</v>
       </c>
+      <c r="V29" t="inlineStr">
+        <is>
+          <t>high</t>
+        </is>
+      </c>
+      <c r="W29" t="inlineStr">
+        <is>
+          <t>pass</t>
+        </is>
+      </c>
+      <c r="X29" t="inlineStr">
+        <is>
+          <t>pass</t>
+        </is>
+      </c>
+      <c r="Y29" t="inlineStr">
+        <is>
+          <t>pass</t>
+        </is>
+      </c>
+      <c r="Z29" t="inlineStr">
+        <is>
+          <t>pass</t>
+        </is>
+      </c>
+      <c r="AA29" t="inlineStr">
+        <is>
+          <t>pass</t>
+        </is>
+      </c>
+      <c r="AB29" t="n">
+        <v>-0.7864619692219967</v>
+      </c>
     </row>
     <row r="30">
       <c r="A30" t="inlineStr">
@@ -2615,6 +3574,39 @@
       <c r="U30" t="b">
         <v>0</v>
       </c>
+      <c r="V30" t="inlineStr">
+        <is>
+          <t>medium</t>
+        </is>
+      </c>
+      <c r="W30" t="inlineStr">
+        <is>
+          <t>fail</t>
+        </is>
+      </c>
+      <c r="X30" t="inlineStr">
+        <is>
+          <t>pass</t>
+        </is>
+      </c>
+      <c r="Y30" t="inlineStr">
+        <is>
+          <t>pass</t>
+        </is>
+      </c>
+      <c r="Z30" t="inlineStr">
+        <is>
+          <t>pass</t>
+        </is>
+      </c>
+      <c r="AA30" t="inlineStr">
+        <is>
+          <t>uninformative</t>
+        </is>
+      </c>
+      <c r="AB30" t="n">
+        <v>-0.824318745705738</v>
+      </c>
     </row>
     <row r="31">
       <c r="A31" t="inlineStr">
@@ -2684,6 +3676,39 @@
       <c r="U31" t="b">
         <v>0</v>
       </c>
+      <c r="V31" t="inlineStr">
+        <is>
+          <t>medium</t>
+        </is>
+      </c>
+      <c r="W31" t="inlineStr">
+        <is>
+          <t>pass</t>
+        </is>
+      </c>
+      <c r="X31" t="inlineStr">
+        <is>
+          <t>pass</t>
+        </is>
+      </c>
+      <c r="Y31" t="inlineStr">
+        <is>
+          <t>pass</t>
+        </is>
+      </c>
+      <c r="Z31" t="inlineStr">
+        <is>
+          <t>fail</t>
+        </is>
+      </c>
+      <c r="AA31" t="inlineStr">
+        <is>
+          <t>pass</t>
+        </is>
+      </c>
+      <c r="AB31" t="n">
+        <v>-0.77309606094219</v>
+      </c>
     </row>
     <row r="32">
       <c r="A32" t="inlineStr">
@@ -2757,6 +3782,39 @@
       <c r="U32" t="b">
         <v>0</v>
       </c>
+      <c r="V32" t="inlineStr">
+        <is>
+          <t>high</t>
+        </is>
+      </c>
+      <c r="W32" t="inlineStr">
+        <is>
+          <t>pass</t>
+        </is>
+      </c>
+      <c r="X32" t="inlineStr">
+        <is>
+          <t>pass</t>
+        </is>
+      </c>
+      <c r="Y32" t="inlineStr">
+        <is>
+          <t>pass</t>
+        </is>
+      </c>
+      <c r="Z32" t="inlineStr">
+        <is>
+          <t>pass</t>
+        </is>
+      </c>
+      <c r="AA32" t="inlineStr">
+        <is>
+          <t>uninformative</t>
+        </is>
+      </c>
+      <c r="AB32" t="n">
+        <v>-0.6381595903457972</v>
+      </c>
     </row>
     <row r="33">
       <c r="A33" t="inlineStr">
@@ -2826,6 +3884,39 @@
       <c r="U33" t="b">
         <v>0</v>
       </c>
+      <c r="V33" t="inlineStr">
+        <is>
+          <t>high</t>
+        </is>
+      </c>
+      <c r="W33" t="inlineStr">
+        <is>
+          <t>pass</t>
+        </is>
+      </c>
+      <c r="X33" t="inlineStr">
+        <is>
+          <t>pass</t>
+        </is>
+      </c>
+      <c r="Y33" t="inlineStr">
+        <is>
+          <t>pass</t>
+        </is>
+      </c>
+      <c r="Z33" t="inlineStr">
+        <is>
+          <t>pass</t>
+        </is>
+      </c>
+      <c r="AA33" t="inlineStr">
+        <is>
+          <t>pass</t>
+        </is>
+      </c>
+      <c r="AB33" t="n">
+        <v>-0.7761335756286625</v>
+      </c>
     </row>
     <row r="34">
       <c r="A34" t="inlineStr">
@@ -2895,6 +3986,39 @@
       <c r="U34" t="b">
         <v>0</v>
       </c>
+      <c r="V34" t="inlineStr">
+        <is>
+          <t>medium</t>
+        </is>
+      </c>
+      <c r="W34" t="inlineStr">
+        <is>
+          <t>pass</t>
+        </is>
+      </c>
+      <c r="X34" t="inlineStr">
+        <is>
+          <t>pass</t>
+        </is>
+      </c>
+      <c r="Y34" t="inlineStr">
+        <is>
+          <t>pass</t>
+        </is>
+      </c>
+      <c r="Z34" t="inlineStr">
+        <is>
+          <t>fail</t>
+        </is>
+      </c>
+      <c r="AA34" t="inlineStr">
+        <is>
+          <t>uninformative</t>
+        </is>
+      </c>
+      <c r="AB34" t="n">
+        <v>-0.7640925562537549</v>
+      </c>
     </row>
     <row r="35">
       <c r="A35" t="inlineStr">
@@ -2964,6 +4088,39 @@
       <c r="U35" t="b">
         <v>0</v>
       </c>
+      <c r="V35" t="inlineStr">
+        <is>
+          <t>high</t>
+        </is>
+      </c>
+      <c r="W35" t="inlineStr">
+        <is>
+          <t>pass</t>
+        </is>
+      </c>
+      <c r="X35" t="inlineStr">
+        <is>
+          <t>pass</t>
+        </is>
+      </c>
+      <c r="Y35" t="inlineStr">
+        <is>
+          <t>pass</t>
+        </is>
+      </c>
+      <c r="Z35" t="inlineStr">
+        <is>
+          <t>pass</t>
+        </is>
+      </c>
+      <c r="AA35" t="inlineStr">
+        <is>
+          <t>pass</t>
+        </is>
+      </c>
+      <c r="AB35" t="n">
+        <v>-0.7585993381851116</v>
+      </c>
     </row>
     <row r="36">
       <c r="A36" t="inlineStr">
@@ -3033,6 +4190,39 @@
       <c r="U36" t="b">
         <v>0</v>
       </c>
+      <c r="V36" t="inlineStr">
+        <is>
+          <t>high</t>
+        </is>
+      </c>
+      <c r="W36" t="inlineStr">
+        <is>
+          <t>pass</t>
+        </is>
+      </c>
+      <c r="X36" t="inlineStr">
+        <is>
+          <t>pass</t>
+        </is>
+      </c>
+      <c r="Y36" t="inlineStr">
+        <is>
+          <t>pass</t>
+        </is>
+      </c>
+      <c r="Z36" t="inlineStr">
+        <is>
+          <t>pass</t>
+        </is>
+      </c>
+      <c r="AA36" t="inlineStr">
+        <is>
+          <t>uninformative</t>
+        </is>
+      </c>
+      <c r="AB36" t="n">
+        <v>-0.8011424948958573</v>
+      </c>
     </row>
     <row r="37">
       <c r="A37" t="inlineStr">
@@ -3106,6 +4296,39 @@
       <c r="U37" t="b">
         <v>0</v>
       </c>
+      <c r="V37" t="inlineStr">
+        <is>
+          <t>medium</t>
+        </is>
+      </c>
+      <c r="W37" t="inlineStr">
+        <is>
+          <t>fail</t>
+        </is>
+      </c>
+      <c r="X37" t="inlineStr">
+        <is>
+          <t>pass</t>
+        </is>
+      </c>
+      <c r="Y37" t="inlineStr">
+        <is>
+          <t>pass</t>
+        </is>
+      </c>
+      <c r="Z37" t="inlineStr">
+        <is>
+          <t>pass</t>
+        </is>
+      </c>
+      <c r="AA37" t="inlineStr">
+        <is>
+          <t>uninformative</t>
+        </is>
+      </c>
+      <c r="AB37" t="n">
+        <v>-0.5607301556030795</v>
+      </c>
     </row>
     <row r="38">
       <c r="A38" t="inlineStr">
@@ -3175,6 +4398,39 @@
       <c r="U38" t="b">
         <v>1</v>
       </c>
+      <c r="V38" t="inlineStr">
+        <is>
+          <t>low</t>
+        </is>
+      </c>
+      <c r="W38" t="inlineStr">
+        <is>
+          <t>fail</t>
+        </is>
+      </c>
+      <c r="X38" t="inlineStr">
+        <is>
+          <t>pass</t>
+        </is>
+      </c>
+      <c r="Y38" t="inlineStr">
+        <is>
+          <t>pass</t>
+        </is>
+      </c>
+      <c r="Z38" t="inlineStr">
+        <is>
+          <t>uninformative</t>
+        </is>
+      </c>
+      <c r="AA38" t="inlineStr">
+        <is>
+          <t>uninformative</t>
+        </is>
+      </c>
+      <c r="AB38" t="n">
+        <v>-0.7254931543108373</v>
+      </c>
     </row>
     <row r="39">
       <c r="A39" t="inlineStr">
@@ -3244,6 +4500,39 @@
       <c r="U39" t="b">
         <v>0</v>
       </c>
+      <c r="V39" t="inlineStr">
+        <is>
+          <t>medium</t>
+        </is>
+      </c>
+      <c r="W39" t="inlineStr">
+        <is>
+          <t>pass</t>
+        </is>
+      </c>
+      <c r="X39" t="inlineStr">
+        <is>
+          <t>pass</t>
+        </is>
+      </c>
+      <c r="Y39" t="inlineStr">
+        <is>
+          <t>pass</t>
+        </is>
+      </c>
+      <c r="Z39" t="inlineStr">
+        <is>
+          <t>fail</t>
+        </is>
+      </c>
+      <c r="AA39" t="inlineStr">
+        <is>
+          <t>pass</t>
+        </is>
+      </c>
+      <c r="AB39" t="n">
+        <v>-0.7505522707815774</v>
+      </c>
     </row>
     <row r="40">
       <c r="A40" t="inlineStr">
@@ -3313,6 +4602,39 @@
       <c r="U40" t="b">
         <v>0</v>
       </c>
+      <c r="V40" t="inlineStr">
+        <is>
+          <t>medium</t>
+        </is>
+      </c>
+      <c r="W40" t="inlineStr">
+        <is>
+          <t>pass</t>
+        </is>
+      </c>
+      <c r="X40" t="inlineStr">
+        <is>
+          <t>pass</t>
+        </is>
+      </c>
+      <c r="Y40" t="inlineStr">
+        <is>
+          <t>pass</t>
+        </is>
+      </c>
+      <c r="Z40" t="inlineStr">
+        <is>
+          <t>pass</t>
+        </is>
+      </c>
+      <c r="AA40" t="inlineStr">
+        <is>
+          <t>fail</t>
+        </is>
+      </c>
+      <c r="AB40" t="n">
+        <v>-0.7263489324389152</v>
+      </c>
     </row>
     <row r="41">
       <c r="A41" t="inlineStr">
@@ -3386,6 +4708,39 @@
       <c r="U41" t="b">
         <v>0</v>
       </c>
+      <c r="V41" t="inlineStr">
+        <is>
+          <t>medium</t>
+        </is>
+      </c>
+      <c r="W41" t="inlineStr">
+        <is>
+          <t>fail</t>
+        </is>
+      </c>
+      <c r="X41" t="inlineStr">
+        <is>
+          <t>pass</t>
+        </is>
+      </c>
+      <c r="Y41" t="inlineStr">
+        <is>
+          <t>pass</t>
+        </is>
+      </c>
+      <c r="Z41" t="inlineStr">
+        <is>
+          <t>pass</t>
+        </is>
+      </c>
+      <c r="AA41" t="inlineStr">
+        <is>
+          <t>pass</t>
+        </is>
+      </c>
+      <c r="AB41" t="n">
+        <v>-0.6907123574774108</v>
+      </c>
     </row>
     <row r="42">
       <c r="A42" t="inlineStr">
@@ -3459,6 +4814,39 @@
       <c r="U42" t="b">
         <v>0</v>
       </c>
+      <c r="V42" t="inlineStr">
+        <is>
+          <t>high</t>
+        </is>
+      </c>
+      <c r="W42" t="inlineStr">
+        <is>
+          <t>pass</t>
+        </is>
+      </c>
+      <c r="X42" t="inlineStr">
+        <is>
+          <t>pass</t>
+        </is>
+      </c>
+      <c r="Y42" t="inlineStr">
+        <is>
+          <t>pass</t>
+        </is>
+      </c>
+      <c r="Z42" t="inlineStr">
+        <is>
+          <t>pass</t>
+        </is>
+      </c>
+      <c r="AA42" t="inlineStr">
+        <is>
+          <t>pass</t>
+        </is>
+      </c>
+      <c r="AB42" t="n">
+        <v>-0.7068140094748493</v>
+      </c>
     </row>
     <row r="43">
       <c r="A43" t="inlineStr">
@@ -3532,6 +4920,39 @@
       <c r="U43" t="b">
         <v>0</v>
       </c>
+      <c r="V43" t="inlineStr">
+        <is>
+          <t>low</t>
+        </is>
+      </c>
+      <c r="W43" t="inlineStr">
+        <is>
+          <t>fail</t>
+        </is>
+      </c>
+      <c r="X43" t="inlineStr">
+        <is>
+          <t>fail</t>
+        </is>
+      </c>
+      <c r="Y43" t="inlineStr">
+        <is>
+          <t>fail</t>
+        </is>
+      </c>
+      <c r="Z43" t="inlineStr">
+        <is>
+          <t>pass</t>
+        </is>
+      </c>
+      <c r="AA43" t="inlineStr">
+        <is>
+          <t>uninformative</t>
+        </is>
+      </c>
+      <c r="AB43" t="n">
+        <v>-0.694880903531901</v>
+      </c>
     </row>
     <row r="44">
       <c r="A44" t="inlineStr">
@@ -3601,6 +5022,39 @@
       <c r="U44" t="b">
         <v>0</v>
       </c>
+      <c r="V44" t="inlineStr">
+        <is>
+          <t>medium</t>
+        </is>
+      </c>
+      <c r="W44" t="inlineStr">
+        <is>
+          <t>pass</t>
+        </is>
+      </c>
+      <c r="X44" t="inlineStr">
+        <is>
+          <t>pass</t>
+        </is>
+      </c>
+      <c r="Y44" t="inlineStr">
+        <is>
+          <t>pass</t>
+        </is>
+      </c>
+      <c r="Z44" t="inlineStr">
+        <is>
+          <t>fail</t>
+        </is>
+      </c>
+      <c r="AA44" t="inlineStr">
+        <is>
+          <t>pass</t>
+        </is>
+      </c>
+      <c r="AB44" t="n">
+        <v>-0.7400333291868505</v>
+      </c>
     </row>
     <row r="45">
       <c r="A45" t="inlineStr">
@@ -3674,6 +5128,39 @@
       <c r="U45" t="b">
         <v>0</v>
       </c>
+      <c r="V45" t="inlineStr">
+        <is>
+          <t>medium</t>
+        </is>
+      </c>
+      <c r="W45" t="inlineStr">
+        <is>
+          <t>fail</t>
+        </is>
+      </c>
+      <c r="X45" t="inlineStr">
+        <is>
+          <t>pass</t>
+        </is>
+      </c>
+      <c r="Y45" t="inlineStr">
+        <is>
+          <t>pass</t>
+        </is>
+      </c>
+      <c r="Z45" t="inlineStr">
+        <is>
+          <t>pass</t>
+        </is>
+      </c>
+      <c r="AA45" t="inlineStr">
+        <is>
+          <t>uninformative</t>
+        </is>
+      </c>
+      <c r="AB45" t="n">
+        <v>-0.7014886620371761</v>
+      </c>
     </row>
     <row r="46">
       <c r="A46" t="inlineStr">
@@ -3747,6 +5234,39 @@
       <c r="U46" t="b">
         <v>0</v>
       </c>
+      <c r="V46" t="inlineStr">
+        <is>
+          <t>medium</t>
+        </is>
+      </c>
+      <c r="W46" t="inlineStr">
+        <is>
+          <t>fail</t>
+        </is>
+      </c>
+      <c r="X46" t="inlineStr">
+        <is>
+          <t>pass</t>
+        </is>
+      </c>
+      <c r="Y46" t="inlineStr">
+        <is>
+          <t>pass</t>
+        </is>
+      </c>
+      <c r="Z46" t="inlineStr">
+        <is>
+          <t>pass</t>
+        </is>
+      </c>
+      <c r="AA46" t="inlineStr">
+        <is>
+          <t>pass</t>
+        </is>
+      </c>
+      <c r="AB46" t="n">
+        <v>-0.7082557415859232</v>
+      </c>
     </row>
     <row r="47">
       <c r="A47" t="inlineStr">
@@ -3816,6 +5336,39 @@
       <c r="U47" t="b">
         <v>1</v>
       </c>
+      <c r="V47" t="inlineStr">
+        <is>
+          <t>low</t>
+        </is>
+      </c>
+      <c r="W47" t="inlineStr">
+        <is>
+          <t>fail</t>
+        </is>
+      </c>
+      <c r="X47" t="inlineStr">
+        <is>
+          <t>pass</t>
+        </is>
+      </c>
+      <c r="Y47" t="inlineStr">
+        <is>
+          <t>fail</t>
+        </is>
+      </c>
+      <c r="Z47" t="inlineStr">
+        <is>
+          <t>uninformative</t>
+        </is>
+      </c>
+      <c r="AA47" t="inlineStr">
+        <is>
+          <t>uninformative</t>
+        </is>
+      </c>
+      <c r="AB47" t="n">
+        <v>-0.6854512593382545</v>
+      </c>
     </row>
     <row r="48">
       <c r="A48" t="inlineStr">
@@ -3889,6 +5442,39 @@
       <c r="U48" t="b">
         <v>0</v>
       </c>
+      <c r="V48" t="inlineStr">
+        <is>
+          <t>low</t>
+        </is>
+      </c>
+      <c r="W48" t="inlineStr">
+        <is>
+          <t>fail</t>
+        </is>
+      </c>
+      <c r="X48" t="inlineStr">
+        <is>
+          <t>pass</t>
+        </is>
+      </c>
+      <c r="Y48" t="inlineStr">
+        <is>
+          <t>pass</t>
+        </is>
+      </c>
+      <c r="Z48" t="inlineStr">
+        <is>
+          <t>pass</t>
+        </is>
+      </c>
+      <c r="AA48" t="inlineStr">
+        <is>
+          <t>fail</t>
+        </is>
+      </c>
+      <c r="AB48" t="n">
+        <v>-0.7046353497966003</v>
+      </c>
     </row>
     <row r="49">
       <c r="A49" t="inlineStr">
@@ -3958,6 +5544,39 @@
       <c r="U49" t="b">
         <v>0</v>
       </c>
+      <c r="V49" t="inlineStr">
+        <is>
+          <t>medium</t>
+        </is>
+      </c>
+      <c r="W49" t="inlineStr">
+        <is>
+          <t>pass</t>
+        </is>
+      </c>
+      <c r="X49" t="inlineStr">
+        <is>
+          <t>pass</t>
+        </is>
+      </c>
+      <c r="Y49" t="inlineStr">
+        <is>
+          <t>pass</t>
+        </is>
+      </c>
+      <c r="Z49" t="inlineStr">
+        <is>
+          <t>fail</t>
+        </is>
+      </c>
+      <c r="AA49" t="inlineStr">
+        <is>
+          <t>pass</t>
+        </is>
+      </c>
+      <c r="AB49" t="n">
+        <v>-0.6833950316113085</v>
+      </c>
     </row>
     <row r="50">
       <c r="A50" t="inlineStr">
@@ -4027,6 +5646,39 @@
       <c r="U50" t="b">
         <v>0</v>
       </c>
+      <c r="V50" t="inlineStr">
+        <is>
+          <t>medium</t>
+        </is>
+      </c>
+      <c r="W50" t="inlineStr">
+        <is>
+          <t>pass</t>
+        </is>
+      </c>
+      <c r="X50" t="inlineStr">
+        <is>
+          <t>pass</t>
+        </is>
+      </c>
+      <c r="Y50" t="inlineStr">
+        <is>
+          <t>pass</t>
+        </is>
+      </c>
+      <c r="Z50" t="inlineStr">
+        <is>
+          <t>fail</t>
+        </is>
+      </c>
+      <c r="AA50" t="inlineStr">
+        <is>
+          <t>pass</t>
+        </is>
+      </c>
+      <c r="AB50" t="n">
+        <v>-0.6861349236785185</v>
+      </c>
     </row>
     <row r="51">
       <c r="A51" t="inlineStr">
@@ -4096,6 +5748,39 @@
       <c r="U51" t="b">
         <v>0</v>
       </c>
+      <c r="V51" t="inlineStr">
+        <is>
+          <t>medium</t>
+        </is>
+      </c>
+      <c r="W51" t="inlineStr">
+        <is>
+          <t>fail</t>
+        </is>
+      </c>
+      <c r="X51" t="inlineStr">
+        <is>
+          <t>pass</t>
+        </is>
+      </c>
+      <c r="Y51" t="inlineStr">
+        <is>
+          <t>pass</t>
+        </is>
+      </c>
+      <c r="Z51" t="inlineStr">
+        <is>
+          <t>pass</t>
+        </is>
+      </c>
+      <c r="AA51" t="inlineStr">
+        <is>
+          <t>uninformative</t>
+        </is>
+      </c>
+      <c r="AB51" t="n">
+        <v>-0.6799546558213418</v>
+      </c>
     </row>
     <row r="52">
       <c r="A52" t="inlineStr">
@@ -4169,6 +5854,39 @@
       <c r="U52" t="b">
         <v>0</v>
       </c>
+      <c r="V52" t="inlineStr">
+        <is>
+          <t>medium</t>
+        </is>
+      </c>
+      <c r="W52" t="inlineStr">
+        <is>
+          <t>fail</t>
+        </is>
+      </c>
+      <c r="X52" t="inlineStr">
+        <is>
+          <t>pass</t>
+        </is>
+      </c>
+      <c r="Y52" t="inlineStr">
+        <is>
+          <t>pass</t>
+        </is>
+      </c>
+      <c r="Z52" t="inlineStr">
+        <is>
+          <t>pass</t>
+        </is>
+      </c>
+      <c r="AA52" t="inlineStr">
+        <is>
+          <t>uninformative</t>
+        </is>
+      </c>
+      <c r="AB52" t="n">
+        <v>-0.5460604599363266</v>
+      </c>
     </row>
     <row r="53">
       <c r="A53" t="inlineStr">
@@ -4238,6 +5956,39 @@
       <c r="U53" t="b">
         <v>0</v>
       </c>
+      <c r="V53" t="inlineStr">
+        <is>
+          <t>medium</t>
+        </is>
+      </c>
+      <c r="W53" t="inlineStr">
+        <is>
+          <t>fail</t>
+        </is>
+      </c>
+      <c r="X53" t="inlineStr">
+        <is>
+          <t>pass</t>
+        </is>
+      </c>
+      <c r="Y53" t="inlineStr">
+        <is>
+          <t>pass</t>
+        </is>
+      </c>
+      <c r="Z53" t="inlineStr">
+        <is>
+          <t>pass</t>
+        </is>
+      </c>
+      <c r="AA53" t="inlineStr">
+        <is>
+          <t>pass</t>
+        </is>
+      </c>
+      <c r="AB53" t="n">
+        <v>-0.6639348892766579</v>
+      </c>
     </row>
     <row r="54">
       <c r="A54" t="inlineStr">
@@ -4311,6 +6062,39 @@
       <c r="U54" t="b">
         <v>0</v>
       </c>
+      <c r="V54" t="inlineStr">
+        <is>
+          <t>medium</t>
+        </is>
+      </c>
+      <c r="W54" t="inlineStr">
+        <is>
+          <t>fail</t>
+        </is>
+      </c>
+      <c r="X54" t="inlineStr">
+        <is>
+          <t>pass</t>
+        </is>
+      </c>
+      <c r="Y54" t="inlineStr">
+        <is>
+          <t>pass</t>
+        </is>
+      </c>
+      <c r="Z54" t="inlineStr">
+        <is>
+          <t>pass</t>
+        </is>
+      </c>
+      <c r="AA54" t="inlineStr">
+        <is>
+          <t>uninformative</t>
+        </is>
+      </c>
+      <c r="AB54" t="n">
+        <v>-0.5694626283458697</v>
+      </c>
     </row>
     <row r="55">
       <c r="A55" t="inlineStr">
@@ -4380,6 +6164,39 @@
       <c r="U55" t="b">
         <v>0</v>
       </c>
+      <c r="V55" t="inlineStr">
+        <is>
+          <t>medium</t>
+        </is>
+      </c>
+      <c r="W55" t="inlineStr">
+        <is>
+          <t>fail</t>
+        </is>
+      </c>
+      <c r="X55" t="inlineStr">
+        <is>
+          <t>pass</t>
+        </is>
+      </c>
+      <c r="Y55" t="inlineStr">
+        <is>
+          <t>pass</t>
+        </is>
+      </c>
+      <c r="Z55" t="inlineStr">
+        <is>
+          <t>pass</t>
+        </is>
+      </c>
+      <c r="AA55" t="inlineStr">
+        <is>
+          <t>pass</t>
+        </is>
+      </c>
+      <c r="AB55" t="n">
+        <v>-0.6653824731851539</v>
+      </c>
     </row>
     <row r="56">
       <c r="A56" t="inlineStr">
@@ -4449,6 +6266,39 @@
       <c r="U56" t="b">
         <v>0</v>
       </c>
+      <c r="V56" t="inlineStr">
+        <is>
+          <t>medium</t>
+        </is>
+      </c>
+      <c r="W56" t="inlineStr">
+        <is>
+          <t>fail</t>
+        </is>
+      </c>
+      <c r="X56" t="inlineStr">
+        <is>
+          <t>pass</t>
+        </is>
+      </c>
+      <c r="Y56" t="inlineStr">
+        <is>
+          <t>pass</t>
+        </is>
+      </c>
+      <c r="Z56" t="inlineStr">
+        <is>
+          <t>pass</t>
+        </is>
+      </c>
+      <c r="AA56" t="inlineStr">
+        <is>
+          <t>uninformative</t>
+        </is>
+      </c>
+      <c r="AB56" t="n">
+        <v>-0.6910034810579329</v>
+      </c>
     </row>
     <row r="57">
       <c r="A57" t="inlineStr">
@@ -4522,6 +6372,39 @@
       <c r="U57" t="b">
         <v>0</v>
       </c>
+      <c r="V57" t="inlineStr">
+        <is>
+          <t>low</t>
+        </is>
+      </c>
+      <c r="W57" t="inlineStr">
+        <is>
+          <t>fail</t>
+        </is>
+      </c>
+      <c r="X57" t="inlineStr">
+        <is>
+          <t>pass</t>
+        </is>
+      </c>
+      <c r="Y57" t="inlineStr">
+        <is>
+          <t>pass</t>
+        </is>
+      </c>
+      <c r="Z57" t="inlineStr">
+        <is>
+          <t>pass</t>
+        </is>
+      </c>
+      <c r="AA57" t="inlineStr">
+        <is>
+          <t>fail</t>
+        </is>
+      </c>
+      <c r="AB57" t="n">
+        <v>-0.6427048572454059</v>
+      </c>
     </row>
     <row r="58">
       <c r="A58" t="inlineStr">
@@ -4591,6 +6474,39 @@
       <c r="U58" t="b">
         <v>0</v>
       </c>
+      <c r="V58" t="inlineStr">
+        <is>
+          <t>medium</t>
+        </is>
+      </c>
+      <c r="W58" t="inlineStr">
+        <is>
+          <t>fail</t>
+        </is>
+      </c>
+      <c r="X58" t="inlineStr">
+        <is>
+          <t>pass</t>
+        </is>
+      </c>
+      <c r="Y58" t="inlineStr">
+        <is>
+          <t>pass</t>
+        </is>
+      </c>
+      <c r="Z58" t="inlineStr">
+        <is>
+          <t>pass</t>
+        </is>
+      </c>
+      <c r="AA58" t="inlineStr">
+        <is>
+          <t>pass</t>
+        </is>
+      </c>
+      <c r="AB58" t="n">
+        <v>-0.6479688896188045</v>
+      </c>
     </row>
     <row r="59">
       <c r="A59" t="inlineStr">
@@ -4660,6 +6576,39 @@
       <c r="U59" t="b">
         <v>0</v>
       </c>
+      <c r="V59" t="inlineStr">
+        <is>
+          <t>high</t>
+        </is>
+      </c>
+      <c r="W59" t="inlineStr">
+        <is>
+          <t>pass</t>
+        </is>
+      </c>
+      <c r="X59" t="inlineStr">
+        <is>
+          <t>pass</t>
+        </is>
+      </c>
+      <c r="Y59" t="inlineStr">
+        <is>
+          <t>pass</t>
+        </is>
+      </c>
+      <c r="Z59" t="inlineStr">
+        <is>
+          <t>pass</t>
+        </is>
+      </c>
+      <c r="AA59" t="inlineStr">
+        <is>
+          <t>pass</t>
+        </is>
+      </c>
+      <c r="AB59" t="n">
+        <v>-0.6443710497089925</v>
+      </c>
     </row>
     <row r="60">
       <c r="A60" t="inlineStr">
@@ -4733,6 +6682,39 @@
       <c r="U60" t="b">
         <v>0</v>
       </c>
+      <c r="V60" t="inlineStr">
+        <is>
+          <t>low</t>
+        </is>
+      </c>
+      <c r="W60" t="inlineStr">
+        <is>
+          <t>fail</t>
+        </is>
+      </c>
+      <c r="X60" t="inlineStr">
+        <is>
+          <t>pass</t>
+        </is>
+      </c>
+      <c r="Y60" t="inlineStr">
+        <is>
+          <t>pass</t>
+        </is>
+      </c>
+      <c r="Z60" t="inlineStr">
+        <is>
+          <t>pass</t>
+        </is>
+      </c>
+      <c r="AA60" t="inlineStr">
+        <is>
+          <t>fail</t>
+        </is>
+      </c>
+      <c r="AB60" t="n">
+        <v>-0.5119122545697911</v>
+      </c>
     </row>
     <row r="61">
       <c r="A61" t="inlineStr">
@@ -4802,6 +6784,39 @@
       <c r="U61" t="b">
         <v>0</v>
       </c>
+      <c r="V61" t="inlineStr">
+        <is>
+          <t>medium</t>
+        </is>
+      </c>
+      <c r="W61" t="inlineStr">
+        <is>
+          <t>fail</t>
+        </is>
+      </c>
+      <c r="X61" t="inlineStr">
+        <is>
+          <t>pass</t>
+        </is>
+      </c>
+      <c r="Y61" t="inlineStr">
+        <is>
+          <t>pass</t>
+        </is>
+      </c>
+      <c r="Z61" t="inlineStr">
+        <is>
+          <t>pass</t>
+        </is>
+      </c>
+      <c r="AA61" t="inlineStr">
+        <is>
+          <t>uninformative</t>
+        </is>
+      </c>
+      <c r="AB61" t="n">
+        <v>-0.6833663820876426</v>
+      </c>
     </row>
     <row r="62">
       <c r="A62" t="inlineStr">
@@ -4875,6 +6890,39 @@
       <c r="U62" t="b">
         <v>0</v>
       </c>
+      <c r="V62" t="inlineStr">
+        <is>
+          <t>low</t>
+        </is>
+      </c>
+      <c r="W62" t="inlineStr">
+        <is>
+          <t>fail</t>
+        </is>
+      </c>
+      <c r="X62" t="inlineStr">
+        <is>
+          <t>fail</t>
+        </is>
+      </c>
+      <c r="Y62" t="inlineStr">
+        <is>
+          <t>fail</t>
+        </is>
+      </c>
+      <c r="Z62" t="inlineStr">
+        <is>
+          <t>pass</t>
+        </is>
+      </c>
+      <c r="AA62" t="inlineStr">
+        <is>
+          <t>uninformative</t>
+        </is>
+      </c>
+      <c r="AB62" t="n">
+        <v>-0.6412427632410758</v>
+      </c>
     </row>
     <row r="63">
       <c r="A63" t="inlineStr">
@@ -4944,6 +6992,39 @@
       <c r="U63" t="b">
         <v>0</v>
       </c>
+      <c r="V63" t="inlineStr">
+        <is>
+          <t>low</t>
+        </is>
+      </c>
+      <c r="W63" t="inlineStr">
+        <is>
+          <t>fail</t>
+        </is>
+      </c>
+      <c r="X63" t="inlineStr">
+        <is>
+          <t>pass</t>
+        </is>
+      </c>
+      <c r="Y63" t="inlineStr">
+        <is>
+          <t>pass</t>
+        </is>
+      </c>
+      <c r="Z63" t="inlineStr">
+        <is>
+          <t>fail</t>
+        </is>
+      </c>
+      <c r="AA63" t="inlineStr">
+        <is>
+          <t>uninformative</t>
+        </is>
+      </c>
+      <c r="AB63" t="n">
+        <v>-0.644898374506631</v>
+      </c>
     </row>
     <row r="64">
       <c r="A64" t="inlineStr">
@@ -5017,6 +7098,39 @@
       <c r="U64" t="b">
         <v>0</v>
       </c>
+      <c r="V64" t="inlineStr">
+        <is>
+          <t>low</t>
+        </is>
+      </c>
+      <c r="W64" t="inlineStr">
+        <is>
+          <t>fail</t>
+        </is>
+      </c>
+      <c r="X64" t="inlineStr">
+        <is>
+          <t>pass</t>
+        </is>
+      </c>
+      <c r="Y64" t="inlineStr">
+        <is>
+          <t>pass</t>
+        </is>
+      </c>
+      <c r="Z64" t="inlineStr">
+        <is>
+          <t>fail</t>
+        </is>
+      </c>
+      <c r="AA64" t="inlineStr">
+        <is>
+          <t>uninformative</t>
+        </is>
+      </c>
+      <c r="AB64" t="n">
+        <v>-0.486816425253434</v>
+      </c>
     </row>
     <row r="65">
       <c r="A65" t="inlineStr">
@@ -5090,6 +7204,39 @@
       <c r="U65" t="b">
         <v>0</v>
       </c>
+      <c r="V65" t="inlineStr">
+        <is>
+          <t>medium</t>
+        </is>
+      </c>
+      <c r="W65" t="inlineStr">
+        <is>
+          <t>fail</t>
+        </is>
+      </c>
+      <c r="X65" t="inlineStr">
+        <is>
+          <t>pass</t>
+        </is>
+      </c>
+      <c r="Y65" t="inlineStr">
+        <is>
+          <t>pass</t>
+        </is>
+      </c>
+      <c r="Z65" t="inlineStr">
+        <is>
+          <t>pass</t>
+        </is>
+      </c>
+      <c r="AA65" t="inlineStr">
+        <is>
+          <t>uninformative</t>
+        </is>
+      </c>
+      <c r="AB65" t="n">
+        <v>-0.55992627118602</v>
+      </c>
     </row>
     <row r="66">
       <c r="A66" t="inlineStr">
@@ -5163,6 +7310,39 @@
       <c r="U66" t="b">
         <v>0</v>
       </c>
+      <c r="V66" t="inlineStr">
+        <is>
+          <t>low</t>
+        </is>
+      </c>
+      <c r="W66" t="inlineStr">
+        <is>
+          <t>fail</t>
+        </is>
+      </c>
+      <c r="X66" t="inlineStr">
+        <is>
+          <t>pass</t>
+        </is>
+      </c>
+      <c r="Y66" t="inlineStr">
+        <is>
+          <t>pass</t>
+        </is>
+      </c>
+      <c r="Z66" t="inlineStr">
+        <is>
+          <t>fail</t>
+        </is>
+      </c>
+      <c r="AA66" t="inlineStr">
+        <is>
+          <t>fail</t>
+        </is>
+      </c>
+      <c r="AB66" t="n">
+        <v>-0.4266221884265064</v>
+      </c>
     </row>
     <row r="67">
       <c r="A67" t="inlineStr">
@@ -5232,6 +7412,39 @@
       <c r="U67" t="b">
         <v>0</v>
       </c>
+      <c r="V67" t="inlineStr">
+        <is>
+          <t>medium</t>
+        </is>
+      </c>
+      <c r="W67" t="inlineStr">
+        <is>
+          <t>fail</t>
+        </is>
+      </c>
+      <c r="X67" t="inlineStr">
+        <is>
+          <t>pass</t>
+        </is>
+      </c>
+      <c r="Y67" t="inlineStr">
+        <is>
+          <t>pass</t>
+        </is>
+      </c>
+      <c r="Z67" t="inlineStr">
+        <is>
+          <t>pass</t>
+        </is>
+      </c>
+      <c r="AA67" t="inlineStr">
+        <is>
+          <t>pass</t>
+        </is>
+      </c>
+      <c r="AB67" t="n">
+        <v>-0.5992384677954098</v>
+      </c>
     </row>
     <row r="68">
       <c r="A68" t="inlineStr">
@@ -5305,6 +7518,39 @@
       <c r="U68" t="b">
         <v>0</v>
       </c>
+      <c r="V68" t="inlineStr">
+        <is>
+          <t>low</t>
+        </is>
+      </c>
+      <c r="W68" t="inlineStr">
+        <is>
+          <t>fail</t>
+        </is>
+      </c>
+      <c r="X68" t="inlineStr">
+        <is>
+          <t>pass</t>
+        </is>
+      </c>
+      <c r="Y68" t="inlineStr">
+        <is>
+          <t>pass</t>
+        </is>
+      </c>
+      <c r="Z68" t="inlineStr">
+        <is>
+          <t>pass</t>
+        </is>
+      </c>
+      <c r="AA68" t="inlineStr">
+        <is>
+          <t>fail</t>
+        </is>
+      </c>
+      <c r="AB68" t="n">
+        <v>-0.5018031372424157</v>
+      </c>
     </row>
     <row r="69">
       <c r="A69" t="inlineStr">
@@ -5374,6 +7620,39 @@
       <c r="U69" t="b">
         <v>0</v>
       </c>
+      <c r="V69" t="inlineStr">
+        <is>
+          <t>low</t>
+        </is>
+      </c>
+      <c r="W69" t="inlineStr">
+        <is>
+          <t>fail</t>
+        </is>
+      </c>
+      <c r="X69" t="inlineStr">
+        <is>
+          <t>fail</t>
+        </is>
+      </c>
+      <c r="Y69" t="inlineStr">
+        <is>
+          <t>pass</t>
+        </is>
+      </c>
+      <c r="Z69" t="inlineStr">
+        <is>
+          <t>fail</t>
+        </is>
+      </c>
+      <c r="AA69" t="inlineStr">
+        <is>
+          <t>uninformative</t>
+        </is>
+      </c>
+      <c r="AB69" t="n">
+        <v>-0.6271927275497802</v>
+      </c>
     </row>
     <row r="70">
       <c r="A70" t="inlineStr">
@@ -5443,6 +7722,39 @@
       <c r="U70" t="b">
         <v>0</v>
       </c>
+      <c r="V70" t="inlineStr">
+        <is>
+          <t>medium</t>
+        </is>
+      </c>
+      <c r="W70" t="inlineStr">
+        <is>
+          <t>fail</t>
+        </is>
+      </c>
+      <c r="X70" t="inlineStr">
+        <is>
+          <t>pass</t>
+        </is>
+      </c>
+      <c r="Y70" t="inlineStr">
+        <is>
+          <t>pass</t>
+        </is>
+      </c>
+      <c r="Z70" t="inlineStr">
+        <is>
+          <t>pass</t>
+        </is>
+      </c>
+      <c r="AA70" t="inlineStr">
+        <is>
+          <t>uninformative</t>
+        </is>
+      </c>
+      <c r="AB70" t="n">
+        <v>-0.5898868424969386</v>
+      </c>
     </row>
     <row r="71">
       <c r="A71" t="inlineStr">
@@ -5516,6 +7828,39 @@
       <c r="U71" t="b">
         <v>0</v>
       </c>
+      <c r="V71" t="inlineStr">
+        <is>
+          <t>low</t>
+        </is>
+      </c>
+      <c r="W71" t="inlineStr">
+        <is>
+          <t>fail</t>
+        </is>
+      </c>
+      <c r="X71" t="inlineStr">
+        <is>
+          <t>pass</t>
+        </is>
+      </c>
+      <c r="Y71" t="inlineStr">
+        <is>
+          <t>pass</t>
+        </is>
+      </c>
+      <c r="Z71" t="inlineStr">
+        <is>
+          <t>fail</t>
+        </is>
+      </c>
+      <c r="AA71" t="inlineStr">
+        <is>
+          <t>uninformative</t>
+        </is>
+      </c>
+      <c r="AB71" t="n">
+        <v>-0.4829674976065112</v>
+      </c>
     </row>
     <row r="72">
       <c r="A72" t="inlineStr">
@@ -5589,6 +7934,39 @@
       <c r="U72" t="b">
         <v>0</v>
       </c>
+      <c r="V72" t="inlineStr">
+        <is>
+          <t>medium</t>
+        </is>
+      </c>
+      <c r="W72" t="inlineStr">
+        <is>
+          <t>fail</t>
+        </is>
+      </c>
+      <c r="X72" t="inlineStr">
+        <is>
+          <t>pass</t>
+        </is>
+      </c>
+      <c r="Y72" t="inlineStr">
+        <is>
+          <t>pass</t>
+        </is>
+      </c>
+      <c r="Z72" t="inlineStr">
+        <is>
+          <t>pass</t>
+        </is>
+      </c>
+      <c r="AA72" t="inlineStr">
+        <is>
+          <t>uninformative</t>
+        </is>
+      </c>
+      <c r="AB72" t="n">
+        <v>-0.5809887624308736</v>
+      </c>
     </row>
     <row r="73">
       <c r="A73" t="inlineStr">
@@ -5662,6 +8040,39 @@
       <c r="U73" t="b">
         <v>0</v>
       </c>
+      <c r="V73" t="inlineStr">
+        <is>
+          <t>low</t>
+        </is>
+      </c>
+      <c r="W73" t="inlineStr">
+        <is>
+          <t>fail</t>
+        </is>
+      </c>
+      <c r="X73" t="inlineStr">
+        <is>
+          <t>pass</t>
+        </is>
+      </c>
+      <c r="Y73" t="inlineStr">
+        <is>
+          <t>pass</t>
+        </is>
+      </c>
+      <c r="Z73" t="inlineStr">
+        <is>
+          <t>fail</t>
+        </is>
+      </c>
+      <c r="AA73" t="inlineStr">
+        <is>
+          <t>fail</t>
+        </is>
+      </c>
+      <c r="AB73" t="n">
+        <v>-0.4175859915536748</v>
+      </c>
     </row>
     <row r="74">
       <c r="A74" t="inlineStr">
@@ -5731,6 +8142,39 @@
       <c r="U74" t="b">
         <v>0</v>
       </c>
+      <c r="V74" t="inlineStr">
+        <is>
+          <t>medium</t>
+        </is>
+      </c>
+      <c r="W74" t="inlineStr">
+        <is>
+          <t>fail</t>
+        </is>
+      </c>
+      <c r="X74" t="inlineStr">
+        <is>
+          <t>pass</t>
+        </is>
+      </c>
+      <c r="Y74" t="inlineStr">
+        <is>
+          <t>pass</t>
+        </is>
+      </c>
+      <c r="Z74" t="inlineStr">
+        <is>
+          <t>pass</t>
+        </is>
+      </c>
+      <c r="AA74" t="inlineStr">
+        <is>
+          <t>uninformative</t>
+        </is>
+      </c>
+      <c r="AB74" t="n">
+        <v>-0.6075948579839998</v>
+      </c>
     </row>
     <row r="75">
       <c r="A75" t="inlineStr">
@@ -5804,6 +8248,39 @@
       <c r="U75" t="b">
         <v>0</v>
       </c>
+      <c r="V75" t="inlineStr">
+        <is>
+          <t>low</t>
+        </is>
+      </c>
+      <c r="W75" t="inlineStr">
+        <is>
+          <t>fail</t>
+        </is>
+      </c>
+      <c r="X75" t="inlineStr">
+        <is>
+          <t>pass</t>
+        </is>
+      </c>
+      <c r="Y75" t="inlineStr">
+        <is>
+          <t>pass</t>
+        </is>
+      </c>
+      <c r="Z75" t="inlineStr">
+        <is>
+          <t>pass</t>
+        </is>
+      </c>
+      <c r="AA75" t="inlineStr">
+        <is>
+          <t>fail</t>
+        </is>
+      </c>
+      <c r="AB75" t="n">
+        <v>-0.5691540206146471</v>
+      </c>
     </row>
     <row r="76">
       <c r="A76" t="inlineStr">
@@ -5873,6 +8350,39 @@
       <c r="U76" t="b">
         <v>0</v>
       </c>
+      <c r="V76" t="inlineStr">
+        <is>
+          <t>low</t>
+        </is>
+      </c>
+      <c r="W76" t="inlineStr">
+        <is>
+          <t>fail</t>
+        </is>
+      </c>
+      <c r="X76" t="inlineStr">
+        <is>
+          <t>pass</t>
+        </is>
+      </c>
+      <c r="Y76" t="inlineStr">
+        <is>
+          <t>pass</t>
+        </is>
+      </c>
+      <c r="Z76" t="inlineStr">
+        <is>
+          <t>fail</t>
+        </is>
+      </c>
+      <c r="AA76" t="inlineStr">
+        <is>
+          <t>uninformative</t>
+        </is>
+      </c>
+      <c r="AB76" t="n">
+        <v>-0.6334569158062046</v>
+      </c>
     </row>
     <row r="77">
       <c r="A77" t="inlineStr">
@@ -5942,6 +8452,39 @@
       <c r="U77" t="b">
         <v>0</v>
       </c>
+      <c r="V77" t="inlineStr">
+        <is>
+          <t>medium</t>
+        </is>
+      </c>
+      <c r="W77" t="inlineStr">
+        <is>
+          <t>fail</t>
+        </is>
+      </c>
+      <c r="X77" t="inlineStr">
+        <is>
+          <t>pass</t>
+        </is>
+      </c>
+      <c r="Y77" t="inlineStr">
+        <is>
+          <t>pass</t>
+        </is>
+      </c>
+      <c r="Z77" t="inlineStr">
+        <is>
+          <t>pass</t>
+        </is>
+      </c>
+      <c r="AA77" t="inlineStr">
+        <is>
+          <t>uninformative</t>
+        </is>
+      </c>
+      <c r="AB77" t="n">
+        <v>-0.5825202649451341</v>
+      </c>
     </row>
     <row r="78">
       <c r="A78" t="inlineStr">
@@ -6011,6 +8554,39 @@
       <c r="U78" t="b">
         <v>0</v>
       </c>
+      <c r="V78" t="inlineStr">
+        <is>
+          <t>medium</t>
+        </is>
+      </c>
+      <c r="W78" t="inlineStr">
+        <is>
+          <t>fail</t>
+        </is>
+      </c>
+      <c r="X78" t="inlineStr">
+        <is>
+          <t>pass</t>
+        </is>
+      </c>
+      <c r="Y78" t="inlineStr">
+        <is>
+          <t>pass</t>
+        </is>
+      </c>
+      <c r="Z78" t="inlineStr">
+        <is>
+          <t>pass</t>
+        </is>
+      </c>
+      <c r="AA78" t="inlineStr">
+        <is>
+          <t>uninformative</t>
+        </is>
+      </c>
+      <c r="AB78" t="n">
+        <v>-0.5709986819612969</v>
+      </c>
     </row>
     <row r="79">
       <c r="A79" t="inlineStr">
@@ -6080,6 +8656,39 @@
       <c r="U79" t="b">
         <v>0</v>
       </c>
+      <c r="V79" t="inlineStr">
+        <is>
+          <t>low</t>
+        </is>
+      </c>
+      <c r="W79" t="inlineStr">
+        <is>
+          <t>fail</t>
+        </is>
+      </c>
+      <c r="X79" t="inlineStr">
+        <is>
+          <t>pass</t>
+        </is>
+      </c>
+      <c r="Y79" t="inlineStr">
+        <is>
+          <t>uninformative</t>
+        </is>
+      </c>
+      <c r="Z79" t="inlineStr">
+        <is>
+          <t>fail</t>
+        </is>
+      </c>
+      <c r="AA79" t="inlineStr">
+        <is>
+          <t>uninformative</t>
+        </is>
+      </c>
+      <c r="AB79" t="n">
+        <v>-0.5793128756550876</v>
+      </c>
     </row>
     <row r="80">
       <c r="A80" t="inlineStr">
@@ -6153,6 +8762,39 @@
       <c r="U80" t="b">
         <v>0</v>
       </c>
+      <c r="V80" t="inlineStr">
+        <is>
+          <t>medium</t>
+        </is>
+      </c>
+      <c r="W80" t="inlineStr">
+        <is>
+          <t>fail</t>
+        </is>
+      </c>
+      <c r="X80" t="inlineStr">
+        <is>
+          <t>pass</t>
+        </is>
+      </c>
+      <c r="Y80" t="inlineStr">
+        <is>
+          <t>uninformative</t>
+        </is>
+      </c>
+      <c r="Z80" t="inlineStr">
+        <is>
+          <t>pass</t>
+        </is>
+      </c>
+      <c r="AA80" t="inlineStr">
+        <is>
+          <t>uninformative</t>
+        </is>
+      </c>
+      <c r="AB80" t="n">
+        <v>-0.557999846716411</v>
+      </c>
     </row>
     <row r="81">
       <c r="A81" t="inlineStr">
@@ -6222,6 +8864,39 @@
       <c r="U81" t="b">
         <v>0</v>
       </c>
+      <c r="V81" t="inlineStr">
+        <is>
+          <t>low</t>
+        </is>
+      </c>
+      <c r="W81" t="inlineStr">
+        <is>
+          <t>fail</t>
+        </is>
+      </c>
+      <c r="X81" t="inlineStr">
+        <is>
+          <t>pass</t>
+        </is>
+      </c>
+      <c r="Y81" t="inlineStr">
+        <is>
+          <t>pass</t>
+        </is>
+      </c>
+      <c r="Z81" t="inlineStr">
+        <is>
+          <t>fail</t>
+        </is>
+      </c>
+      <c r="AA81" t="inlineStr">
+        <is>
+          <t>uninformative</t>
+        </is>
+      </c>
+      <c r="AB81" t="n">
+        <v>-0.5907005201326848</v>
+      </c>
     </row>
     <row r="82">
       <c r="A82" t="inlineStr">
@@ -6295,6 +8970,39 @@
       <c r="U82" t="b">
         <v>0</v>
       </c>
+      <c r="V82" t="inlineStr">
+        <is>
+          <t>low</t>
+        </is>
+      </c>
+      <c r="W82" t="inlineStr">
+        <is>
+          <t>fail</t>
+        </is>
+      </c>
+      <c r="X82" t="inlineStr">
+        <is>
+          <t>pass</t>
+        </is>
+      </c>
+      <c r="Y82" t="inlineStr">
+        <is>
+          <t>fail</t>
+        </is>
+      </c>
+      <c r="Z82" t="inlineStr">
+        <is>
+          <t>pass</t>
+        </is>
+      </c>
+      <c r="AA82" t="inlineStr">
+        <is>
+          <t>uninformative</t>
+        </is>
+      </c>
+      <c r="AB82" t="n">
+        <v>-0.5490552745799622</v>
+      </c>
     </row>
     <row r="83">
       <c r="A83" t="inlineStr">
@@ -6368,6 +9076,39 @@
       <c r="U83" t="b">
         <v>0</v>
       </c>
+      <c r="V83" t="inlineStr">
+        <is>
+          <t>low</t>
+        </is>
+      </c>
+      <c r="W83" t="inlineStr">
+        <is>
+          <t>fail</t>
+        </is>
+      </c>
+      <c r="X83" t="inlineStr">
+        <is>
+          <t>pass</t>
+        </is>
+      </c>
+      <c r="Y83" t="inlineStr">
+        <is>
+          <t>pass</t>
+        </is>
+      </c>
+      <c r="Z83" t="inlineStr">
+        <is>
+          <t>fail</t>
+        </is>
+      </c>
+      <c r="AA83" t="inlineStr">
+        <is>
+          <t>pass</t>
+        </is>
+      </c>
+      <c r="AB83" t="n">
+        <v>-0.4329038982552768</v>
+      </c>
     </row>
     <row r="84">
       <c r="A84" t="inlineStr">
@@ -6441,6 +9182,39 @@
       <c r="U84" t="b">
         <v>0</v>
       </c>
+      <c r="V84" t="inlineStr">
+        <is>
+          <t>low</t>
+        </is>
+      </c>
+      <c r="W84" t="inlineStr">
+        <is>
+          <t>fail</t>
+        </is>
+      </c>
+      <c r="X84" t="inlineStr">
+        <is>
+          <t>pass</t>
+        </is>
+      </c>
+      <c r="Y84" t="inlineStr">
+        <is>
+          <t>fail</t>
+        </is>
+      </c>
+      <c r="Z84" t="inlineStr">
+        <is>
+          <t>pass</t>
+        </is>
+      </c>
+      <c r="AA84" t="inlineStr">
+        <is>
+          <t>fail</t>
+        </is>
+      </c>
+      <c r="AB84" t="n">
+        <v>-0.5434854187372423</v>
+      </c>
     </row>
     <row r="85">
       <c r="A85" t="inlineStr">
@@ -6510,6 +9284,39 @@
       <c r="U85" t="b">
         <v>0</v>
       </c>
+      <c r="V85" t="inlineStr">
+        <is>
+          <t>medium</t>
+        </is>
+      </c>
+      <c r="W85" t="inlineStr">
+        <is>
+          <t>fail</t>
+        </is>
+      </c>
+      <c r="X85" t="inlineStr">
+        <is>
+          <t>pass</t>
+        </is>
+      </c>
+      <c r="Y85" t="inlineStr">
+        <is>
+          <t>pass</t>
+        </is>
+      </c>
+      <c r="Z85" t="inlineStr">
+        <is>
+          <t>pass</t>
+        </is>
+      </c>
+      <c r="AA85" t="inlineStr">
+        <is>
+          <t>uninformative</t>
+        </is>
+      </c>
+      <c r="AB85" t="n">
+        <v>-0.5541170994409248</v>
+      </c>
     </row>
     <row r="86">
       <c r="A86" t="inlineStr">
@@ -6583,6 +9390,39 @@
       <c r="U86" t="b">
         <v>0</v>
       </c>
+      <c r="V86" t="inlineStr">
+        <is>
+          <t>low</t>
+        </is>
+      </c>
+      <c r="W86" t="inlineStr">
+        <is>
+          <t>fail</t>
+        </is>
+      </c>
+      <c r="X86" t="inlineStr">
+        <is>
+          <t>pass</t>
+        </is>
+      </c>
+      <c r="Y86" t="inlineStr">
+        <is>
+          <t>pass</t>
+        </is>
+      </c>
+      <c r="Z86" t="inlineStr">
+        <is>
+          <t>fail</t>
+        </is>
+      </c>
+      <c r="AA86" t="inlineStr">
+        <is>
+          <t>uninformative</t>
+        </is>
+      </c>
+      <c r="AB86" t="n">
+        <v>-0.4659543924848717</v>
+      </c>
     </row>
     <row r="87">
       <c r="A87" t="inlineStr">
@@ -6656,6 +9496,39 @@
       <c r="U87" t="b">
         <v>0</v>
       </c>
+      <c r="V87" t="inlineStr">
+        <is>
+          <t>low</t>
+        </is>
+      </c>
+      <c r="W87" t="inlineStr">
+        <is>
+          <t>fail</t>
+        </is>
+      </c>
+      <c r="X87" t="inlineStr">
+        <is>
+          <t>pass</t>
+        </is>
+      </c>
+      <c r="Y87" t="inlineStr">
+        <is>
+          <t>pass</t>
+        </is>
+      </c>
+      <c r="Z87" t="inlineStr">
+        <is>
+          <t>pass</t>
+        </is>
+      </c>
+      <c r="AA87" t="inlineStr">
+        <is>
+          <t>fail</t>
+        </is>
+      </c>
+      <c r="AB87" t="n">
+        <v>-0.5238564368019141</v>
+      </c>
     </row>
     <row r="88">
       <c r="A88" t="inlineStr">
@@ -6729,6 +9602,39 @@
       <c r="U88" t="b">
         <v>0</v>
       </c>
+      <c r="V88" t="inlineStr">
+        <is>
+          <t>low</t>
+        </is>
+      </c>
+      <c r="W88" t="inlineStr">
+        <is>
+          <t>fail</t>
+        </is>
+      </c>
+      <c r="X88" t="inlineStr">
+        <is>
+          <t>fail</t>
+        </is>
+      </c>
+      <c r="Y88" t="inlineStr">
+        <is>
+          <t>pass</t>
+        </is>
+      </c>
+      <c r="Z88" t="inlineStr">
+        <is>
+          <t>pass</t>
+        </is>
+      </c>
+      <c r="AA88" t="inlineStr">
+        <is>
+          <t>uninformative</t>
+        </is>
+      </c>
+      <c r="AB88" t="n">
+        <v>-0.5197542792992306</v>
+      </c>
     </row>
     <row r="89">
       <c r="A89" t="inlineStr">
@@ -6798,6 +9704,39 @@
       <c r="U89" t="b">
         <v>0</v>
       </c>
+      <c r="V89" t="inlineStr">
+        <is>
+          <t>low</t>
+        </is>
+      </c>
+      <c r="W89" t="inlineStr">
+        <is>
+          <t>fail</t>
+        </is>
+      </c>
+      <c r="X89" t="inlineStr">
+        <is>
+          <t>pass</t>
+        </is>
+      </c>
+      <c r="Y89" t="inlineStr">
+        <is>
+          <t>pass</t>
+        </is>
+      </c>
+      <c r="Z89" t="inlineStr">
+        <is>
+          <t>pass</t>
+        </is>
+      </c>
+      <c r="AA89" t="inlineStr">
+        <is>
+          <t>fail</t>
+        </is>
+      </c>
+      <c r="AB89" t="n">
+        <v>-0.5326815806970289</v>
+      </c>
     </row>
     <row r="90">
       <c r="A90" t="inlineStr">
@@ -6867,6 +9806,39 @@
       <c r="U90" t="b">
         <v>0</v>
       </c>
+      <c r="V90" t="inlineStr">
+        <is>
+          <t>low</t>
+        </is>
+      </c>
+      <c r="W90" t="inlineStr">
+        <is>
+          <t>fail</t>
+        </is>
+      </c>
+      <c r="X90" t="inlineStr">
+        <is>
+          <t>pass</t>
+        </is>
+      </c>
+      <c r="Y90" t="inlineStr">
+        <is>
+          <t>pass</t>
+        </is>
+      </c>
+      <c r="Z90" t="inlineStr">
+        <is>
+          <t>pass</t>
+        </is>
+      </c>
+      <c r="AA90" t="inlineStr">
+        <is>
+          <t>fail</t>
+        </is>
+      </c>
+      <c r="AB90" t="n">
+        <v>-0.524422411281307</v>
+      </c>
     </row>
     <row r="91">
       <c r="A91" t="inlineStr">
@@ -6936,6 +9908,39 @@
       <c r="U91" t="b">
         <v>0</v>
       </c>
+      <c r="V91" t="inlineStr">
+        <is>
+          <t>medium</t>
+        </is>
+      </c>
+      <c r="W91" t="inlineStr">
+        <is>
+          <t>fail</t>
+        </is>
+      </c>
+      <c r="X91" t="inlineStr">
+        <is>
+          <t>pass</t>
+        </is>
+      </c>
+      <c r="Y91" t="inlineStr">
+        <is>
+          <t>pass</t>
+        </is>
+      </c>
+      <c r="Z91" t="inlineStr">
+        <is>
+          <t>pass</t>
+        </is>
+      </c>
+      <c r="AA91" t="inlineStr">
+        <is>
+          <t>uninformative</t>
+        </is>
+      </c>
+      <c r="AB91" t="n">
+        <v>-0.5419115711284188</v>
+      </c>
     </row>
     <row r="92">
       <c r="A92" t="inlineStr">
@@ -7009,6 +10014,39 @@
       <c r="U92" t="b">
         <v>0</v>
       </c>
+      <c r="V92" t="inlineStr">
+        <is>
+          <t>low</t>
+        </is>
+      </c>
+      <c r="W92" t="inlineStr">
+        <is>
+          <t>fail</t>
+        </is>
+      </c>
+      <c r="X92" t="inlineStr">
+        <is>
+          <t>fail</t>
+        </is>
+      </c>
+      <c r="Y92" t="inlineStr">
+        <is>
+          <t>pass</t>
+        </is>
+      </c>
+      <c r="Z92" t="inlineStr">
+        <is>
+          <t>pass</t>
+        </is>
+      </c>
+      <c r="AA92" t="inlineStr">
+        <is>
+          <t>fail</t>
+        </is>
+      </c>
+      <c r="AB92" t="n">
+        <v>-0.5120978512924145</v>
+      </c>
     </row>
     <row r="93">
       <c r="A93" t="inlineStr">
@@ -7082,6 +10120,39 @@
       <c r="U93" t="b">
         <v>0</v>
       </c>
+      <c r="V93" t="inlineStr">
+        <is>
+          <t>low</t>
+        </is>
+      </c>
+      <c r="W93" t="inlineStr">
+        <is>
+          <t>fail</t>
+        </is>
+      </c>
+      <c r="X93" t="inlineStr">
+        <is>
+          <t>pass</t>
+        </is>
+      </c>
+      <c r="Y93" t="inlineStr">
+        <is>
+          <t>pass</t>
+        </is>
+      </c>
+      <c r="Z93" t="inlineStr">
+        <is>
+          <t>pass</t>
+        </is>
+      </c>
+      <c r="AA93" t="inlineStr">
+        <is>
+          <t>fail</t>
+        </is>
+      </c>
+      <c r="AB93" t="n">
+        <v>-0.543504133826032</v>
+      </c>
     </row>
     <row r="94">
       <c r="A94" t="inlineStr">
@@ -7155,6 +10226,39 @@
       <c r="U94" t="b">
         <v>0</v>
       </c>
+      <c r="V94" t="inlineStr">
+        <is>
+          <t>low</t>
+        </is>
+      </c>
+      <c r="W94" t="inlineStr">
+        <is>
+          <t>fail</t>
+        </is>
+      </c>
+      <c r="X94" t="inlineStr">
+        <is>
+          <t>fail</t>
+        </is>
+      </c>
+      <c r="Y94" t="inlineStr">
+        <is>
+          <t>fail</t>
+        </is>
+      </c>
+      <c r="Z94" t="inlineStr">
+        <is>
+          <t>fail</t>
+        </is>
+      </c>
+      <c r="AA94" t="inlineStr">
+        <is>
+          <t>uninformative</t>
+        </is>
+      </c>
+      <c r="AB94" t="n">
+        <v>-0.4855774995215112</v>
+      </c>
     </row>
     <row r="95">
       <c r="A95" t="inlineStr">
@@ -7227,6 +10331,39 @@
       </c>
       <c r="U95" t="b">
         <v>0</v>
+      </c>
+      <c r="V95" t="inlineStr">
+        <is>
+          <t>low</t>
+        </is>
+      </c>
+      <c r="W95" t="inlineStr">
+        <is>
+          <t>fail</t>
+        </is>
+      </c>
+      <c r="X95" t="inlineStr">
+        <is>
+          <t>pass</t>
+        </is>
+      </c>
+      <c r="Y95" t="inlineStr">
+        <is>
+          <t>pass</t>
+        </is>
+      </c>
+      <c r="Z95" t="inlineStr">
+        <is>
+          <t>pass</t>
+        </is>
+      </c>
+      <c r="AA95" t="inlineStr">
+        <is>
+          <t>fail</t>
+        </is>
+      </c>
+      <c r="AB95" t="n">
+        <v>-0.6150292625587572</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
rnai_validation.py: orthogonal check of the prioritised pairs in DEMETER2 RNAi screens; S2/S3 Tables, README, checksums
Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/figures/supporting_information/S2_Table.xlsx
+++ b/figures/supporting_information/S2_Table.xlsx
@@ -425,7 +425,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:AB95"/>
+  <dimension ref="A1:AG95"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -569,6 +569,31 @@
           <t>Selectivity without suspension lines in the comparison group</t>
         </is>
       </c>
+      <c r="AC1" s="1" t="inlineStr">
+        <is>
+          <t>RNAi: n target</t>
+        </is>
+      </c>
+      <c r="AD1" s="1" t="inlineStr">
+        <is>
+          <t>RNAi: median DEMETER2 score, target lineage</t>
+        </is>
+      </c>
+      <c r="AE1" s="1" t="inlineStr">
+        <is>
+          <t>RNAi: selectivity</t>
+        </is>
+      </c>
+      <c r="AF1" s="1" t="inlineStr">
+        <is>
+          <t>RNAi: q (BH over all RNAi tests)</t>
+        </is>
+      </c>
+      <c r="AG1" s="1" t="inlineStr">
+        <is>
+          <t>RNAi: confirmed (q &lt; 0.05, negative selectivity)</t>
+        </is>
+      </c>
     </row>
     <row r="2">
       <c r="A2" t="inlineStr">
@@ -675,6 +700,21 @@
       <c r="AB2" t="n">
         <v>-1.58201152192072</v>
       </c>
+      <c r="AC2" t="n">
+        <v>32</v>
+      </c>
+      <c r="AD2" t="n">
+        <v>-0.7907249264314999</v>
+      </c>
+      <c r="AE2" t="n">
+        <v>-0.6770184262954999</v>
+      </c>
+      <c r="AF2" t="n">
+        <v>1.07355091345946e-10</v>
+      </c>
+      <c r="AG2" t="b">
+        <v>1</v>
+      </c>
     </row>
     <row r="3">
       <c r="A3" t="inlineStr">
@@ -781,6 +821,21 @@
       <c r="AB3" t="n">
         <v>-1.365346268416268</v>
       </c>
+      <c r="AC3" t="n">
+        <v>47</v>
+      </c>
+      <c r="AD3" t="n">
+        <v>-0.626230675443</v>
+      </c>
+      <c r="AE3" t="n">
+        <v>-0.66765903132215</v>
+      </c>
+      <c r="AF3" t="n">
+        <v>1.203768181296743e-13</v>
+      </c>
+      <c r="AG3" t="b">
+        <v>1</v>
+      </c>
     </row>
     <row r="4">
       <c r="A4" t="inlineStr">
@@ -887,6 +942,21 @@
       <c r="AB4" t="n">
         <v>-1.26224975866103</v>
       </c>
+      <c r="AC4" t="n">
+        <v>30</v>
+      </c>
+      <c r="AD4" t="n">
+        <v>-0.6122337129855</v>
+      </c>
+      <c r="AE4" t="n">
+        <v>-0.6370989342779</v>
+      </c>
+      <c r="AF4" t="n">
+        <v>3.944109540741884e-06</v>
+      </c>
+      <c r="AG4" t="b">
+        <v>1</v>
+      </c>
     </row>
     <row r="5">
       <c r="A5" t="inlineStr">
@@ -993,6 +1063,21 @@
       <c r="AB5" t="n">
         <v>-1.238492317464168</v>
       </c>
+      <c r="AC5" t="n">
+        <v>7</v>
+      </c>
+      <c r="AD5" t="n">
+        <v>-0.559273768043</v>
+      </c>
+      <c r="AE5" t="n">
+        <v>-0.5059126675251</v>
+      </c>
+      <c r="AF5" t="n">
+        <v>0.0094071474978044</v>
+      </c>
+      <c r="AG5" t="b">
+        <v>1</v>
+      </c>
     </row>
     <row r="6">
       <c r="A6" t="inlineStr">
@@ -1099,6 +1184,13 @@
       <c r="AB6" t="n">
         <v>-1.125345804313242</v>
       </c>
+      <c r="AC6" t="inlineStr"/>
+      <c r="AD6" t="inlineStr"/>
+      <c r="AE6" t="inlineStr"/>
+      <c r="AF6" t="inlineStr"/>
+      <c r="AG6" t="b">
+        <v>0</v>
+      </c>
     </row>
     <row r="7">
       <c r="A7" t="inlineStr">
@@ -1205,6 +1297,21 @@
       <c r="AB7" t="n">
         <v>-1.113757459659644</v>
       </c>
+      <c r="AC7" t="n">
+        <v>48</v>
+      </c>
+      <c r="AD7" t="n">
+        <v>-1.48870180113</v>
+      </c>
+      <c r="AE7" t="n">
+        <v>-1.4186712161405</v>
+      </c>
+      <c r="AF7" t="n">
+        <v>6.973581087284193e-16</v>
+      </c>
+      <c r="AG7" t="b">
+        <v>1</v>
+      </c>
     </row>
     <row r="8">
       <c r="A8" t="inlineStr">
@@ -1311,6 +1418,21 @@
       <c r="AB8" t="n">
         <v>-1.072469868432948</v>
       </c>
+      <c r="AC8" t="n">
+        <v>30</v>
+      </c>
+      <c r="AD8" t="n">
+        <v>-0.396646494149</v>
+      </c>
+      <c r="AE8" t="n">
+        <v>-0.218886220542</v>
+      </c>
+      <c r="AF8" t="n">
+        <v>0.09940649233118209</v>
+      </c>
+      <c r="AG8" t="b">
+        <v>0</v>
+      </c>
     </row>
     <row r="9">
       <c r="A9" t="inlineStr">
@@ -1413,6 +1535,21 @@
       <c r="AB9" t="n">
         <v>-1.072872853944649</v>
       </c>
+      <c r="AC9" t="n">
+        <v>25</v>
+      </c>
+      <c r="AD9" t="n">
+        <v>-0.659220502448</v>
+      </c>
+      <c r="AE9" t="n">
+        <v>-0.6955904556900501</v>
+      </c>
+      <c r="AF9" t="n">
+        <v>1.22585880086157e-11</v>
+      </c>
+      <c r="AG9" t="b">
+        <v>1</v>
+      </c>
     </row>
     <row r="10">
       <c r="A10" t="inlineStr">
@@ -1515,6 +1652,21 @@
       <c r="AB10" t="n">
         <v>-1.082806882382966</v>
       </c>
+      <c r="AC10" t="n">
+        <v>25</v>
+      </c>
+      <c r="AD10" t="n">
+        <v>-0.6616096315510001</v>
+      </c>
+      <c r="AE10" t="n">
+        <v>-0.66306432792573</v>
+      </c>
+      <c r="AF10" t="n">
+        <v>3.14609244905087e-10</v>
+      </c>
+      <c r="AG10" t="b">
+        <v>1</v>
+      </c>
     </row>
     <row r="11">
       <c r="A11" t="inlineStr">
@@ -1621,6 +1773,13 @@
       <c r="AB11" t="n">
         <v>-1.031480749922119</v>
       </c>
+      <c r="AC11" t="inlineStr"/>
+      <c r="AD11" t="inlineStr"/>
+      <c r="AE11" t="inlineStr"/>
+      <c r="AF11" t="inlineStr"/>
+      <c r="AG11" t="b">
+        <v>0</v>
+      </c>
     </row>
     <row r="12">
       <c r="A12" t="inlineStr">
@@ -1727,6 +1886,21 @@
       <c r="AB12" t="n">
         <v>-1.012640543351392</v>
       </c>
+      <c r="AC12" t="n">
+        <v>30</v>
+      </c>
+      <c r="AD12" t="n">
+        <v>-0.466436227065</v>
+      </c>
+      <c r="AE12" t="n">
+        <v>-0.4531535384439999</v>
+      </c>
+      <c r="AF12" t="n">
+        <v>2.952616087655184e-09</v>
+      </c>
+      <c r="AG12" t="b">
+        <v>1</v>
+      </c>
     </row>
     <row r="13">
       <c r="A13" t="inlineStr">
@@ -1833,6 +2007,21 @@
       <c r="AB13" t="n">
         <v>-1.004424871336947</v>
       </c>
+      <c r="AC13" t="n">
+        <v>47</v>
+      </c>
+      <c r="AD13" t="n">
+        <v>-0.745276630305</v>
+      </c>
+      <c r="AE13" t="n">
+        <v>-0.7480611459936151</v>
+      </c>
+      <c r="AF13" t="n">
+        <v>1.051333992974078e-12</v>
+      </c>
+      <c r="AG13" t="b">
+        <v>1</v>
+      </c>
     </row>
     <row r="14">
       <c r="A14" t="inlineStr">
@@ -1939,6 +2128,13 @@
       <c r="AB14" t="n">
         <v>-0.9882905978980336</v>
       </c>
+      <c r="AC14" t="inlineStr"/>
+      <c r="AD14" t="inlineStr"/>
+      <c r="AE14" t="inlineStr"/>
+      <c r="AF14" t="inlineStr"/>
+      <c r="AG14" t="b">
+        <v>0</v>
+      </c>
     </row>
     <row r="15">
       <c r="A15" t="inlineStr">
@@ -2041,6 +2237,21 @@
       <c r="AB15" t="n">
         <v>-0.9639799440870452</v>
       </c>
+      <c r="AC15" t="n">
+        <v>35</v>
+      </c>
+      <c r="AD15" t="n">
+        <v>-0.107121873769</v>
+      </c>
+      <c r="AE15" t="n">
+        <v>-0.06294062613665</v>
+      </c>
+      <c r="AF15" t="n">
+        <v>0.6754463501916057</v>
+      </c>
+      <c r="AG15" t="b">
+        <v>0</v>
+      </c>
     </row>
     <row r="16">
       <c r="A16" t="inlineStr">
@@ -2143,6 +2354,21 @@
       <c r="AB16" t="n">
         <v>-0.9432738793226464</v>
       </c>
+      <c r="AC16" t="n">
+        <v>35</v>
+      </c>
+      <c r="AD16" t="n">
+        <v>-0.189123495356</v>
+      </c>
+      <c r="AE16" t="n">
+        <v>-0.22483615498405</v>
+      </c>
+      <c r="AF16" t="n">
+        <v>1.142024211032387e-08</v>
+      </c>
+      <c r="AG16" t="b">
+        <v>1</v>
+      </c>
     </row>
     <row r="17">
       <c r="A17" t="inlineStr">
@@ -2249,6 +2475,21 @@
       <c r="AB17" t="n">
         <v>-0.7701057966378611</v>
       </c>
+      <c r="AC17" t="n">
+        <v>9</v>
+      </c>
+      <c r="AD17" t="n">
+        <v>-1.10664584035</v>
+      </c>
+      <c r="AE17" t="n">
+        <v>-0.8968104558529999</v>
+      </c>
+      <c r="AF17" t="n">
+        <v>0.0012293943732588</v>
+      </c>
+      <c r="AG17" t="b">
+        <v>1</v>
+      </c>
     </row>
     <row r="18">
       <c r="A18" t="inlineStr">
@@ -2355,6 +2596,21 @@
       <c r="AB18" t="n">
         <v>-0.8094174294517624</v>
       </c>
+      <c r="AC18" t="n">
+        <v>24</v>
+      </c>
+      <c r="AD18" t="n">
+        <v>-0.4696132029559999</v>
+      </c>
+      <c r="AE18" t="n">
+        <v>-0.3640232577259999</v>
+      </c>
+      <c r="AF18" t="n">
+        <v>0.0002857162094531</v>
+      </c>
+      <c r="AG18" t="b">
+        <v>1</v>
+      </c>
     </row>
     <row r="19">
       <c r="A19" t="inlineStr">
@@ -2461,6 +2717,13 @@
       <c r="AB19" t="n">
         <v>-0.8991478476896867</v>
       </c>
+      <c r="AC19" t="inlineStr"/>
+      <c r="AD19" t="inlineStr"/>
+      <c r="AE19" t="inlineStr"/>
+      <c r="AF19" t="inlineStr"/>
+      <c r="AG19" t="b">
+        <v>0</v>
+      </c>
     </row>
     <row r="20">
       <c r="A20" t="inlineStr">
@@ -2567,6 +2830,21 @@
       <c r="AB20" t="n">
         <v>-0.8633316194200893</v>
       </c>
+      <c r="AC20" t="n">
+        <v>30</v>
+      </c>
+      <c r="AD20" t="n">
+        <v>-0.4194120681415</v>
+      </c>
+      <c r="AE20" t="n">
+        <v>-0.462016267625</v>
+      </c>
+      <c r="AF20" t="n">
+        <v>6.867916923524099e-05</v>
+      </c>
+      <c r="AG20" t="b">
+        <v>1</v>
+      </c>
     </row>
     <row r="21">
       <c r="A21" t="inlineStr">
@@ -2673,6 +2951,21 @@
       <c r="AB21" t="n">
         <v>-0.850555099680339</v>
       </c>
+      <c r="AC21" t="n">
+        <v>6</v>
+      </c>
+      <c r="AD21" t="n">
+        <v>-0.35521191935135</v>
+      </c>
+      <c r="AE21" t="n">
+        <v>-0.39305793268485</v>
+      </c>
+      <c r="AF21" t="n">
+        <v>0.4397213776505249</v>
+      </c>
+      <c r="AG21" t="b">
+        <v>0</v>
+      </c>
     </row>
     <row r="22">
       <c r="A22" t="inlineStr">
@@ -2779,6 +3072,13 @@
       <c r="AB22" t="n">
         <v>-0.8294961143416411</v>
       </c>
+      <c r="AC22" t="inlineStr"/>
+      <c r="AD22" t="inlineStr"/>
+      <c r="AE22" t="inlineStr"/>
+      <c r="AF22" t="inlineStr"/>
+      <c r="AG22" t="b">
+        <v>0</v>
+      </c>
     </row>
     <row r="23">
       <c r="A23" t="inlineStr">
@@ -2885,6 +3185,21 @@
       <c r="AB23" t="n">
         <v>-0.8114075168145537</v>
       </c>
+      <c r="AC23" t="n">
+        <v>47</v>
+      </c>
+      <c r="AD23" t="n">
+        <v>-0.403139552433</v>
+      </c>
+      <c r="AE23" t="n">
+        <v>-0.4452628291852</v>
+      </c>
+      <c r="AF23" t="n">
+        <v>0.0001866365310995</v>
+      </c>
+      <c r="AG23" t="b">
+        <v>1</v>
+      </c>
     </row>
     <row r="24">
       <c r="A24" t="inlineStr">
@@ -2987,6 +3302,21 @@
       <c r="AB24" t="n">
         <v>-0.8205412491305067</v>
       </c>
+      <c r="AC24" t="n">
+        <v>25</v>
+      </c>
+      <c r="AD24" t="n">
+        <v>-0.0258159656912</v>
+      </c>
+      <c r="AE24" t="n">
+        <v>-0.02792919759184</v>
+      </c>
+      <c r="AF24" t="n">
+        <v>0.2986652126343077</v>
+      </c>
+      <c r="AG24" t="b">
+        <v>0</v>
+      </c>
     </row>
     <row r="25">
       <c r="A25" t="inlineStr">
@@ -3089,6 +3419,21 @@
       <c r="AB25" t="n">
         <v>-0.8322255705482856</v>
       </c>
+      <c r="AC25" t="n">
+        <v>21</v>
+      </c>
+      <c r="AD25" t="n">
+        <v>-0.0478276672339</v>
+      </c>
+      <c r="AE25" t="n">
+        <v>-0.1442039907944</v>
+      </c>
+      <c r="AF25" t="n">
+        <v>0.0171163661506576</v>
+      </c>
+      <c r="AG25" t="b">
+        <v>1</v>
+      </c>
     </row>
     <row r="26">
       <c r="A26" t="inlineStr">
@@ -3191,6 +3536,21 @@
       <c r="AB26" t="n">
         <v>-0.8447951576685384</v>
       </c>
+      <c r="AC26" t="n">
+        <v>11</v>
+      </c>
+      <c r="AD26" t="n">
+        <v>-0.446324731511</v>
+      </c>
+      <c r="AE26" t="n">
+        <v>-0.189546274989</v>
+      </c>
+      <c r="AF26" t="n">
+        <v>0.0502625644887586</v>
+      </c>
+      <c r="AG26" t="b">
+        <v>0</v>
+      </c>
     </row>
     <row r="27">
       <c r="A27" t="inlineStr">
@@ -3293,6 +3653,21 @@
       <c r="AB27" t="n">
         <v>-0.7995231952144938</v>
       </c>
+      <c r="AC27" t="n">
+        <v>35</v>
+      </c>
+      <c r="AD27" t="n">
+        <v>-0.0845733806453</v>
+      </c>
+      <c r="AE27" t="n">
+        <v>0.0804879410477</v>
+      </c>
+      <c r="AF27" t="n">
+        <v>1</v>
+      </c>
+      <c r="AG27" t="b">
+        <v>0</v>
+      </c>
     </row>
     <row r="28">
       <c r="A28" t="inlineStr">
@@ -3399,6 +3774,21 @@
       <c r="AB28" t="n">
         <v>-0.7963184334088669</v>
       </c>
+      <c r="AC28" t="n">
+        <v>44</v>
+      </c>
+      <c r="AD28" t="n">
+        <v>-0.061038496264</v>
+      </c>
+      <c r="AE28" t="n">
+        <v>-0.05063221455227</v>
+      </c>
+      <c r="AF28" t="n">
+        <v>0.3222360544805334</v>
+      </c>
+      <c r="AG28" t="b">
+        <v>0</v>
+      </c>
     </row>
     <row r="29">
       <c r="A29" t="inlineStr">
@@ -3501,6 +3891,21 @@
       <c r="AB29" t="n">
         <v>-0.7864619692219967</v>
       </c>
+      <c r="AC29" t="n">
+        <v>25</v>
+      </c>
+      <c r="AD29" t="n">
+        <v>0.07713426860979999</v>
+      </c>
+      <c r="AE29" t="n">
+        <v>-0.0145622134985499</v>
+      </c>
+      <c r="AF29" t="n">
+        <v>0.6853664252519956</v>
+      </c>
+      <c r="AG29" t="b">
+        <v>0</v>
+      </c>
     </row>
     <row r="30">
       <c r="A30" t="inlineStr">
@@ -3607,6 +4012,21 @@
       <c r="AB30" t="n">
         <v>-0.824318745705738</v>
       </c>
+      <c r="AC30" t="n">
+        <v>24</v>
+      </c>
+      <c r="AD30" t="n">
+        <v>0.2431812023945</v>
+      </c>
+      <c r="AE30" t="n">
+        <v>0.15547158197</v>
+      </c>
+      <c r="AF30" t="n">
+        <v>1</v>
+      </c>
+      <c r="AG30" t="b">
+        <v>0</v>
+      </c>
     </row>
     <row r="31">
       <c r="A31" t="inlineStr">
@@ -3709,6 +4129,21 @@
       <c r="AB31" t="n">
         <v>-0.77309606094219</v>
       </c>
+      <c r="AC31" t="n">
+        <v>25</v>
+      </c>
+      <c r="AD31" t="n">
+        <v>-0.0719897096119</v>
+      </c>
+      <c r="AE31" t="n">
+        <v>-0.1688276451951</v>
+      </c>
+      <c r="AF31" t="n">
+        <v>0.0010066982974493</v>
+      </c>
+      <c r="AG31" t="b">
+        <v>1</v>
+      </c>
     </row>
     <row r="32">
       <c r="A32" t="inlineStr">
@@ -3815,6 +4250,21 @@
       <c r="AB32" t="n">
         <v>-0.6381595903457972</v>
       </c>
+      <c r="AC32" t="n">
+        <v>45</v>
+      </c>
+      <c r="AD32" t="n">
+        <v>-0.384492686807</v>
+      </c>
+      <c r="AE32" t="n">
+        <v>-0.2812998829699999</v>
+      </c>
+      <c r="AF32" t="n">
+        <v>6.455073790426178e-05</v>
+      </c>
+      <c r="AG32" t="b">
+        <v>1</v>
+      </c>
     </row>
     <row r="33">
       <c r="A33" t="inlineStr">
@@ -3917,6 +4367,21 @@
       <c r="AB33" t="n">
         <v>-0.7761335756286625</v>
       </c>
+      <c r="AC33" t="n">
+        <v>35</v>
+      </c>
+      <c r="AD33" t="n">
+        <v>-0.6337740700259999</v>
+      </c>
+      <c r="AE33" t="n">
+        <v>-0.0711168508259999</v>
+      </c>
+      <c r="AF33" t="n">
+        <v>0.5215960393226162</v>
+      </c>
+      <c r="AG33" t="b">
+        <v>0</v>
+      </c>
     </row>
     <row r="34">
       <c r="A34" t="inlineStr">
@@ -4019,6 +4484,21 @@
       <c r="AB34" t="n">
         <v>-0.7640925562537549</v>
       </c>
+      <c r="AC34" t="n">
+        <v>25</v>
+      </c>
+      <c r="AD34" t="n">
+        <v>-0.213719030698</v>
+      </c>
+      <c r="AE34" t="n">
+        <v>-0.0522154659394999</v>
+      </c>
+      <c r="AF34" t="n">
+        <v>0.292293207802129</v>
+      </c>
+      <c r="AG34" t="b">
+        <v>0</v>
+      </c>
     </row>
     <row r="35">
       <c r="A35" t="inlineStr">
@@ -4121,6 +4601,21 @@
       <c r="AB35" t="n">
         <v>-0.7585993381851116</v>
       </c>
+      <c r="AC35" t="n">
+        <v>35</v>
+      </c>
+      <c r="AD35" t="n">
+        <v>-0.187107842751</v>
+      </c>
+      <c r="AE35" t="n">
+        <v>-0.09264280502900001</v>
+      </c>
+      <c r="AF35" t="n">
+        <v>0.0467332025525786</v>
+      </c>
+      <c r="AG35" t="b">
+        <v>1</v>
+      </c>
     </row>
     <row r="36">
       <c r="A36" t="inlineStr">
@@ -4223,6 +4718,21 @@
       <c r="AB36" t="n">
         <v>-0.8011424948958573</v>
       </c>
+      <c r="AC36" t="n">
+        <v>25</v>
+      </c>
+      <c r="AD36" t="n">
+        <v>-0.393947061792</v>
+      </c>
+      <c r="AE36" t="n">
+        <v>-0.092751146469</v>
+      </c>
+      <c r="AF36" t="n">
+        <v>0.6847871497545607</v>
+      </c>
+      <c r="AG36" t="b">
+        <v>0</v>
+      </c>
     </row>
     <row r="37">
       <c r="A37" t="inlineStr">
@@ -4329,6 +4839,21 @@
       <c r="AB37" t="n">
         <v>-0.5607301556030795</v>
       </c>
+      <c r="AC37" t="n">
+        <v>47</v>
+      </c>
+      <c r="AD37" t="n">
+        <v>-0.486904345647</v>
+      </c>
+      <c r="AE37" t="n">
+        <v>-0.294173121605</v>
+      </c>
+      <c r="AF37" t="n">
+        <v>0.0012190304751744</v>
+      </c>
+      <c r="AG37" t="b">
+        <v>1</v>
+      </c>
     </row>
     <row r="38">
       <c r="A38" t="inlineStr">
@@ -4431,6 +4956,21 @@
       <c r="AB38" t="n">
         <v>-0.7254931543108373</v>
       </c>
+      <c r="AC38" t="n">
+        <v>35</v>
+      </c>
+      <c r="AD38" t="n">
+        <v>-0.170524945827</v>
+      </c>
+      <c r="AE38" t="n">
+        <v>0.002708399016</v>
+      </c>
+      <c r="AF38" t="n">
+        <v>1</v>
+      </c>
+      <c r="AG38" t="b">
+        <v>0</v>
+      </c>
     </row>
     <row r="39">
       <c r="A39" t="inlineStr">
@@ -4533,6 +5073,21 @@
       <c r="AB39" t="n">
         <v>-0.7505522707815774</v>
       </c>
+      <c r="AC39" t="n">
+        <v>25</v>
+      </c>
+      <c r="AD39" t="n">
+        <v>0.154529995619</v>
+      </c>
+      <c r="AE39" t="n">
+        <v>0.0281688132604999</v>
+      </c>
+      <c r="AF39" t="n">
+        <v>1</v>
+      </c>
+      <c r="AG39" t="b">
+        <v>0</v>
+      </c>
     </row>
     <row r="40">
       <c r="A40" t="inlineStr">
@@ -4635,6 +5190,21 @@
       <c r="AB40" t="n">
         <v>-0.7263489324389152</v>
       </c>
+      <c r="AC40" t="n">
+        <v>35</v>
+      </c>
+      <c r="AD40" t="n">
+        <v>-0.297505737766</v>
+      </c>
+      <c r="AE40" t="n">
+        <v>-0.35171071011765</v>
+      </c>
+      <c r="AF40" t="n">
+        <v>2.068007602419394e-06</v>
+      </c>
+      <c r="AG40" t="b">
+        <v>1</v>
+      </c>
     </row>
     <row r="41">
       <c r="A41" t="inlineStr">
@@ -4741,6 +5311,21 @@
       <c r="AB41" t="n">
         <v>-0.6907123574774108</v>
       </c>
+      <c r="AC41" t="n">
+        <v>48</v>
+      </c>
+      <c r="AD41" t="n">
+        <v>-0.3108893870965</v>
+      </c>
+      <c r="AE41" t="n">
+        <v>-0.2090858874085</v>
+      </c>
+      <c r="AF41" t="n">
+        <v>0.210816233115083</v>
+      </c>
+      <c r="AG41" t="b">
+        <v>0</v>
+      </c>
     </row>
     <row r="42">
       <c r="A42" t="inlineStr">
@@ -4847,6 +5432,21 @@
       <c r="AB42" t="n">
         <v>-0.7068140094748493</v>
       </c>
+      <c r="AC42" t="n">
+        <v>48</v>
+      </c>
+      <c r="AD42" t="n">
+        <v>-0.335423061252</v>
+      </c>
+      <c r="AE42" t="n">
+        <v>-0.217096837904</v>
+      </c>
+      <c r="AF42" t="n">
+        <v>0.0525555149851436</v>
+      </c>
+      <c r="AG42" t="b">
+        <v>0</v>
+      </c>
     </row>
     <row r="43">
       <c r="A43" t="inlineStr">
@@ -4953,6 +5553,13 @@
       <c r="AB43" t="n">
         <v>-0.694880903531901</v>
       </c>
+      <c r="AC43" t="inlineStr"/>
+      <c r="AD43" t="inlineStr"/>
+      <c r="AE43" t="inlineStr"/>
+      <c r="AF43" t="inlineStr"/>
+      <c r="AG43" t="b">
+        <v>0</v>
+      </c>
     </row>
     <row r="44">
       <c r="A44" t="inlineStr">
@@ -5055,6 +5662,21 @@
       <c r="AB44" t="n">
         <v>-0.7400333291868505</v>
       </c>
+      <c r="AC44" t="n">
+        <v>35</v>
+      </c>
+      <c r="AD44" t="n">
+        <v>-0.4774201206</v>
+      </c>
+      <c r="AE44" t="n">
+        <v>-0.1797593753399999</v>
+      </c>
+      <c r="AF44" t="n">
+        <v>0.1006053061546971</v>
+      </c>
+      <c r="AG44" t="b">
+        <v>0</v>
+      </c>
     </row>
     <row r="45">
       <c r="A45" t="inlineStr">
@@ -5161,6 +5783,21 @@
       <c r="AB45" t="n">
         <v>-0.7014886620371761</v>
       </c>
+      <c r="AC45" t="n">
+        <v>5</v>
+      </c>
+      <c r="AD45" t="n">
+        <v>0.0569621106372</v>
+      </c>
+      <c r="AE45" t="n">
+        <v>0.0700453744579999</v>
+      </c>
+      <c r="AF45" t="n">
+        <v>1</v>
+      </c>
+      <c r="AG45" t="b">
+        <v>0</v>
+      </c>
     </row>
     <row r="46">
       <c r="A46" t="inlineStr">
@@ -5267,6 +5904,21 @@
       <c r="AB46" t="n">
         <v>-0.7082557415859232</v>
       </c>
+      <c r="AC46" t="n">
+        <v>48</v>
+      </c>
+      <c r="AD46" t="n">
+        <v>-0.3783910751804999</v>
+      </c>
+      <c r="AE46" t="n">
+        <v>-0.1951922491984999</v>
+      </c>
+      <c r="AF46" t="n">
+        <v>0.0018158748052098</v>
+      </c>
+      <c r="AG46" t="b">
+        <v>1</v>
+      </c>
     </row>
     <row r="47">
       <c r="A47" t="inlineStr">
@@ -5369,6 +6021,21 @@
       <c r="AB47" t="n">
         <v>-0.6854512593382545</v>
       </c>
+      <c r="AC47" t="n">
+        <v>11</v>
+      </c>
+      <c r="AD47" t="n">
+        <v>-0.691623201557</v>
+      </c>
+      <c r="AE47" t="n">
+        <v>0.148270535992</v>
+      </c>
+      <c r="AF47" t="n">
+        <v>1</v>
+      </c>
+      <c r="AG47" t="b">
+        <v>0</v>
+      </c>
     </row>
     <row r="48">
       <c r="A48" t="inlineStr">
@@ -5475,6 +6142,21 @@
       <c r="AB48" t="n">
         <v>-0.7046353497966003</v>
       </c>
+      <c r="AC48" t="n">
+        <v>6</v>
+      </c>
+      <c r="AD48" t="n">
+        <v>-0.2365382849805</v>
+      </c>
+      <c r="AE48" t="n">
+        <v>-0.034824478637</v>
+      </c>
+      <c r="AF48" t="n">
+        <v>0.5634748184963327</v>
+      </c>
+      <c r="AG48" t="b">
+        <v>0</v>
+      </c>
     </row>
     <row r="49">
       <c r="A49" t="inlineStr">
@@ -5577,6 +6259,21 @@
       <c r="AB49" t="n">
         <v>-0.6833950316113085</v>
       </c>
+      <c r="AC49" t="n">
+        <v>25</v>
+      </c>
+      <c r="AD49" t="n">
+        <v>0.0235020796742</v>
+      </c>
+      <c r="AE49" t="n">
+        <v>0.0593630115319</v>
+      </c>
+      <c r="AF49" t="n">
+        <v>1</v>
+      </c>
+      <c r="AG49" t="b">
+        <v>0</v>
+      </c>
     </row>
     <row r="50">
       <c r="A50" t="inlineStr">
@@ -5679,6 +6376,21 @@
       <c r="AB50" t="n">
         <v>-0.6861349236785185</v>
       </c>
+      <c r="AC50" t="n">
+        <v>35</v>
+      </c>
+      <c r="AD50" t="n">
+        <v>-0.336740396517</v>
+      </c>
+      <c r="AE50" t="n">
+        <v>-0.2104751638845</v>
+      </c>
+      <c r="AF50" t="n">
+        <v>2.159259261715311e-05</v>
+      </c>
+      <c r="AG50" t="b">
+        <v>1</v>
+      </c>
     </row>
     <row r="51">
       <c r="A51" t="inlineStr">
@@ -5781,6 +6493,21 @@
       <c r="AB51" t="n">
         <v>-0.6799546558213418</v>
       </c>
+      <c r="AC51" t="n">
+        <v>25</v>
+      </c>
+      <c r="AD51" t="n">
+        <v>-0.288892229694</v>
+      </c>
+      <c r="AE51" t="n">
+        <v>-0.159675398326</v>
+      </c>
+      <c r="AF51" t="n">
+        <v>0.5236754523565743</v>
+      </c>
+      <c r="AG51" t="b">
+        <v>0</v>
+      </c>
     </row>
     <row r="52">
       <c r="A52" t="inlineStr">
@@ -5887,6 +6614,21 @@
       <c r="AB52" t="n">
         <v>-0.5460604599363266</v>
       </c>
+      <c r="AC52" t="n">
+        <v>17</v>
+      </c>
+      <c r="AD52" t="n">
+        <v>-0.243470477062</v>
+      </c>
+      <c r="AE52" t="n">
+        <v>-0.136727396118</v>
+      </c>
+      <c r="AF52" t="n">
+        <v>0.1314240485531233</v>
+      </c>
+      <c r="AG52" t="b">
+        <v>0</v>
+      </c>
     </row>
     <row r="53">
       <c r="A53" t="inlineStr">
@@ -5989,6 +6731,21 @@
       <c r="AB53" t="n">
         <v>-0.6639348892766579</v>
       </c>
+      <c r="AC53" t="n">
+        <v>14</v>
+      </c>
+      <c r="AD53" t="n">
+        <v>-0.2805461602285</v>
+      </c>
+      <c r="AE53" t="n">
+        <v>-0.0800005499204999</v>
+      </c>
+      <c r="AF53" t="n">
+        <v>0.4920255606300718</v>
+      </c>
+      <c r="AG53" t="b">
+        <v>0</v>
+      </c>
     </row>
     <row r="54">
       <c r="A54" t="inlineStr">
@@ -6095,6 +6852,21 @@
       <c r="AB54" t="n">
         <v>-0.5694626283458697</v>
       </c>
+      <c r="AC54" t="n">
+        <v>18</v>
+      </c>
+      <c r="AD54" t="n">
+        <v>-0.280512214878</v>
+      </c>
+      <c r="AE54" t="n">
+        <v>-0.07292970157799999</v>
+      </c>
+      <c r="AF54" t="n">
+        <v>0.2395665827603949</v>
+      </c>
+      <c r="AG54" t="b">
+        <v>0</v>
+      </c>
     </row>
     <row r="55">
       <c r="A55" t="inlineStr">
@@ -6197,6 +6969,21 @@
       <c r="AB55" t="n">
         <v>-0.6653824731851539</v>
       </c>
+      <c r="AC55" t="n">
+        <v>14</v>
+      </c>
+      <c r="AD55" t="n">
+        <v>-0.0006818359853499</v>
+      </c>
+      <c r="AE55" t="n">
+        <v>0.03048334540425</v>
+      </c>
+      <c r="AF55" t="n">
+        <v>1</v>
+      </c>
+      <c r="AG55" t="b">
+        <v>0</v>
+      </c>
     </row>
     <row r="56">
       <c r="A56" t="inlineStr">
@@ -6299,6 +7086,21 @@
       <c r="AB56" t="n">
         <v>-0.6910034810579329</v>
       </c>
+      <c r="AC56" t="n">
+        <v>25</v>
+      </c>
+      <c r="AD56" t="n">
+        <v>-0.265654514286</v>
+      </c>
+      <c r="AE56" t="n">
+        <v>-0.1004546762425</v>
+      </c>
+      <c r="AF56" t="n">
+        <v>0.2350182983032872</v>
+      </c>
+      <c r="AG56" t="b">
+        <v>0</v>
+      </c>
     </row>
     <row r="57">
       <c r="A57" t="inlineStr">
@@ -6405,6 +7207,13 @@
       <c r="AB57" t="n">
         <v>-0.6427048572454059</v>
       </c>
+      <c r="AC57" t="inlineStr"/>
+      <c r="AD57" t="inlineStr"/>
+      <c r="AE57" t="inlineStr"/>
+      <c r="AF57" t="inlineStr"/>
+      <c r="AG57" t="b">
+        <v>0</v>
+      </c>
     </row>
     <row r="58">
       <c r="A58" t="inlineStr">
@@ -6507,6 +7316,21 @@
       <c r="AB58" t="n">
         <v>-0.6479688896188045</v>
       </c>
+      <c r="AC58" t="n">
+        <v>25</v>
+      </c>
+      <c r="AD58" t="n">
+        <v>-0.0652348290771</v>
+      </c>
+      <c r="AE58" t="n">
+        <v>-0.05377081106105</v>
+      </c>
+      <c r="AF58" t="n">
+        <v>0.5248538701707878</v>
+      </c>
+      <c r="AG58" t="b">
+        <v>0</v>
+      </c>
     </row>
     <row r="59">
       <c r="A59" t="inlineStr">
@@ -6609,6 +7433,21 @@
       <c r="AB59" t="n">
         <v>-0.6443710497089925</v>
       </c>
+      <c r="AC59" t="n">
+        <v>35</v>
+      </c>
+      <c r="AD59" t="n">
+        <v>-0.617436224993</v>
+      </c>
+      <c r="AE59" t="n">
+        <v>-0.371163641586</v>
+      </c>
+      <c r="AF59" t="n">
+        <v>1.687217081284497e-06</v>
+      </c>
+      <c r="AG59" t="b">
+        <v>1</v>
+      </c>
     </row>
     <row r="60">
       <c r="A60" t="inlineStr">
@@ -6715,6 +7554,21 @@
       <c r="AB60" t="n">
         <v>-0.5119122545697911</v>
       </c>
+      <c r="AC60" t="n">
+        <v>32</v>
+      </c>
+      <c r="AD60" t="n">
+        <v>-0.2472523245894999</v>
+      </c>
+      <c r="AE60" t="n">
+        <v>-0.1399259291984999</v>
+      </c>
+      <c r="AF60" t="n">
+        <v>0.1007903360365369</v>
+      </c>
+      <c r="AG60" t="b">
+        <v>0</v>
+      </c>
     </row>
     <row r="61">
       <c r="A61" t="inlineStr">
@@ -6817,6 +7671,21 @@
       <c r="AB61" t="n">
         <v>-0.6833663820876426</v>
       </c>
+      <c r="AC61" t="n">
+        <v>25</v>
+      </c>
+      <c r="AD61" t="n">
+        <v>-0.610077451019</v>
+      </c>
+      <c r="AE61" t="n">
+        <v>-0.044181977698</v>
+      </c>
+      <c r="AF61" t="n">
+        <v>0.82738840833081</v>
+      </c>
+      <c r="AG61" t="b">
+        <v>0</v>
+      </c>
     </row>
     <row r="62">
       <c r="A62" t="inlineStr">
@@ -6923,6 +7792,13 @@
       <c r="AB62" t="n">
         <v>-0.6412427632410758</v>
       </c>
+      <c r="AC62" t="inlineStr"/>
+      <c r="AD62" t="inlineStr"/>
+      <c r="AE62" t="inlineStr"/>
+      <c r="AF62" t="inlineStr"/>
+      <c r="AG62" t="b">
+        <v>0</v>
+      </c>
     </row>
     <row r="63">
       <c r="A63" t="inlineStr">
@@ -7025,6 +7901,21 @@
       <c r="AB63" t="n">
         <v>-0.644898374506631</v>
       </c>
+      <c r="AC63" t="n">
+        <v>21</v>
+      </c>
+      <c r="AD63" t="n">
+        <v>-0.0261221007745</v>
+      </c>
+      <c r="AE63" t="n">
+        <v>-0.12010561018175</v>
+      </c>
+      <c r="AF63" t="n">
+        <v>0.1460442504849308</v>
+      </c>
+      <c r="AG63" t="b">
+        <v>0</v>
+      </c>
     </row>
     <row r="64">
       <c r="A64" t="inlineStr">
@@ -7131,6 +8022,21 @@
       <c r="AB64" t="n">
         <v>-0.486816425253434</v>
       </c>
+      <c r="AC64" t="n">
+        <v>5</v>
+      </c>
+      <c r="AD64" t="n">
+        <v>-0.367136619132</v>
+      </c>
+      <c r="AE64" t="n">
+        <v>-0.255540380586</v>
+      </c>
+      <c r="AF64" t="n">
+        <v>0.1082651935270724</v>
+      </c>
+      <c r="AG64" t="b">
+        <v>0</v>
+      </c>
     </row>
     <row r="65">
       <c r="A65" t="inlineStr">
@@ -7237,6 +8143,21 @@
       <c r="AB65" t="n">
         <v>-0.55992627118602</v>
       </c>
+      <c r="AC65" t="n">
+        <v>38</v>
+      </c>
+      <c r="AD65" t="n">
+        <v>0.0528174952845</v>
+      </c>
+      <c r="AE65" t="n">
+        <v>-0.0336521796372999</v>
+      </c>
+      <c r="AF65" t="n">
+        <v>0.5067175097180633</v>
+      </c>
+      <c r="AG65" t="b">
+        <v>0</v>
+      </c>
     </row>
     <row r="66">
       <c r="A66" t="inlineStr">
@@ -7343,6 +8264,21 @@
       <c r="AB66" t="n">
         <v>-0.4266221884265064</v>
       </c>
+      <c r="AC66" t="n">
+        <v>48</v>
+      </c>
+      <c r="AD66" t="n">
+        <v>-0.3028122728819999</v>
+      </c>
+      <c r="AE66" t="n">
+        <v>-0.0954147164859999</v>
+      </c>
+      <c r="AF66" t="n">
+        <v>0.8765247489113656</v>
+      </c>
+      <c r="AG66" t="b">
+        <v>0</v>
+      </c>
     </row>
     <row r="67">
       <c r="A67" t="inlineStr">
@@ -7445,6 +8381,21 @@
       <c r="AB67" t="n">
         <v>-0.5992384677954098</v>
       </c>
+      <c r="AC67" t="n">
+        <v>25</v>
+      </c>
+      <c r="AD67" t="n">
+        <v>-0.45211730827</v>
+      </c>
+      <c r="AE67" t="n">
+        <v>-0.0564342156425</v>
+      </c>
+      <c r="AF67" t="n">
+        <v>0.4285135595374503</v>
+      </c>
+      <c r="AG67" t="b">
+        <v>0</v>
+      </c>
     </row>
     <row r="68">
       <c r="A68" t="inlineStr">
@@ -7551,6 +8502,21 @@
       <c r="AB68" t="n">
         <v>-0.5018031372424157</v>
       </c>
+      <c r="AC68" t="n">
+        <v>20</v>
+      </c>
+      <c r="AD68" t="n">
+        <v>-0.320074420485</v>
+      </c>
+      <c r="AE68" t="n">
+        <v>-0.115636263893</v>
+      </c>
+      <c r="AF68" t="n">
+        <v>0.0449411757623897</v>
+      </c>
+      <c r="AG68" t="b">
+        <v>1</v>
+      </c>
     </row>
     <row r="69">
       <c r="A69" t="inlineStr">
@@ -7653,6 +8619,21 @@
       <c r="AB69" t="n">
         <v>-0.6271927275497802</v>
       </c>
+      <c r="AC69" t="n">
+        <v>25</v>
+      </c>
+      <c r="AD69" t="n">
+        <v>-0.18429861025</v>
+      </c>
+      <c r="AE69" t="n">
+        <v>-0.08712639498874999</v>
+      </c>
+      <c r="AF69" t="n">
+        <v>0.9206771991228559</v>
+      </c>
+      <c r="AG69" t="b">
+        <v>0</v>
+      </c>
     </row>
     <row r="70">
       <c r="A70" t="inlineStr">
@@ -7755,6 +8736,21 @@
       <c r="AB70" t="n">
         <v>-0.5898868424969386</v>
       </c>
+      <c r="AC70" t="n">
+        <v>25</v>
+      </c>
+      <c r="AD70" t="n">
+        <v>-0.355756171858</v>
+      </c>
+      <c r="AE70" t="n">
+        <v>-0.0340363046559999</v>
+      </c>
+      <c r="AF70" t="n">
+        <v>0.8093837764468539</v>
+      </c>
+      <c r="AG70" t="b">
+        <v>0</v>
+      </c>
     </row>
     <row r="71">
       <c r="A71" t="inlineStr">
@@ -7861,6 +8857,21 @@
       <c r="AB71" t="n">
         <v>-0.4829674976065112</v>
       </c>
+      <c r="AC71" t="n">
+        <v>30</v>
+      </c>
+      <c r="AD71" t="n">
+        <v>-0.2387476415505</v>
+      </c>
+      <c r="AE71" t="n">
+        <v>-0.0311651282504999</v>
+      </c>
+      <c r="AF71" t="n">
+        <v>0.7312175116270664</v>
+      </c>
+      <c r="AG71" t="b">
+        <v>0</v>
+      </c>
     </row>
     <row r="72">
       <c r="A72" t="inlineStr">
@@ -7967,6 +8978,21 @@
       <c r="AB72" t="n">
         <v>-0.5809887624308736</v>
       </c>
+      <c r="AC72" t="n">
+        <v>11</v>
+      </c>
+      <c r="AD72" t="n">
+        <v>-0.0612493949165</v>
+      </c>
+      <c r="AE72" t="n">
+        <v>-0.2003053143665</v>
+      </c>
+      <c r="AF72" t="n">
+        <v>0.1270973663551465</v>
+      </c>
+      <c r="AG72" t="b">
+        <v>0</v>
+      </c>
     </row>
     <row r="73">
       <c r="A73" t="inlineStr">
@@ -8073,6 +9099,21 @@
       <c r="AB73" t="n">
         <v>-0.4175859915536748</v>
       </c>
+      <c r="AC73" t="n">
+        <v>32</v>
+      </c>
+      <c r="AD73" t="n">
+        <v>-0.3175561580785</v>
+      </c>
+      <c r="AE73" t="n">
+        <v>-0.1127117610025</v>
+      </c>
+      <c r="AF73" t="n">
+        <v>0.2672931533651203</v>
+      </c>
+      <c r="AG73" t="b">
+        <v>0</v>
+      </c>
     </row>
     <row r="74">
       <c r="A74" t="inlineStr">
@@ -8175,6 +9216,21 @@
       <c r="AB74" t="n">
         <v>-0.6075948579839998</v>
       </c>
+      <c r="AC74" t="n">
+        <v>21</v>
+      </c>
+      <c r="AD74" t="n">
+        <v>-0.0120882335513</v>
+      </c>
+      <c r="AE74" t="n">
+        <v>0.0053141426217999</v>
+      </c>
+      <c r="AF74" t="n">
+        <v>1</v>
+      </c>
+      <c r="AG74" t="b">
+        <v>0</v>
+      </c>
     </row>
     <row r="75">
       <c r="A75" t="inlineStr">
@@ -8281,6 +9337,21 @@
       <c r="AB75" t="n">
         <v>-0.5691540206146471</v>
       </c>
+      <c r="AC75" t="n">
+        <v>44</v>
+      </c>
+      <c r="AD75" t="n">
+        <v>-0.0333988888443</v>
+      </c>
+      <c r="AE75" t="n">
+        <v>-0.0250535125772849</v>
+      </c>
+      <c r="AF75" t="n">
+        <v>0.2488610196540167</v>
+      </c>
+      <c r="AG75" t="b">
+        <v>0</v>
+      </c>
     </row>
     <row r="76">
       <c r="A76" t="inlineStr">
@@ -8383,6 +9454,21 @@
       <c r="AB76" t="n">
         <v>-0.6334569158062046</v>
       </c>
+      <c r="AC76" t="n">
+        <v>21</v>
+      </c>
+      <c r="AD76" t="n">
+        <v>-3.06717053112e-05</v>
+      </c>
+      <c r="AE76" t="n">
+        <v>-0.1290431923988112</v>
+      </c>
+      <c r="AF76" t="n">
+        <v>0.0139595536418847</v>
+      </c>
+      <c r="AG76" t="b">
+        <v>1</v>
+      </c>
     </row>
     <row r="77">
       <c r="A77" t="inlineStr">
@@ -8485,6 +9571,13 @@
       <c r="AB77" t="n">
         <v>-0.5825202649451341</v>
       </c>
+      <c r="AC77" t="inlineStr"/>
+      <c r="AD77" t="inlineStr"/>
+      <c r="AE77" t="inlineStr"/>
+      <c r="AF77" t="inlineStr"/>
+      <c r="AG77" t="b">
+        <v>0</v>
+      </c>
     </row>
     <row r="78">
       <c r="A78" t="inlineStr">
@@ -8587,6 +9680,21 @@
       <c r="AB78" t="n">
         <v>-0.5709986819612969</v>
       </c>
+      <c r="AC78" t="n">
+        <v>25</v>
+      </c>
+      <c r="AD78" t="n">
+        <v>-0.806502908258</v>
+      </c>
+      <c r="AE78" t="n">
+        <v>-0.5739256359145</v>
+      </c>
+      <c r="AF78" t="n">
+        <v>4.880381313946173e-06</v>
+      </c>
+      <c r="AG78" t="b">
+        <v>1</v>
+      </c>
     </row>
     <row r="79">
       <c r="A79" t="inlineStr">
@@ -8689,6 +9797,21 @@
       <c r="AB79" t="n">
         <v>-0.5793128756550876</v>
       </c>
+      <c r="AC79" t="n">
+        <v>35</v>
+      </c>
+      <c r="AD79" t="n">
+        <v>0.0463590077088</v>
+      </c>
+      <c r="AE79" t="n">
+        <v>0.0569307739236</v>
+      </c>
+      <c r="AF79" t="n">
+        <v>1</v>
+      </c>
+      <c r="AG79" t="b">
+        <v>0</v>
+      </c>
     </row>
     <row r="80">
       <c r="A80" t="inlineStr">
@@ -8795,6 +9918,13 @@
       <c r="AB80" t="n">
         <v>-0.557999846716411</v>
       </c>
+      <c r="AC80" t="inlineStr"/>
+      <c r="AD80" t="inlineStr"/>
+      <c r="AE80" t="inlineStr"/>
+      <c r="AF80" t="inlineStr"/>
+      <c r="AG80" t="b">
+        <v>0</v>
+      </c>
     </row>
     <row r="81">
       <c r="A81" t="inlineStr">
@@ -8897,6 +10027,21 @@
       <c r="AB81" t="n">
         <v>-0.5907005201326848</v>
       </c>
+      <c r="AC81" t="n">
+        <v>25</v>
+      </c>
+      <c r="AD81" t="n">
+        <v>-0.260110071114</v>
+      </c>
+      <c r="AE81" t="n">
+        <v>-0.1269716404524999</v>
+      </c>
+      <c r="AF81" t="n">
+        <v>0.0581305131456747</v>
+      </c>
+      <c r="AG81" t="b">
+        <v>0</v>
+      </c>
     </row>
     <row r="82">
       <c r="A82" t="inlineStr">
@@ -9003,6 +10148,13 @@
       <c r="AB82" t="n">
         <v>-0.5490552745799622</v>
       </c>
+      <c r="AC82" t="inlineStr"/>
+      <c r="AD82" t="inlineStr"/>
+      <c r="AE82" t="inlineStr"/>
+      <c r="AF82" t="inlineStr"/>
+      <c r="AG82" t="b">
+        <v>0</v>
+      </c>
     </row>
     <row r="83">
       <c r="A83" t="inlineStr">
@@ -9109,6 +10261,21 @@
       <c r="AB83" t="n">
         <v>-0.4329038982552768</v>
       </c>
+      <c r="AC83" t="n">
+        <v>20</v>
+      </c>
+      <c r="AD83" t="n">
+        <v>-0.2439922061815</v>
+      </c>
+      <c r="AE83" t="n">
+        <v>-0.131450956184</v>
+      </c>
+      <c r="AF83" t="n">
+        <v>0.2605525109645124</v>
+      </c>
+      <c r="AG83" t="b">
+        <v>0</v>
+      </c>
     </row>
     <row r="84">
       <c r="A84" t="inlineStr">
@@ -9215,6 +10382,21 @@
       <c r="AB84" t="n">
         <v>-0.5434854187372423</v>
       </c>
+      <c r="AC84" t="n">
+        <v>31</v>
+      </c>
+      <c r="AD84" t="n">
+        <v>-0.345979715204</v>
+      </c>
+      <c r="AE84" t="n">
+        <v>-0.1610288049535</v>
+      </c>
+      <c r="AF84" t="n">
+        <v>0.0116686999347966</v>
+      </c>
+      <c r="AG84" t="b">
+        <v>1</v>
+      </c>
     </row>
     <row r="85">
       <c r="A85" t="inlineStr">
@@ -9317,6 +10499,21 @@
       <c r="AB85" t="n">
         <v>-0.5541170994409248</v>
       </c>
+      <c r="AC85" t="n">
+        <v>25</v>
+      </c>
+      <c r="AD85" t="n">
+        <v>-0.555531353466</v>
+      </c>
+      <c r="AE85" t="n">
+        <v>-0.19374070244</v>
+      </c>
+      <c r="AF85" t="n">
+        <v>0.0419983086835975</v>
+      </c>
+      <c r="AG85" t="b">
+        <v>1</v>
+      </c>
     </row>
     <row r="86">
       <c r="A86" t="inlineStr">
@@ -9423,6 +10620,21 @@
       <c r="AB86" t="n">
         <v>-0.4659543924848717</v>
       </c>
+      <c r="AC86" t="n">
+        <v>18</v>
+      </c>
+      <c r="AD86" t="n">
+        <v>-0.07436234298204999</v>
+      </c>
+      <c r="AE86" t="n">
+        <v>0.00144607521335</v>
+      </c>
+      <c r="AF86" t="n">
+        <v>1</v>
+      </c>
+      <c r="AG86" t="b">
+        <v>0</v>
+      </c>
     </row>
     <row r="87">
       <c r="A87" t="inlineStr">
@@ -9529,6 +10741,21 @@
       <c r="AB87" t="n">
         <v>-0.5238564368019141</v>
       </c>
+      <c r="AC87" t="n">
+        <v>30</v>
+      </c>
+      <c r="AD87" t="n">
+        <v>-0.275352354099</v>
+      </c>
+      <c r="AE87" t="n">
+        <v>-0.09759208049199999</v>
+      </c>
+      <c r="AF87" t="n">
+        <v>0.2590426996636222</v>
+      </c>
+      <c r="AG87" t="b">
+        <v>0</v>
+      </c>
     </row>
     <row r="88">
       <c r="A88" t="inlineStr">
@@ -9635,6 +10862,13 @@
       <c r="AB88" t="n">
         <v>-0.5197542792992306</v>
       </c>
+      <c r="AC88" t="inlineStr"/>
+      <c r="AD88" t="inlineStr"/>
+      <c r="AE88" t="inlineStr"/>
+      <c r="AF88" t="inlineStr"/>
+      <c r="AG88" t="b">
+        <v>0</v>
+      </c>
     </row>
     <row r="89">
       <c r="A89" t="inlineStr">
@@ -9737,6 +10971,21 @@
       <c r="AB89" t="n">
         <v>-0.5326815806970289</v>
       </c>
+      <c r="AC89" t="n">
+        <v>35</v>
+      </c>
+      <c r="AD89" t="n">
+        <v>-0.336948941277</v>
+      </c>
+      <c r="AE89" t="n">
+        <v>-0.2617517219281</v>
+      </c>
+      <c r="AF89" t="n">
+        <v>0.000457973393415</v>
+      </c>
+      <c r="AG89" t="b">
+        <v>1</v>
+      </c>
     </row>
     <row r="90">
       <c r="A90" t="inlineStr">
@@ -9839,6 +11088,21 @@
       <c r="AB90" t="n">
         <v>-0.524422411281307</v>
       </c>
+      <c r="AC90" t="n">
+        <v>35</v>
+      </c>
+      <c r="AD90" t="n">
+        <v>-0.639197272786</v>
+      </c>
+      <c r="AE90" t="n">
+        <v>-0.287709354222</v>
+      </c>
+      <c r="AF90" t="n">
+        <v>2.07912848719522e-06</v>
+      </c>
+      <c r="AG90" t="b">
+        <v>1</v>
+      </c>
     </row>
     <row r="91">
       <c r="A91" t="inlineStr">
@@ -9941,6 +11205,21 @@
       <c r="AB91" t="n">
         <v>-0.5419115711284188</v>
       </c>
+      <c r="AC91" t="n">
+        <v>21</v>
+      </c>
+      <c r="AD91" t="n">
+        <v>-0.375844723301</v>
+      </c>
+      <c r="AE91" t="n">
+        <v>0.0226837776155</v>
+      </c>
+      <c r="AF91" t="n">
+        <v>0.8521893311806578</v>
+      </c>
+      <c r="AG91" t="b">
+        <v>0</v>
+      </c>
     </row>
     <row r="92">
       <c r="A92" t="inlineStr">
@@ -10047,6 +11326,21 @@
       <c r="AB92" t="n">
         <v>-0.5120978512924145</v>
       </c>
+      <c r="AC92" t="n">
+        <v>47</v>
+      </c>
+      <c r="AD92" t="n">
+        <v>-0.27460803094</v>
+      </c>
+      <c r="AE92" t="n">
+        <v>-0.140219236027</v>
+      </c>
+      <c r="AF92" t="n">
+        <v>0.0021314325680103</v>
+      </c>
+      <c r="AG92" t="b">
+        <v>1</v>
+      </c>
     </row>
     <row r="93">
       <c r="A93" t="inlineStr">
@@ -10153,6 +11447,21 @@
       <c r="AB93" t="n">
         <v>-0.543504133826032</v>
       </c>
+      <c r="AC93" t="n">
+        <v>31</v>
+      </c>
+      <c r="AD93" t="n">
+        <v>-0.563627372559</v>
+      </c>
+      <c r="AE93" t="n">
+        <v>-0.071262988571</v>
+      </c>
+      <c r="AF93" t="n">
+        <v>0.2687944170079644</v>
+      </c>
+      <c r="AG93" t="b">
+        <v>0</v>
+      </c>
     </row>
     <row r="94">
       <c r="A94" t="inlineStr">
@@ -10259,6 +11568,13 @@
       <c r="AB94" t="n">
         <v>-0.4855774995215112</v>
       </c>
+      <c r="AC94" t="inlineStr"/>
+      <c r="AD94" t="inlineStr"/>
+      <c r="AE94" t="inlineStr"/>
+      <c r="AF94" t="inlineStr"/>
+      <c r="AG94" t="b">
+        <v>0</v>
+      </c>
     </row>
     <row r="95">
       <c r="A95" t="inlineStr">
@@ -10364,6 +11680,21 @@
       </c>
       <c r="AB95" t="n">
         <v>-0.6150292625587572</v>
+      </c>
+      <c r="AC95" t="n">
+        <v>74</v>
+      </c>
+      <c r="AD95" t="n">
+        <v>-0.4874507911125</v>
+      </c>
+      <c r="AE95" t="n">
+        <v>-0.190430881344</v>
+      </c>
+      <c r="AF95" t="n">
+        <v>0.0057281527614398</v>
+      </c>
+      <c r="AG95" t="b">
+        <v>1</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
S2 Table: RNAi column marks pairs that could not be tested
Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/figures/supporting_information/S2_Table.xlsx
+++ b/figures/supporting_information/S2_Table.xlsx
@@ -1188,8 +1188,10 @@
       <c r="AD6" t="inlineStr"/>
       <c r="AE6" t="inlineStr"/>
       <c r="AF6" t="inlineStr"/>
-      <c r="AG6" t="b">
-        <v>0</v>
+      <c r="AG6" t="inlineStr">
+        <is>
+          <t>not testable</t>
+        </is>
       </c>
     </row>
     <row r="7">
@@ -1777,8 +1779,10 @@
       <c r="AD11" t="inlineStr"/>
       <c r="AE11" t="inlineStr"/>
       <c r="AF11" t="inlineStr"/>
-      <c r="AG11" t="b">
-        <v>0</v>
+      <c r="AG11" t="inlineStr">
+        <is>
+          <t>not testable</t>
+        </is>
       </c>
     </row>
     <row r="12">
@@ -2132,8 +2136,10 @@
       <c r="AD14" t="inlineStr"/>
       <c r="AE14" t="inlineStr"/>
       <c r="AF14" t="inlineStr"/>
-      <c r="AG14" t="b">
-        <v>0</v>
+      <c r="AG14" t="inlineStr">
+        <is>
+          <t>not testable</t>
+        </is>
       </c>
     </row>
     <row r="15">
@@ -2721,8 +2727,10 @@
       <c r="AD19" t="inlineStr"/>
       <c r="AE19" t="inlineStr"/>
       <c r="AF19" t="inlineStr"/>
-      <c r="AG19" t="b">
-        <v>0</v>
+      <c r="AG19" t="inlineStr">
+        <is>
+          <t>not testable</t>
+        </is>
       </c>
     </row>
     <row r="20">
@@ -3076,8 +3084,10 @@
       <c r="AD22" t="inlineStr"/>
       <c r="AE22" t="inlineStr"/>
       <c r="AF22" t="inlineStr"/>
-      <c r="AG22" t="b">
-        <v>0</v>
+      <c r="AG22" t="inlineStr">
+        <is>
+          <t>not testable</t>
+        </is>
       </c>
     </row>
     <row r="23">
@@ -5557,8 +5567,10 @@
       <c r="AD43" t="inlineStr"/>
       <c r="AE43" t="inlineStr"/>
       <c r="AF43" t="inlineStr"/>
-      <c r="AG43" t="b">
-        <v>0</v>
+      <c r="AG43" t="inlineStr">
+        <is>
+          <t>not testable</t>
+        </is>
       </c>
     </row>
     <row r="44">
@@ -7211,8 +7223,10 @@
       <c r="AD57" t="inlineStr"/>
       <c r="AE57" t="inlineStr"/>
       <c r="AF57" t="inlineStr"/>
-      <c r="AG57" t="b">
-        <v>0</v>
+      <c r="AG57" t="inlineStr">
+        <is>
+          <t>not testable</t>
+        </is>
       </c>
     </row>
     <row r="58">
@@ -7796,8 +7810,10 @@
       <c r="AD62" t="inlineStr"/>
       <c r="AE62" t="inlineStr"/>
       <c r="AF62" t="inlineStr"/>
-      <c r="AG62" t="b">
-        <v>0</v>
+      <c r="AG62" t="inlineStr">
+        <is>
+          <t>not testable</t>
+        </is>
       </c>
     </row>
     <row r="63">
@@ -9575,8 +9591,10 @@
       <c r="AD77" t="inlineStr"/>
       <c r="AE77" t="inlineStr"/>
       <c r="AF77" t="inlineStr"/>
-      <c r="AG77" t="b">
-        <v>0</v>
+      <c r="AG77" t="inlineStr">
+        <is>
+          <t>not testable</t>
+        </is>
       </c>
     </row>
     <row r="78">
@@ -9922,8 +9940,10 @@
       <c r="AD80" t="inlineStr"/>
       <c r="AE80" t="inlineStr"/>
       <c r="AF80" t="inlineStr"/>
-      <c r="AG80" t="b">
-        <v>0</v>
+      <c r="AG80" t="inlineStr">
+        <is>
+          <t>not testable</t>
+        </is>
       </c>
     </row>
     <row r="81">
@@ -10152,8 +10172,10 @@
       <c r="AD82" t="inlineStr"/>
       <c r="AE82" t="inlineStr"/>
       <c r="AF82" t="inlineStr"/>
-      <c r="AG82" t="b">
-        <v>0</v>
+      <c r="AG82" t="inlineStr">
+        <is>
+          <t>not testable</t>
+        </is>
       </c>
     </row>
     <row r="83">
@@ -10866,8 +10888,10 @@
       <c r="AD88" t="inlineStr"/>
       <c r="AE88" t="inlineStr"/>
       <c r="AF88" t="inlineStr"/>
-      <c r="AG88" t="b">
-        <v>0</v>
+      <c r="AG88" t="inlineStr">
+        <is>
+          <t>not testable</t>
+        </is>
       </c>
     </row>
     <row r="89">
@@ -11572,8 +11596,10 @@
       <c r="AD94" t="inlineStr"/>
       <c r="AE94" t="inlineStr"/>
       <c r="AF94" t="inlineStr"/>
-      <c r="AG94" t="b">
-        <v>0</v>
+      <c r="AG94" t="inlineStr">
+        <is>
+          <t>not testable</t>
+        </is>
       </c>
     </row>
     <row r="95">

</xml_diff>

<commit_message>
rnai_validation.py: exclude multi-gene entries before BH, Fisher test high vs other tiers, sample_info not needed; S2 column names
Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/figures/supporting_information/S2_Table.xlsx
+++ b/figures/supporting_information/S2_Table.xlsx
@@ -481,7 +481,7 @@
       </c>
       <c r="K1" s="1" t="inlineStr">
         <is>
-          <t>confidence_flag</t>
+          <t>Low-n flag (fewer than 10 target lines)</t>
         </is>
       </c>
       <c r="L1" s="1" t="inlineStr">
@@ -561,7 +561,7 @@
       </c>
       <c r="AA1" s="1" t="inlineStr">
         <is>
-          <t>Evidence: independent replication (Project Score)</t>
+          <t>Evidence: re-prioritised in the discovery cohort and replicated in Project Score</t>
         </is>
       </c>
       <c r="AB1" s="1" t="inlineStr">
@@ -710,7 +710,7 @@
         <v>-0.6770184262954999</v>
       </c>
       <c r="AF2" t="n">
-        <v>1.07355091345946e-10</v>
+        <v>1.058558278623814e-10</v>
       </c>
       <c r="AG2" t="b">
         <v>1</v>
@@ -831,7 +831,7 @@
         <v>-0.66765903132215</v>
       </c>
       <c r="AF3" t="n">
-        <v>1.203768181296743e-13</v>
+        <v>1.18695700211308e-13</v>
       </c>
       <c r="AG3" t="b">
         <v>1</v>
@@ -952,7 +952,7 @@
         <v>-0.6370989342779</v>
       </c>
       <c r="AF4" t="n">
-        <v>3.944109540741884e-06</v>
+        <v>3.95725679294141e-06</v>
       </c>
       <c r="AG4" t="b">
         <v>1</v>
@@ -1073,7 +1073,7 @@
         <v>-0.5059126675251</v>
       </c>
       <c r="AF5" t="n">
-        <v>0.0094071474978044</v>
+        <v>0.009372982929631001</v>
       </c>
       <c r="AG5" t="b">
         <v>1</v>
@@ -1309,7 +1309,7 @@
         <v>-1.4186712161405</v>
       </c>
       <c r="AF7" t="n">
-        <v>6.973581087284193e-16</v>
+        <v>6.876191803340964e-16</v>
       </c>
       <c r="AG7" t="b">
         <v>1</v>
@@ -1430,7 +1430,7 @@
         <v>-0.218886220542</v>
       </c>
       <c r="AF8" t="n">
-        <v>0.09940649233118209</v>
+        <v>0.0991184314769991</v>
       </c>
       <c r="AG8" t="b">
         <v>0</v>
@@ -1547,7 +1547,7 @@
         <v>-0.6955904556900501</v>
       </c>
       <c r="AF9" t="n">
-        <v>1.22585880086157e-11</v>
+        <v>1.208739115962644e-11</v>
       </c>
       <c r="AG9" t="b">
         <v>1</v>
@@ -1664,7 +1664,7 @@
         <v>-0.66306432792573</v>
       </c>
       <c r="AF10" t="n">
-        <v>3.14609244905087e-10</v>
+        <v>3.102155813483391e-10</v>
       </c>
       <c r="AG10" t="b">
         <v>1</v>
@@ -1900,7 +1900,7 @@
         <v>-0.4531535384439999</v>
       </c>
       <c r="AF12" t="n">
-        <v>2.952616087655184e-09</v>
+        <v>2.911381438923511e-09</v>
       </c>
       <c r="AG12" t="b">
         <v>1</v>
@@ -2021,7 +2021,7 @@
         <v>-0.7480611459936151</v>
       </c>
       <c r="AF13" t="n">
-        <v>1.051333992974078e-12</v>
+        <v>1.036651627704443e-12</v>
       </c>
       <c r="AG13" t="b">
         <v>1</v>
@@ -2253,7 +2253,7 @@
         <v>-0.06294062613665</v>
       </c>
       <c r="AF15" t="n">
-        <v>0.6754463501916057</v>
+        <v>0.6751706000764186</v>
       </c>
       <c r="AG15" t="b">
         <v>0</v>
@@ -2370,7 +2370,7 @@
         <v>-0.22483615498405</v>
       </c>
       <c r="AF16" t="n">
-        <v>1.142024211032387e-08</v>
+        <v>1.126075314939233e-08</v>
       </c>
       <c r="AG16" t="b">
         <v>1</v>
@@ -2491,7 +2491,7 @@
         <v>-0.8968104558529999</v>
       </c>
       <c r="AF17" t="n">
-        <v>0.0012293943732588</v>
+        <v>0.001228342268178</v>
       </c>
       <c r="AG17" t="b">
         <v>1</v>
@@ -2612,7 +2612,7 @@
         <v>-0.3640232577259999</v>
       </c>
       <c r="AF18" t="n">
-        <v>0.0002857162094531</v>
+        <v>0.0002861978925657</v>
       </c>
       <c r="AG18" t="b">
         <v>1</v>
@@ -2848,7 +2848,7 @@
         <v>-0.462016267625</v>
       </c>
       <c r="AF20" t="n">
-        <v>6.867916923524099e-05</v>
+        <v>6.926413786913311e-05</v>
       </c>
       <c r="AG20" t="b">
         <v>1</v>
@@ -2969,7 +2969,7 @@
         <v>-0.39305793268485</v>
       </c>
       <c r="AF21" t="n">
-        <v>0.4397213776505249</v>
+        <v>0.4391951634532907</v>
       </c>
       <c r="AG21" t="b">
         <v>0</v>
@@ -3205,7 +3205,7 @@
         <v>-0.4452628291852</v>
       </c>
       <c r="AF23" t="n">
-        <v>0.0001866365310995</v>
+        <v>0.000187480629387</v>
       </c>
       <c r="AG23" t="b">
         <v>1</v>
@@ -3322,7 +3322,7 @@
         <v>-0.02792919759184</v>
       </c>
       <c r="AF24" t="n">
-        <v>0.2986652126343077</v>
+        <v>0.298050688006109</v>
       </c>
       <c r="AG24" t="b">
         <v>0</v>
@@ -3439,7 +3439,7 @@
         <v>-0.1442039907944</v>
       </c>
       <c r="AF25" t="n">
-        <v>0.0171163661506576</v>
+        <v>0.0170509802623703</v>
       </c>
       <c r="AG25" t="b">
         <v>1</v>
@@ -3556,7 +3556,7 @@
         <v>-0.189546274989</v>
       </c>
       <c r="AF26" t="n">
-        <v>0.0502625644887586</v>
+        <v>0.0501361754355637</v>
       </c>
       <c r="AG26" t="b">
         <v>0</v>
@@ -3794,7 +3794,7 @@
         <v>-0.05063221455227</v>
       </c>
       <c r="AF28" t="n">
-        <v>0.3222360544805334</v>
+        <v>0.3215658854459068</v>
       </c>
       <c r="AG28" t="b">
         <v>0</v>
@@ -3911,7 +3911,7 @@
         <v>-0.0145622134985499</v>
       </c>
       <c r="AF29" t="n">
-        <v>0.6853664252519956</v>
+        <v>0.6851340982661516</v>
       </c>
       <c r="AG29" t="b">
         <v>0</v>
@@ -4149,7 +4149,7 @@
         <v>-0.1688276451951</v>
       </c>
       <c r="AF31" t="n">
-        <v>0.0010066982974493</v>
+        <v>0.0010050214851933</v>
       </c>
       <c r="AG31" t="b">
         <v>1</v>
@@ -4270,7 +4270,7 @@
         <v>-0.2812998829699999</v>
       </c>
       <c r="AF32" t="n">
-        <v>6.455073790426178e-05</v>
+        <v>6.515447592170636e-05</v>
       </c>
       <c r="AG32" t="b">
         <v>1</v>
@@ -4387,7 +4387,7 @@
         <v>-0.0711168508259999</v>
       </c>
       <c r="AF33" t="n">
-        <v>0.5215960393226162</v>
+        <v>0.5211835554144526</v>
       </c>
       <c r="AG33" t="b">
         <v>0</v>
@@ -4504,7 +4504,7 @@
         <v>-0.0522154659394999</v>
       </c>
       <c r="AF34" t="n">
-        <v>0.292293207802129</v>
+        <v>0.2917154953964482</v>
       </c>
       <c r="AG34" t="b">
         <v>0</v>
@@ -4621,7 +4621,7 @@
         <v>-0.09264280502900001</v>
       </c>
       <c r="AF35" t="n">
-        <v>0.0467332025525786</v>
+        <v>0.0466207037541857</v>
       </c>
       <c r="AG35" t="b">
         <v>1</v>
@@ -4738,7 +4738,7 @@
         <v>-0.092751146469</v>
       </c>
       <c r="AF36" t="n">
-        <v>0.6847871497545607</v>
+        <v>0.6845601799122838</v>
       </c>
       <c r="AG36" t="b">
         <v>0</v>
@@ -4859,7 +4859,7 @@
         <v>-0.294173121605</v>
       </c>
       <c r="AF37" t="n">
-        <v>0.0012190304751744</v>
+        <v>0.0012180788215966</v>
       </c>
       <c r="AG37" t="b">
         <v>1</v>
@@ -5210,7 +5210,7 @@
         <v>-0.35171071011765</v>
       </c>
       <c r="AF40" t="n">
-        <v>2.068007602419394e-06</v>
+        <v>2.061534908294088e-06</v>
       </c>
       <c r="AG40" t="b">
         <v>1</v>
@@ -5331,7 +5331,7 @@
         <v>-0.2090858874085</v>
       </c>
       <c r="AF41" t="n">
-        <v>0.210816233115083</v>
+        <v>0.2102015638717295</v>
       </c>
       <c r="AG41" t="b">
         <v>0</v>
@@ -5452,7 +5452,7 @@
         <v>-0.217096837904</v>
       </c>
       <c r="AF42" t="n">
-        <v>0.0525555149851436</v>
+        <v>0.052406707569596</v>
       </c>
       <c r="AG42" t="b">
         <v>0</v>
@@ -5684,7 +5684,7 @@
         <v>-0.1797593753399999</v>
       </c>
       <c r="AF44" t="n">
-        <v>0.1006053061546971</v>
+        <v>0.1003266999991317</v>
       </c>
       <c r="AG44" t="b">
         <v>0</v>
@@ -5926,7 +5926,7 @@
         <v>-0.1951922491984999</v>
       </c>
       <c r="AF46" t="n">
-        <v>0.0018158748052098</v>
+        <v>0.0018114162305374</v>
       </c>
       <c r="AG46" t="b">
         <v>1</v>
@@ -6164,7 +6164,7 @@
         <v>-0.034824478637</v>
       </c>
       <c r="AF48" t="n">
-        <v>0.5634748184963327</v>
+        <v>0.5630929028545996</v>
       </c>
       <c r="AG48" t="b">
         <v>0</v>
@@ -6398,7 +6398,7 @@
         <v>-0.2104751638845</v>
       </c>
       <c r="AF50" t="n">
-        <v>2.159259261715311e-05</v>
+        <v>2.164589277977178e-05</v>
       </c>
       <c r="AG50" t="b">
         <v>1</v>
@@ -6515,7 +6515,7 @@
         <v>-0.159675398326</v>
       </c>
       <c r="AF51" t="n">
-        <v>0.5236754523565743</v>
+        <v>0.5232443451432316</v>
       </c>
       <c r="AG51" t="b">
         <v>0</v>
@@ -6636,7 +6636,7 @@
         <v>-0.136727396118</v>
       </c>
       <c r="AF52" t="n">
-        <v>0.1314240485531233</v>
+        <v>0.1310261244486585</v>
       </c>
       <c r="AG52" t="b">
         <v>0</v>
@@ -6753,7 +6753,7 @@
         <v>-0.0800005499204999</v>
       </c>
       <c r="AF53" t="n">
-        <v>0.4920255606300718</v>
+        <v>0.4915206088287679</v>
       </c>
       <c r="AG53" t="b">
         <v>0</v>
@@ -6874,7 +6874,7 @@
         <v>-0.07292970157799999</v>
       </c>
       <c r="AF54" t="n">
-        <v>0.2395665827603949</v>
+        <v>0.2390204333848072</v>
       </c>
       <c r="AG54" t="b">
         <v>0</v>
@@ -7108,7 +7108,7 @@
         <v>-0.1004546762425</v>
       </c>
       <c r="AF56" t="n">
-        <v>0.2350182983032872</v>
+        <v>0.2344077814339213</v>
       </c>
       <c r="AG56" t="b">
         <v>0</v>
@@ -7340,7 +7340,7 @@
         <v>-0.05377081106105</v>
       </c>
       <c r="AF58" t="n">
-        <v>0.5248538701707878</v>
+        <v>0.5244223820183999</v>
       </c>
       <c r="AG58" t="b">
         <v>0</v>
@@ -7457,7 +7457,7 @@
         <v>-0.371163641586</v>
       </c>
       <c r="AF59" t="n">
-        <v>1.687217081284497e-06</v>
+        <v>1.682999132314917e-06</v>
       </c>
       <c r="AG59" t="b">
         <v>1</v>
@@ -7578,7 +7578,7 @@
         <v>-0.1399259291984999</v>
       </c>
       <c r="AF60" t="n">
-        <v>0.1007903360365369</v>
+        <v>0.1005173119275306</v>
       </c>
       <c r="AG60" t="b">
         <v>0</v>
@@ -7695,7 +7695,7 @@
         <v>-0.044181977698</v>
       </c>
       <c r="AF61" t="n">
-        <v>0.82738840833081</v>
+        <v>0.8273721640177254</v>
       </c>
       <c r="AG61" t="b">
         <v>0</v>
@@ -7927,7 +7927,7 @@
         <v>-0.12010561018175</v>
       </c>
       <c r="AF63" t="n">
-        <v>0.1460442504849308</v>
+        <v>0.1456150863225919</v>
       </c>
       <c r="AG63" t="b">
         <v>0</v>
@@ -8048,7 +8048,7 @@
         <v>-0.255540380586</v>
       </c>
       <c r="AF64" t="n">
-        <v>0.1082651935270724</v>
+        <v>0.1079429789017231</v>
       </c>
       <c r="AG64" t="b">
         <v>0</v>
@@ -8169,7 +8169,7 @@
         <v>-0.0336521796372999</v>
       </c>
       <c r="AF65" t="n">
-        <v>0.5067175097180633</v>
+        <v>0.5061783731912427</v>
       </c>
       <c r="AG65" t="b">
         <v>0</v>
@@ -8290,7 +8290,7 @@
         <v>-0.0954147164859999</v>
       </c>
       <c r="AF66" t="n">
-        <v>0.8765247489113656</v>
+        <v>0.8765659525443154</v>
       </c>
       <c r="AG66" t="b">
         <v>0</v>
@@ -8407,7 +8407,7 @@
         <v>-0.0564342156425</v>
       </c>
       <c r="AF67" t="n">
-        <v>0.4285135595374503</v>
+        <v>0.4280075656543383</v>
       </c>
       <c r="AG67" t="b">
         <v>0</v>
@@ -8528,7 +8528,7 @@
         <v>-0.115636263893</v>
       </c>
       <c r="AF68" t="n">
-        <v>0.0449411757623897</v>
+        <v>0.044811732960064</v>
       </c>
       <c r="AG68" t="b">
         <v>1</v>
@@ -8645,7 +8645,7 @@
         <v>-0.08712639498874999</v>
       </c>
       <c r="AF69" t="n">
-        <v>0.9206771991228559</v>
+        <v>0.9208419478218036</v>
       </c>
       <c r="AG69" t="b">
         <v>0</v>
@@ -8762,7 +8762,7 @@
         <v>-0.0340363046559999</v>
       </c>
       <c r="AF70" t="n">
-        <v>0.8093837764468539</v>
+        <v>0.8093307762351802</v>
       </c>
       <c r="AG70" t="b">
         <v>0</v>
@@ -8883,7 +8883,7 @@
         <v>-0.0311651282504999</v>
       </c>
       <c r="AF71" t="n">
-        <v>0.7312175116270664</v>
+        <v>0.7310452233076115</v>
       </c>
       <c r="AG71" t="b">
         <v>0</v>
@@ -9004,7 +9004,7 @@
         <v>-0.2003053143665</v>
       </c>
       <c r="AF72" t="n">
-        <v>0.1270973663551465</v>
+        <v>0.1267216314648649</v>
       </c>
       <c r="AG72" t="b">
         <v>0</v>
@@ -9125,7 +9125,7 @@
         <v>-0.1127117610025</v>
       </c>
       <c r="AF73" t="n">
-        <v>0.2672931533651203</v>
+        <v>0.2667095721374268</v>
       </c>
       <c r="AG73" t="b">
         <v>0</v>
@@ -9363,7 +9363,7 @@
         <v>-0.0250535125772849</v>
       </c>
       <c r="AF75" t="n">
-        <v>0.2488610196540167</v>
+        <v>0.2483092879482216</v>
       </c>
       <c r="AG75" t="b">
         <v>0</v>
@@ -9480,7 +9480,7 @@
         <v>-0.1290431923988112</v>
       </c>
       <c r="AF76" t="n">
-        <v>0.0139595536418847</v>
+        <v>0.0139101376020666</v>
       </c>
       <c r="AG76" t="b">
         <v>1</v>
@@ -9708,7 +9708,7 @@
         <v>-0.5739256359145</v>
       </c>
       <c r="AF78" t="n">
-        <v>4.880381313946173e-06</v>
+        <v>4.890472085950937e-06</v>
       </c>
       <c r="AG78" t="b">
         <v>1</v>
@@ -10057,7 +10057,7 @@
         <v>-0.1269716404524999</v>
       </c>
       <c r="AF81" t="n">
-        <v>0.0581305131456747</v>
+        <v>0.0579577871028306</v>
       </c>
       <c r="AG81" t="b">
         <v>0</v>
@@ -10293,7 +10293,7 @@
         <v>-0.131450956184</v>
       </c>
       <c r="AF83" t="n">
-        <v>0.2605525109645124</v>
+        <v>0.2600134893204817</v>
       </c>
       <c r="AG83" t="b">
         <v>0</v>
@@ -10414,7 +10414,7 @@
         <v>-0.1610288049535</v>
       </c>
       <c r="AF84" t="n">
-        <v>0.0116686999347966</v>
+        <v>0.0116259240022972</v>
       </c>
       <c r="AG84" t="b">
         <v>1</v>
@@ -10531,7 +10531,7 @@
         <v>-0.19374070244</v>
       </c>
       <c r="AF85" t="n">
-        <v>0.0419983086835975</v>
+        <v>0.0418683758787672</v>
       </c>
       <c r="AG85" t="b">
         <v>1</v>
@@ -10773,7 +10773,7 @@
         <v>-0.09759208049199999</v>
       </c>
       <c r="AF87" t="n">
-        <v>0.2590426996636222</v>
+        <v>0.2585059524084093</v>
       </c>
       <c r="AG87" t="b">
         <v>0</v>
@@ -11005,7 +11005,7 @@
         <v>-0.2617517219281</v>
       </c>
       <c r="AF89" t="n">
-        <v>0.000457973393415</v>
+        <v>0.0004583075025169</v>
       </c>
       <c r="AG89" t="b">
         <v>1</v>
@@ -11122,7 +11122,7 @@
         <v>-0.287709354222</v>
       </c>
       <c r="AF90" t="n">
-        <v>2.07912848719522e-06</v>
+        <v>2.072136501979133e-06</v>
       </c>
       <c r="AG90" t="b">
         <v>1</v>
@@ -11239,7 +11239,7 @@
         <v>0.0226837776155</v>
       </c>
       <c r="AF91" t="n">
-        <v>0.8521893311806578</v>
+        <v>0.8522521068986072</v>
       </c>
       <c r="AG91" t="b">
         <v>0</v>
@@ -11360,7 +11360,7 @@
         <v>-0.140219236027</v>
       </c>
       <c r="AF92" t="n">
-        <v>0.0021314325680103</v>
+        <v>0.0021259628450126</v>
       </c>
       <c r="AG92" t="b">
         <v>1</v>
@@ -11481,7 +11481,7 @@
         <v>-0.071262988571</v>
       </c>
       <c r="AF93" t="n">
-        <v>0.2687944170079644</v>
+        <v>0.2681896655320817</v>
       </c>
       <c r="AG93" t="b">
         <v>0</v>
@@ -11717,7 +11717,7 @@
         <v>-0.190430881344</v>
       </c>
       <c r="AF95" t="n">
-        <v>0.0057281527614398</v>
+        <v>0.0057096564213125</v>
       </c>
       <c r="AG95" t="b">
         <v>1</v>

</xml_diff>

<commit_message>
RNAi mapping and lineage counts written out; tables: robustness tiers, RNAi 'supported'
Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/figures/supporting_information/S2_Table.xlsx
+++ b/figures/supporting_information/S2_Table.xlsx
@@ -536,7 +536,7 @@
       </c>
       <c r="V1" s="1" t="inlineStr">
         <is>
-          <t>Confidence tier</t>
+          <t>Robustness tier</t>
         </is>
       </c>
       <c r="W1" s="1" t="inlineStr">
@@ -591,7 +591,7 @@
       </c>
       <c r="AG1" s="1" t="inlineStr">
         <is>
-          <t>RNAi: confirmed (q &lt; 0.05, negative selectivity)</t>
+          <t>RNAi: supported (q &lt; 0.05, negative selectivity)</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
S2 Table: column marking pairs whose lineage signal is largely explained by genotype or TP53 status
Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/figures/supporting_information/S2_Table.xlsx
+++ b/figures/supporting_information/S2_Table.xlsx
@@ -425,7 +425,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:AG95"/>
+  <dimension ref="A1:AH95"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -594,6 +594,11 @@
           <t>RNAi: supported (q &lt; 0.05, negative selectivity)</t>
         </is>
       </c>
+      <c r="AH1" s="1" t="inlineStr">
+        <is>
+          <t>Possible genotype explanation of the lineage signal</t>
+        </is>
+      </c>
     </row>
     <row r="2">
       <c r="A2" t="inlineStr">
@@ -715,6 +720,11 @@
       <c r="AG2" t="b">
         <v>1</v>
       </c>
+      <c r="AH2" t="inlineStr">
+        <is>
+          <t>KRAS hotspot mutation (lineage coefficient reduced to 28% after adjustment for genotype)</t>
+        </is>
+      </c>
     </row>
     <row r="3">
       <c r="A3" t="inlineStr">
@@ -836,6 +846,7 @@
       <c r="AG3" t="b">
         <v>1</v>
       </c>
+      <c r="AH3" t="inlineStr"/>
     </row>
     <row r="4">
       <c r="A4" t="inlineStr">
@@ -957,6 +968,7 @@
       <c r="AG4" t="b">
         <v>1</v>
       </c>
+      <c r="AH4" t="inlineStr"/>
     </row>
     <row r="5">
       <c r="A5" t="inlineStr">
@@ -1078,6 +1090,7 @@
       <c r="AG5" t="b">
         <v>1</v>
       </c>
+      <c r="AH5" t="inlineStr"/>
     </row>
     <row r="6">
       <c r="A6" t="inlineStr">
@@ -1193,6 +1206,11 @@
           <t>not testable</t>
         </is>
       </c>
+      <c r="AH6" t="inlineStr">
+        <is>
+          <t>TP53 status (selectivity -0.36 among lines without a detected TP53 variant)</t>
+        </is>
+      </c>
     </row>
     <row r="7">
       <c r="A7" t="inlineStr">
@@ -1314,6 +1332,11 @@
       <c r="AG7" t="b">
         <v>1</v>
       </c>
+      <c r="AH7" t="inlineStr">
+        <is>
+          <t>APC truncating or CTNNB1 hotspot mutation (lineage coefficient reduced to 50% after adjustment for genotype)</t>
+        </is>
+      </c>
     </row>
     <row r="8">
       <c r="A8" t="inlineStr">
@@ -1435,6 +1458,7 @@
       <c r="AG8" t="b">
         <v>0</v>
       </c>
+      <c r="AH8" t="inlineStr"/>
     </row>
     <row r="9">
       <c r="A9" t="inlineStr">
@@ -1552,6 +1576,7 @@
       <c r="AG9" t="b">
         <v>1</v>
       </c>
+      <c r="AH9" t="inlineStr"/>
     </row>
     <row r="10">
       <c r="A10" t="inlineStr">
@@ -1669,6 +1694,7 @@
       <c r="AG10" t="b">
         <v>1</v>
       </c>
+      <c r="AH10" t="inlineStr"/>
     </row>
     <row r="11">
       <c r="A11" t="inlineStr">
@@ -1784,6 +1810,7 @@
           <t>not testable</t>
         </is>
       </c>
+      <c r="AH11" t="inlineStr"/>
     </row>
     <row r="12">
       <c r="A12" t="inlineStr">
@@ -1905,6 +1932,7 @@
       <c r="AG12" t="b">
         <v>1</v>
       </c>
+      <c r="AH12" t="inlineStr"/>
     </row>
     <row r="13">
       <c r="A13" t="inlineStr">
@@ -2025,6 +2053,11 @@
       </c>
       <c r="AG13" t="b">
         <v>1</v>
+      </c>
+      <c r="AH13" t="inlineStr">
+        <is>
+          <t>BRAF V600 mutation (lineage coefficient reduced to 22% after adjustment for genotype)</t>
+        </is>
       </c>
     </row>
     <row r="14">
@@ -2141,6 +2174,7 @@
           <t>not testable</t>
         </is>
       </c>
+      <c r="AH14" t="inlineStr"/>
     </row>
     <row r="15">
       <c r="A15" t="inlineStr">
@@ -2258,6 +2292,7 @@
       <c r="AG15" t="b">
         <v>0</v>
       </c>
+      <c r="AH15" t="inlineStr"/>
     </row>
     <row r="16">
       <c r="A16" t="inlineStr">
@@ -2375,6 +2410,7 @@
       <c r="AG16" t="b">
         <v>1</v>
       </c>
+      <c r="AH16" t="inlineStr"/>
     </row>
     <row r="17">
       <c r="A17" t="inlineStr">
@@ -2496,6 +2532,7 @@
       <c r="AG17" t="b">
         <v>1</v>
       </c>
+      <c r="AH17" t="inlineStr"/>
     </row>
     <row r="18">
       <c r="A18" t="inlineStr">
@@ -2617,6 +2654,7 @@
       <c r="AG18" t="b">
         <v>1</v>
       </c>
+      <c r="AH18" t="inlineStr"/>
     </row>
     <row r="19">
       <c r="A19" t="inlineStr">
@@ -2732,6 +2770,7 @@
           <t>not testable</t>
         </is>
       </c>
+      <c r="AH19" t="inlineStr"/>
     </row>
     <row r="20">
       <c r="A20" t="inlineStr">
@@ -2853,6 +2892,11 @@
       <c r="AG20" t="b">
         <v>1</v>
       </c>
+      <c r="AH20" t="inlineStr">
+        <is>
+          <t>TP53 status (selectivity -0.24 among lines without a detected TP53 variant)</t>
+        </is>
+      </c>
     </row>
     <row r="21">
       <c r="A21" t="inlineStr">
@@ -2973,6 +3017,11 @@
       </c>
       <c r="AG21" t="b">
         <v>0</v>
+      </c>
+      <c r="AH21" t="inlineStr">
+        <is>
+          <t>TP53 status (selectivity -0.14 among lines without a detected TP53 variant)</t>
+        </is>
       </c>
     </row>
     <row r="22">
@@ -3089,6 +3138,7 @@
           <t>not testable</t>
         </is>
       </c>
+      <c r="AH22" t="inlineStr"/>
     </row>
     <row r="23">
       <c r="A23" t="inlineStr">
@@ -3210,6 +3260,11 @@
       <c r="AG23" t="b">
         <v>1</v>
       </c>
+      <c r="AH23" t="inlineStr">
+        <is>
+          <t>TP53 status, partly (selectivity -0.55 among lines without a detected TP53 variant)</t>
+        </is>
+      </c>
     </row>
     <row r="24">
       <c r="A24" t="inlineStr">
@@ -3327,6 +3382,7 @@
       <c r="AG24" t="b">
         <v>0</v>
       </c>
+      <c r="AH24" t="inlineStr"/>
     </row>
     <row r="25">
       <c r="A25" t="inlineStr">
@@ -3444,6 +3500,7 @@
       <c r="AG25" t="b">
         <v>1</v>
       </c>
+      <c r="AH25" t="inlineStr"/>
     </row>
     <row r="26">
       <c r="A26" t="inlineStr">
@@ -3561,6 +3618,7 @@
       <c r="AG26" t="b">
         <v>0</v>
       </c>
+      <c r="AH26" t="inlineStr"/>
     </row>
     <row r="27">
       <c r="A27" t="inlineStr">
@@ -3678,6 +3736,7 @@
       <c r="AG27" t="b">
         <v>0</v>
       </c>
+      <c r="AH27" t="inlineStr"/>
     </row>
     <row r="28">
       <c r="A28" t="inlineStr">
@@ -3799,6 +3858,7 @@
       <c r="AG28" t="b">
         <v>0</v>
       </c>
+      <c r="AH28" t="inlineStr"/>
     </row>
     <row r="29">
       <c r="A29" t="inlineStr">
@@ -3916,6 +3976,7 @@
       <c r="AG29" t="b">
         <v>0</v>
       </c>
+      <c r="AH29" t="inlineStr"/>
     </row>
     <row r="30">
       <c r="A30" t="inlineStr">
@@ -4037,6 +4098,7 @@
       <c r="AG30" t="b">
         <v>0</v>
       </c>
+      <c r="AH30" t="inlineStr"/>
     </row>
     <row r="31">
       <c r="A31" t="inlineStr">
@@ -4154,6 +4216,7 @@
       <c r="AG31" t="b">
         <v>1</v>
       </c>
+      <c r="AH31" t="inlineStr"/>
     </row>
     <row r="32">
       <c r="A32" t="inlineStr">
@@ -4275,6 +4338,7 @@
       <c r="AG32" t="b">
         <v>1</v>
       </c>
+      <c r="AH32" t="inlineStr"/>
     </row>
     <row r="33">
       <c r="A33" t="inlineStr">
@@ -4392,6 +4456,7 @@
       <c r="AG33" t="b">
         <v>0</v>
       </c>
+      <c r="AH33" t="inlineStr"/>
     </row>
     <row r="34">
       <c r="A34" t="inlineStr">
@@ -4509,6 +4574,7 @@
       <c r="AG34" t="b">
         <v>0</v>
       </c>
+      <c r="AH34" t="inlineStr"/>
     </row>
     <row r="35">
       <c r="A35" t="inlineStr">
@@ -4626,6 +4692,7 @@
       <c r="AG35" t="b">
         <v>1</v>
       </c>
+      <c r="AH35" t="inlineStr"/>
     </row>
     <row r="36">
       <c r="A36" t="inlineStr">
@@ -4743,6 +4810,7 @@
       <c r="AG36" t="b">
         <v>0</v>
       </c>
+      <c r="AH36" t="inlineStr"/>
     </row>
     <row r="37">
       <c r="A37" t="inlineStr">
@@ -4864,6 +4932,7 @@
       <c r="AG37" t="b">
         <v>1</v>
       </c>
+      <c r="AH37" t="inlineStr"/>
     </row>
     <row r="38">
       <c r="A38" t="inlineStr">
@@ -4981,6 +5050,7 @@
       <c r="AG38" t="b">
         <v>0</v>
       </c>
+      <c r="AH38" t="inlineStr"/>
     </row>
     <row r="39">
       <c r="A39" t="inlineStr">
@@ -5098,6 +5168,7 @@
       <c r="AG39" t="b">
         <v>0</v>
       </c>
+      <c r="AH39" t="inlineStr"/>
     </row>
     <row r="40">
       <c r="A40" t="inlineStr">
@@ -5215,6 +5286,7 @@
       <c r="AG40" t="b">
         <v>1</v>
       </c>
+      <c r="AH40" t="inlineStr"/>
     </row>
     <row r="41">
       <c r="A41" t="inlineStr">
@@ -5336,6 +5408,7 @@
       <c r="AG41" t="b">
         <v>0</v>
       </c>
+      <c r="AH41" t="inlineStr"/>
     </row>
     <row r="42">
       <c r="A42" t="inlineStr">
@@ -5456,6 +5529,11 @@
       </c>
       <c r="AG42" t="b">
         <v>0</v>
+      </c>
+      <c r="AH42" t="inlineStr">
+        <is>
+          <t>KRAS hotspot mutation (frequent in this lineage; see Genotype-associated dependencies)</t>
+        </is>
       </c>
     </row>
     <row r="43">
@@ -5572,6 +5650,7 @@
           <t>not testable</t>
         </is>
       </c>
+      <c r="AH43" t="inlineStr"/>
     </row>
     <row r="44">
       <c r="A44" t="inlineStr">
@@ -5689,6 +5768,7 @@
       <c r="AG44" t="b">
         <v>0</v>
       </c>
+      <c r="AH44" t="inlineStr"/>
     </row>
     <row r="45">
       <c r="A45" t="inlineStr">
@@ -5810,6 +5890,7 @@
       <c r="AG45" t="b">
         <v>0</v>
       </c>
+      <c r="AH45" t="inlineStr"/>
     </row>
     <row r="46">
       <c r="A46" t="inlineStr">
@@ -5931,6 +6012,7 @@
       <c r="AG46" t="b">
         <v>1</v>
       </c>
+      <c r="AH46" t="inlineStr"/>
     </row>
     <row r="47">
       <c r="A47" t="inlineStr">
@@ -6048,6 +6130,7 @@
       <c r="AG47" t="b">
         <v>0</v>
       </c>
+      <c r="AH47" t="inlineStr"/>
     </row>
     <row r="48">
       <c r="A48" t="inlineStr">
@@ -6169,6 +6252,7 @@
       <c r="AG48" t="b">
         <v>0</v>
       </c>
+      <c r="AH48" t="inlineStr"/>
     </row>
     <row r="49">
       <c r="A49" t="inlineStr">
@@ -6286,6 +6370,7 @@
       <c r="AG49" t="b">
         <v>0</v>
       </c>
+      <c r="AH49" t="inlineStr"/>
     </row>
     <row r="50">
       <c r="A50" t="inlineStr">
@@ -6403,6 +6488,7 @@
       <c r="AG50" t="b">
         <v>1</v>
       </c>
+      <c r="AH50" t="inlineStr"/>
     </row>
     <row r="51">
       <c r="A51" t="inlineStr">
@@ -6520,6 +6606,7 @@
       <c r="AG51" t="b">
         <v>0</v>
       </c>
+      <c r="AH51" t="inlineStr"/>
     </row>
     <row r="52">
       <c r="A52" t="inlineStr">
@@ -6641,6 +6728,7 @@
       <c r="AG52" t="b">
         <v>0</v>
       </c>
+      <c r="AH52" t="inlineStr"/>
     </row>
     <row r="53">
       <c r="A53" t="inlineStr">
@@ -6758,6 +6846,7 @@
       <c r="AG53" t="b">
         <v>0</v>
       </c>
+      <c r="AH53" t="inlineStr"/>
     </row>
     <row r="54">
       <c r="A54" t="inlineStr">
@@ -6879,6 +6968,7 @@
       <c r="AG54" t="b">
         <v>0</v>
       </c>
+      <c r="AH54" t="inlineStr"/>
     </row>
     <row r="55">
       <c r="A55" t="inlineStr">
@@ -6996,6 +7086,7 @@
       <c r="AG55" t="b">
         <v>0</v>
       </c>
+      <c r="AH55" t="inlineStr"/>
     </row>
     <row r="56">
       <c r="A56" t="inlineStr">
@@ -7113,6 +7204,7 @@
       <c r="AG56" t="b">
         <v>0</v>
       </c>
+      <c r="AH56" t="inlineStr"/>
     </row>
     <row r="57">
       <c r="A57" t="inlineStr">
@@ -7228,6 +7320,7 @@
           <t>not testable</t>
         </is>
       </c>
+      <c r="AH57" t="inlineStr"/>
     </row>
     <row r="58">
       <c r="A58" t="inlineStr">
@@ -7345,6 +7438,7 @@
       <c r="AG58" t="b">
         <v>0</v>
       </c>
+      <c r="AH58" t="inlineStr"/>
     </row>
     <row r="59">
       <c r="A59" t="inlineStr">
@@ -7462,6 +7556,7 @@
       <c r="AG59" t="b">
         <v>1</v>
       </c>
+      <c r="AH59" t="inlineStr"/>
     </row>
     <row r="60">
       <c r="A60" t="inlineStr">
@@ -7583,6 +7678,7 @@
       <c r="AG60" t="b">
         <v>0</v>
       </c>
+      <c r="AH60" t="inlineStr"/>
     </row>
     <row r="61">
       <c r="A61" t="inlineStr">
@@ -7700,6 +7796,7 @@
       <c r="AG61" t="b">
         <v>0</v>
       </c>
+      <c r="AH61" t="inlineStr"/>
     </row>
     <row r="62">
       <c r="A62" t="inlineStr">
@@ -7815,6 +7912,7 @@
           <t>not testable</t>
         </is>
       </c>
+      <c r="AH62" t="inlineStr"/>
     </row>
     <row r="63">
       <c r="A63" t="inlineStr">
@@ -7932,6 +8030,7 @@
       <c r="AG63" t="b">
         <v>0</v>
       </c>
+      <c r="AH63" t="inlineStr"/>
     </row>
     <row r="64">
       <c r="A64" t="inlineStr">
@@ -8053,6 +8152,7 @@
       <c r="AG64" t="b">
         <v>0</v>
       </c>
+      <c r="AH64" t="inlineStr"/>
     </row>
     <row r="65">
       <c r="A65" t="inlineStr">
@@ -8174,6 +8274,7 @@
       <c r="AG65" t="b">
         <v>0</v>
       </c>
+      <c r="AH65" t="inlineStr"/>
     </row>
     <row r="66">
       <c r="A66" t="inlineStr">
@@ -8295,6 +8396,7 @@
       <c r="AG66" t="b">
         <v>0</v>
       </c>
+      <c r="AH66" t="inlineStr"/>
     </row>
     <row r="67">
       <c r="A67" t="inlineStr">
@@ -8412,6 +8514,7 @@
       <c r="AG67" t="b">
         <v>0</v>
       </c>
+      <c r="AH67" t="inlineStr"/>
     </row>
     <row r="68">
       <c r="A68" t="inlineStr">
@@ -8533,6 +8636,7 @@
       <c r="AG68" t="b">
         <v>1</v>
       </c>
+      <c r="AH68" t="inlineStr"/>
     </row>
     <row r="69">
       <c r="A69" t="inlineStr">
@@ -8650,6 +8754,7 @@
       <c r="AG69" t="b">
         <v>0</v>
       </c>
+      <c r="AH69" t="inlineStr"/>
     </row>
     <row r="70">
       <c r="A70" t="inlineStr">
@@ -8767,6 +8872,7 @@
       <c r="AG70" t="b">
         <v>0</v>
       </c>
+      <c r="AH70" t="inlineStr"/>
     </row>
     <row r="71">
       <c r="A71" t="inlineStr">
@@ -8888,6 +8994,7 @@
       <c r="AG71" t="b">
         <v>0</v>
       </c>
+      <c r="AH71" t="inlineStr"/>
     </row>
     <row r="72">
       <c r="A72" t="inlineStr">
@@ -9009,6 +9116,7 @@
       <c r="AG72" t="b">
         <v>0</v>
       </c>
+      <c r="AH72" t="inlineStr"/>
     </row>
     <row r="73">
       <c r="A73" t="inlineStr">
@@ -9130,6 +9238,7 @@
       <c r="AG73" t="b">
         <v>0</v>
       </c>
+      <c r="AH73" t="inlineStr"/>
     </row>
     <row r="74">
       <c r="A74" t="inlineStr">
@@ -9247,6 +9356,7 @@
       <c r="AG74" t="b">
         <v>0</v>
       </c>
+      <c r="AH74" t="inlineStr"/>
     </row>
     <row r="75">
       <c r="A75" t="inlineStr">
@@ -9368,6 +9478,7 @@
       <c r="AG75" t="b">
         <v>0</v>
       </c>
+      <c r="AH75" t="inlineStr"/>
     </row>
     <row r="76">
       <c r="A76" t="inlineStr">
@@ -9485,6 +9596,7 @@
       <c r="AG76" t="b">
         <v>1</v>
       </c>
+      <c r="AH76" t="inlineStr"/>
     </row>
     <row r="77">
       <c r="A77" t="inlineStr">
@@ -9596,6 +9708,7 @@
           <t>not testable</t>
         </is>
       </c>
+      <c r="AH77" t="inlineStr"/>
     </row>
     <row r="78">
       <c r="A78" t="inlineStr">
@@ -9713,6 +9826,7 @@
       <c r="AG78" t="b">
         <v>1</v>
       </c>
+      <c r="AH78" t="inlineStr"/>
     </row>
     <row r="79">
       <c r="A79" t="inlineStr">
@@ -9830,6 +9944,7 @@
       <c r="AG79" t="b">
         <v>0</v>
       </c>
+      <c r="AH79" t="inlineStr"/>
     </row>
     <row r="80">
       <c r="A80" t="inlineStr">
@@ -9945,6 +10060,7 @@
           <t>not testable</t>
         </is>
       </c>
+      <c r="AH80" t="inlineStr"/>
     </row>
     <row r="81">
       <c r="A81" t="inlineStr">
@@ -10062,6 +10178,7 @@
       <c r="AG81" t="b">
         <v>0</v>
       </c>
+      <c r="AH81" t="inlineStr"/>
     </row>
     <row r="82">
       <c r="A82" t="inlineStr">
@@ -10177,6 +10294,7 @@
           <t>not testable</t>
         </is>
       </c>
+      <c r="AH82" t="inlineStr"/>
     </row>
     <row r="83">
       <c r="A83" t="inlineStr">
@@ -10298,6 +10416,7 @@
       <c r="AG83" t="b">
         <v>0</v>
       </c>
+      <c r="AH83" t="inlineStr"/>
     </row>
     <row r="84">
       <c r="A84" t="inlineStr">
@@ -10419,6 +10538,7 @@
       <c r="AG84" t="b">
         <v>1</v>
       </c>
+      <c r="AH84" t="inlineStr"/>
     </row>
     <row r="85">
       <c r="A85" t="inlineStr">
@@ -10536,6 +10656,7 @@
       <c r="AG85" t="b">
         <v>1</v>
       </c>
+      <c r="AH85" t="inlineStr"/>
     </row>
     <row r="86">
       <c r="A86" t="inlineStr">
@@ -10657,6 +10778,7 @@
       <c r="AG86" t="b">
         <v>0</v>
       </c>
+      <c r="AH86" t="inlineStr"/>
     </row>
     <row r="87">
       <c r="A87" t="inlineStr">
@@ -10778,6 +10900,7 @@
       <c r="AG87" t="b">
         <v>0</v>
       </c>
+      <c r="AH87" t="inlineStr"/>
     </row>
     <row r="88">
       <c r="A88" t="inlineStr">
@@ -10893,6 +11016,7 @@
           <t>not testable</t>
         </is>
       </c>
+      <c r="AH88" t="inlineStr"/>
     </row>
     <row r="89">
       <c r="A89" t="inlineStr">
@@ -11010,6 +11134,7 @@
       <c r="AG89" t="b">
         <v>1</v>
       </c>
+      <c r="AH89" t="inlineStr"/>
     </row>
     <row r="90">
       <c r="A90" t="inlineStr">
@@ -11127,6 +11252,7 @@
       <c r="AG90" t="b">
         <v>1</v>
       </c>
+      <c r="AH90" t="inlineStr"/>
     </row>
     <row r="91">
       <c r="A91" t="inlineStr">
@@ -11244,6 +11370,7 @@
       <c r="AG91" t="b">
         <v>0</v>
       </c>
+      <c r="AH91" t="inlineStr"/>
     </row>
     <row r="92">
       <c r="A92" t="inlineStr">
@@ -11365,6 +11492,7 @@
       <c r="AG92" t="b">
         <v>1</v>
       </c>
+      <c r="AH92" t="inlineStr"/>
     </row>
     <row r="93">
       <c r="A93" t="inlineStr">
@@ -11486,6 +11614,7 @@
       <c r="AG93" t="b">
         <v>0</v>
       </c>
+      <c r="AH93" t="inlineStr"/>
     </row>
     <row r="94">
       <c r="A94" t="inlineStr">
@@ -11601,6 +11730,7 @@
           <t>not testable</t>
         </is>
       </c>
+      <c r="AH94" t="inlineStr"/>
     </row>
     <row r="95">
       <c r="A95" t="inlineStr">
@@ -11722,6 +11852,7 @@
       <c r="AG95" t="b">
         <v>1</v>
       </c>
+      <c r="AH95" t="inlineStr"/>
     </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>

</xml_diff>